<commit_message>
Publica mapas XG-AE mapa_aderencia 2026-07-02 16:24:50
</commit_message>
<xml_diff>
--- a/mapas2/mapa_aderencia_xg_aderencia_eleitoral.xlsx
+++ b/mapas2/mapa_aderencia_xg_aderencia_eleitoral.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z9"/>
+  <dimension ref="A1:Z11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1002,7 +1002,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>salto</t>
+          <t>itu</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -1032,37 +1032,37 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Saúde - UBS, consultas, exames básicos, acesso SUS</t>
+          <t>Comportamento Político - Qualidade de gestão, eficiência, entrega de serviços</t>
         </is>
       </c>
       <c r="I6" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="J6" t="n">
-        <v>66.65348872129978</v>
+        <v>41.94822057230441</v>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Aderência positiva moderada</t>
+          <t>Relação inversa moderada</t>
         </is>
       </c>
       <c r="L6" t="n">
-        <v>0.4471947495393861</v>
+        <v>-0.1709908111569954</v>
       </c>
       <c r="M6" t="n">
-        <v>72.35973747696931</v>
+        <v>41.45045944215023</v>
       </c>
       <c r="N6" t="n">
-        <v>1.182833315726986</v>
+        <v>0.8206877726483239</v>
       </c>
       <c r="O6" t="n">
-        <v>56.05616960362779</v>
+        <v>42.8726340997336</v>
       </c>
       <c r="P6" t="n">
-        <v>14.48635634028892</v>
+        <v>171.0927612606071</v>
       </c>
       <c r="Q6" t="n">
-        <v>17.13494490278659</v>
+        <v>140.4137371552191</v>
       </c>
       <c r="R6" t="inlineStr">
         <is>
@@ -1070,10 +1070,10 @@
         </is>
       </c>
       <c r="S6" t="n">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="T6" t="n">
-        <v>1083</v>
+        <v>16493</v>
       </c>
       <c r="U6" t="n">
         <v>0</v>
@@ -1093,12 +1093,12 @@
       </c>
       <c r="Y6" t="inlineStr">
         <is>
-          <t>C:\Users\guilh\Trabalho\Relatórios Alisson\Documentos gerais\Git\2\dataquadri\mapas2\mapa_aderencia_rita_salto_sp_2022_saude_ubs_consultas_exames_basicos_acesso_sus_cidade_inteira.html</t>
+          <t>C:\Users\guilh\Trabalho\Relatórios Alisson\Documentos gerais\Git\2\dataquadri\mapas2\mapa_aderencia_rita_itu_sp_2022_comportamento_politico_qualidade_de_gestao_eficiencia_entrega_de_servicos_cidade_inteira.html</t>
         </is>
       </c>
       <c r="Z6" t="inlineStr">
         <is>
-          <t>https://quadrifygit.github.io/dataquadri/mapas2/mapa_aderencia_rita_salto_sp_2022_saude_ubs_consultas_exames_basicos_acesso_sus_cidade_inteira.html</t>
+          <t>https://quadrifygit.github.io/dataquadri/mapas2/mapa_aderencia_rita_itu_sp_2022_comportamento_politico_qualidade_de_gestao_eficiencia_entrega_de_servicos_cidade_inteira.html</t>
         </is>
       </c>
     </row>
@@ -1140,14 +1140,14 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Assistência Social - Proteção social, seguridade, assistência, rede pública</t>
+          <t>Saúde - UBS, consultas, exames básicos, acesso SUS</t>
         </is>
       </c>
       <c r="I7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J7" t="n">
-        <v>66.21252792890854</v>
+        <v>66.65348872129978</v>
       </c>
       <c r="K7" t="inlineStr">
         <is>
@@ -1155,10 +1155,10 @@
         </is>
       </c>
       <c r="L7" t="n">
-        <v>0.4336267251581173</v>
+        <v>0.4471947495393861</v>
       </c>
       <c r="M7" t="n">
-        <v>71.68133625790587</v>
+        <v>72.35973747696931</v>
       </c>
       <c r="N7" t="n">
         <v>1.182833315726986</v>
@@ -1201,12 +1201,12 @@
       </c>
       <c r="Y7" t="inlineStr">
         <is>
-          <t>C:\Users\guilh\Trabalho\Relatórios Alisson\Documentos gerais\Git\2\dataquadri\mapas2\mapa_aderencia_rita_salto_sp_2022_assistencia_social_protecao_social_seguridade_assistencia_rede_publica_cidade_inteira.html</t>
+          <t>C:\Users\guilh\Trabalho\Relatórios Alisson\Documentos gerais\Git\2\dataquadri\mapas2\mapa_aderencia_rita_salto_sp_2022_saude_ubs_consultas_exames_basicos_acesso_sus_cidade_inteira.html</t>
         </is>
       </c>
       <c r="Z7" t="inlineStr">
         <is>
-          <t>https://quadrifygit.github.io/dataquadri/mapas2/mapa_aderencia_rita_salto_sp_2022_assistencia_social_protecao_social_seguridade_assistencia_rede_publica_cidade_inteira.html</t>
+          <t>https://quadrifygit.github.io/dataquadri/mapas2/mapa_aderencia_rita_salto_sp_2022_saude_ubs_consultas_exames_basicos_acesso_sus_cidade_inteira.html</t>
         </is>
       </c>
     </row>
@@ -1248,37 +1248,37 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Saúde - Doenças crônicas, cuidado do idoso, acesso</t>
+          <t>Assistência Social - Proteção social, seguridade, assistência, rede pública</t>
         </is>
       </c>
       <c r="I8" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J8" t="n">
-        <v>54.93134641137685</v>
+        <v>66.21252792890854</v>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>Relação fraca ou neutra</t>
+          <t>Aderência positiva moderada</t>
         </is>
       </c>
       <c r="L8" t="n">
-        <v>0.1387972223867631</v>
+        <v>0.4336267251581173</v>
       </c>
       <c r="M8" t="n">
-        <v>56.93986111933815</v>
+        <v>71.68133625790587</v>
       </c>
       <c r="N8" t="n">
-        <v>1.033866499865964</v>
+        <v>1.182833315726986</v>
       </c>
       <c r="O8" t="n">
-        <v>51.20124766802015</v>
+        <v>56.05616960362779</v>
       </c>
       <c r="P8" t="n">
         <v>14.48635634028892</v>
       </c>
       <c r="Q8" t="n">
-        <v>14.97695852534562</v>
+        <v>17.13494490278659</v>
       </c>
       <c r="R8" t="inlineStr">
         <is>
@@ -1309,12 +1309,12 @@
       </c>
       <c r="Y8" t="inlineStr">
         <is>
-          <t>C:\Users\guilh\Trabalho\Relatórios Alisson\Documentos gerais\Git\2\dataquadri\mapas2\mapa_aderencia_rita_salto_sp_2022_saude_doencas_cronicas_cuidado_do_idoso_acesso_cidade_inteira.html</t>
+          <t>C:\Users\guilh\Trabalho\Relatórios Alisson\Documentos gerais\Git\2\dataquadri\mapas2\mapa_aderencia_rita_salto_sp_2022_assistencia_social_protecao_social_seguridade_assistencia_rede_publica_cidade_inteira.html</t>
         </is>
       </c>
       <c r="Z8" t="inlineStr">
         <is>
-          <t>https://quadrifygit.github.io/dataquadri/mapas2/mapa_aderencia_rita_salto_sp_2022_saude_doencas_cronicas_cuidado_do_idoso_acesso_cidade_inteira.html</t>
+          <t>https://quadrifygit.github.io/dataquadri/mapas2/mapa_aderencia_rita_salto_sp_2022_assistencia_social_protecao_social_seguridade_assistencia_rede_publica_cidade_inteira.html</t>
         </is>
       </c>
     </row>
@@ -1356,14 +1356,14 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Religião e Valores - Religiosidade, valores morais, costumes, família</t>
+          <t>Saúde - Doenças crônicas, cuidado do idoso, acesso</t>
         </is>
       </c>
       <c r="I9" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J9" t="n">
-        <v>53.79421781101134</v>
+        <v>54.93134641137685</v>
       </c>
       <c r="K9" t="inlineStr">
         <is>
@@ -1371,22 +1371,22 @@
         </is>
       </c>
       <c r="L9" t="n">
-        <v>0.09699303915798903</v>
+        <v>0.1387972223867631</v>
       </c>
       <c r="M9" t="n">
-        <v>54.84965195789945</v>
+        <v>56.93986111933815</v>
       </c>
       <c r="N9" t="n">
-        <v>1.052167966712642</v>
+        <v>1.033866499865964</v>
       </c>
       <c r="O9" t="n">
-        <v>51.83412582393341</v>
+        <v>51.20124766802015</v>
       </c>
       <c r="P9" t="n">
         <v>14.48635634028892</v>
       </c>
       <c r="Q9" t="n">
-        <v>15.24208009563658</v>
+        <v>14.97695852534562</v>
       </c>
       <c r="R9" t="inlineStr">
         <is>
@@ -1417,12 +1417,228 @@
       </c>
       <c r="Y9" t="inlineStr">
         <is>
+          <t>C:\Users\guilh\Trabalho\Relatórios Alisson\Documentos gerais\Git\2\dataquadri\mapas2\mapa_aderencia_rita_salto_sp_2022_saude_doencas_cronicas_cuidado_do_idoso_acesso_cidade_inteira.html</t>
+        </is>
+      </c>
+      <c r="Z9" t="inlineStr">
+        <is>
+          <t>https://quadrifygit.github.io/dataquadri/mapas2/mapa_aderencia_rita_salto_sp_2022_saude_doencas_cronicas_cuidado_do_idoso_acesso_cidade_inteira.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>salto</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>RITA DE CASSIA TRINCA PASSOS</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>DEPUTADO FEDERAL</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>cidade_inteira</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Religião e Valores - Religiosidade, valores morais, costumes, família</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
+        <v>4</v>
+      </c>
+      <c r="J10" t="n">
+        <v>53.79421781101134</v>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>Relação fraca ou neutra</t>
+        </is>
+      </c>
+      <c r="L10" t="n">
+        <v>0.09699303915798903</v>
+      </c>
+      <c r="M10" t="n">
+        <v>54.84965195789945</v>
+      </c>
+      <c r="N10" t="n">
+        <v>1.052167966712642</v>
+      </c>
+      <c r="O10" t="n">
+        <v>51.83412582393341</v>
+      </c>
+      <c r="P10" t="n">
+        <v>14.48635634028892</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>15.24208009563658</v>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>votos por mil</t>
+        </is>
+      </c>
+      <c r="S10" t="n">
+        <v>32</v>
+      </c>
+      <c r="T10" t="n">
+        <v>1083</v>
+      </c>
+      <c r="U10" t="n">
+        <v>0</v>
+      </c>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="W10" t="inlineStr">
+        <is>
+          <t>Total de votos do cargo/turno no local</t>
+        </is>
+      </c>
+      <c r="X10" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y10" t="inlineStr">
+        <is>
           <t>C:\Users\guilh\Trabalho\Relatórios Alisson\Documentos gerais\Git\2\dataquadri\mapas2\mapa_aderencia_rita_salto_sp_2022_religiao_e_valores_religiosidade_valores_morais_costumes_familia_cidade_inteira.html</t>
         </is>
       </c>
-      <c r="Z9" t="inlineStr">
+      <c r="Z10" t="inlineStr">
         <is>
           <t>https://quadrifygit.github.io/dataquadri/mapas2/mapa_aderencia_rita_salto_sp_2022_religiao_e_valores_religiosidade_valores_morais_costumes_familia_cidade_inteira.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>salto</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>RITA DE CASSIA TRINCA PASSOS</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>DEPUTADO FEDERAL</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>cidade_inteira</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Comportamento Político - Qualidade de gestão, eficiência, entrega de serviços</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
+        <v>5</v>
+      </c>
+      <c r="J11" t="n">
+        <v>53.27357156732022</v>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>Relação fraca ou neutra</t>
+        </is>
+      </c>
+      <c r="L11" t="n">
+        <v>0.1285295282603976</v>
+      </c>
+      <c r="M11" t="n">
+        <v>56.42647641301988</v>
+      </c>
+      <c r="N11" t="n">
+        <v>0.9309186940394231</v>
+      </c>
+      <c r="O11" t="n">
+        <v>47.41817685387798</v>
+      </c>
+      <c r="P11" t="n">
+        <v>14.48635634028892</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>13.48561992569148</v>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>votos por mil</t>
+        </is>
+      </c>
+      <c r="S11" t="n">
+        <v>32</v>
+      </c>
+      <c r="T11" t="n">
+        <v>1083</v>
+      </c>
+      <c r="U11" t="n">
+        <v>0</v>
+      </c>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="W11" t="inlineStr">
+        <is>
+          <t>Total de votos do cargo/turno no local</t>
+        </is>
+      </c>
+      <c r="X11" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y11" t="inlineStr">
+        <is>
+          <t>C:\Users\guilh\Trabalho\Relatórios Alisson\Documentos gerais\Git\2\dataquadri\mapas2\mapa_aderencia_rita_salto_sp_2022_comportamento_politico_qualidade_de_gestao_eficiencia_entrega_de_servicos_cidade_inteira.html</t>
+        </is>
+      </c>
+      <c r="Z11" t="inlineStr">
+        <is>
+          <t>https://quadrifygit.github.io/dataquadri/mapas2/mapa_aderencia_rita_salto_sp_2022_comportamento_politico_qualidade_de_gestao_eficiencia_entrega_de_servicos_cidade_inteira.html</t>
         </is>
       </c>
     </row>
@@ -1437,7 +1653,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M33"/>
+  <dimension ref="A1:M41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1755,26 +1971,26 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Religião e Valores - Religiosidade, valores morais, costumes, família</t>
+          <t>Comportamento Político - Qualidade de gestão, eficiência, entrega de serviços</t>
         </is>
       </c>
       <c r="G6" t="n">
         <v>1</v>
       </c>
       <c r="H6" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="I6" t="n">
-        <v>5282</v>
+        <v>411</v>
       </c>
       <c r="J6" t="n">
-        <v>37231</v>
+        <v>2386</v>
       </c>
       <c r="K6" t="n">
-        <v>141.8710214606108</v>
+        <v>172.254819782062</v>
       </c>
       <c r="L6" t="n">
-        <v>32.02570787606864</v>
+        <v>2.491966288728551</v>
       </c>
       <c r="M6" t="inlineStr">
         <is>
@@ -1810,26 +2026,26 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Religião e Valores - Religiosidade, valores morais, costumes, família</t>
+          <t>Comportamento Político - Qualidade de gestão, eficiência, entrega de serviços</t>
         </is>
       </c>
       <c r="G7" t="n">
         <v>2</v>
       </c>
       <c r="H7" t="n">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="I7" t="n">
-        <v>4714</v>
+        <v>8843</v>
       </c>
       <c r="J7" t="n">
-        <v>27516</v>
+        <v>47466</v>
       </c>
       <c r="K7" t="n">
-        <v>171.3185055967437</v>
+        <v>186.3017739013188</v>
       </c>
       <c r="L7" t="n">
-        <v>28.58182259140241</v>
+        <v>53.61668586673134</v>
       </c>
       <c r="M7" t="inlineStr">
         <is>
@@ -1865,26 +2081,26 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Religião e Valores - Religiosidade, valores morais, costumes, família</t>
+          <t>Comportamento Político - Qualidade de gestão, eficiência, entrega de serviços</t>
         </is>
       </c>
       <c r="G8" t="n">
         <v>3</v>
       </c>
       <c r="H8" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="I8" t="n">
-        <v>2574</v>
+        <v>5162</v>
       </c>
       <c r="J8" t="n">
-        <v>12802</v>
+        <v>31754</v>
       </c>
       <c r="K8" t="n">
-        <v>201.0623340103109</v>
+        <v>162.562196888581</v>
       </c>
       <c r="L8" t="n">
-        <v>15.60662099072334</v>
+        <v>31.29812647789971</v>
       </c>
       <c r="M8" t="inlineStr">
         <is>
@@ -1920,26 +2136,26 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Religião e Valores - Religiosidade, valores morais, costumes, família</t>
+          <t>Comportamento Político - Qualidade de gestão, eficiência, entrega de serviços</t>
         </is>
       </c>
       <c r="G9" t="n">
         <v>4</v>
       </c>
       <c r="H9" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="I9" t="n">
-        <v>3923</v>
+        <v>2077</v>
       </c>
       <c r="J9" t="n">
-        <v>18849</v>
+        <v>14792</v>
       </c>
       <c r="K9" t="n">
-        <v>208.1277521353918</v>
+        <v>140.4137371552191</v>
       </c>
       <c r="L9" t="n">
-        <v>23.78584854180562</v>
+        <v>12.59322136664039</v>
       </c>
       <c r="M9" t="inlineStr">
         <is>
@@ -1975,24 +2191,26 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Saúde - Doenças crônicas, cuidado do idoso, acesso</t>
+          <t>Religião e Valores - Religiosidade, valores morais, costumes, família</t>
         </is>
       </c>
       <c r="G10" t="n">
         <v>1</v>
       </c>
       <c r="H10" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="I10" t="n">
-        <v>0</v>
+        <v>5282</v>
       </c>
       <c r="J10" t="n">
-        <v>0</v>
-      </c>
-      <c r="K10" t="inlineStr"/>
+        <v>37231</v>
+      </c>
+      <c r="K10" t="n">
+        <v>141.8710214606108</v>
+      </c>
       <c r="L10" t="n">
-        <v>0</v>
+        <v>32.02570787606864</v>
       </c>
       <c r="M10" t="inlineStr">
         <is>
@@ -2028,26 +2246,26 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Saúde - Doenças crônicas, cuidado do idoso, acesso</t>
+          <t>Religião e Valores - Religiosidade, valores morais, costumes, família</t>
         </is>
       </c>
       <c r="G11" t="n">
         <v>2</v>
       </c>
       <c r="H11" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="I11" t="n">
-        <v>5633</v>
+        <v>4714</v>
       </c>
       <c r="J11" t="n">
-        <v>35281</v>
+        <v>27516</v>
       </c>
       <c r="K11" t="n">
-        <v>159.6610073410617</v>
+        <v>171.3185055967437</v>
       </c>
       <c r="L11" t="n">
-        <v>34.15388346571272</v>
+        <v>28.58182259140241</v>
       </c>
       <c r="M11" t="inlineStr">
         <is>
@@ -2083,26 +2301,26 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Saúde - Doenças crônicas, cuidado do idoso, acesso</t>
+          <t>Religião e Valores - Religiosidade, valores morais, costumes, família</t>
         </is>
       </c>
       <c r="G12" t="n">
         <v>3</v>
       </c>
       <c r="H12" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="I12" t="n">
-        <v>4046</v>
+        <v>2574</v>
       </c>
       <c r="J12" t="n">
-        <v>23400</v>
+        <v>12802</v>
       </c>
       <c r="K12" t="n">
-        <v>172.9059829059829</v>
+        <v>201.0623340103109</v>
       </c>
       <c r="L12" t="n">
-        <v>24.53161947492876</v>
+        <v>15.60662099072334</v>
       </c>
       <c r="M12" t="inlineStr">
         <is>
@@ -2138,26 +2356,26 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Saúde - Doenças crônicas, cuidado do idoso, acesso</t>
+          <t>Religião e Valores - Religiosidade, valores morais, costumes, família</t>
         </is>
       </c>
       <c r="G13" t="n">
         <v>4</v>
       </c>
       <c r="H13" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="I13" t="n">
-        <v>6814</v>
+        <v>3923</v>
       </c>
       <c r="J13" t="n">
-        <v>37717</v>
+        <v>18849</v>
       </c>
       <c r="K13" t="n">
-        <v>180.6612402895246</v>
+        <v>208.1277521353918</v>
       </c>
       <c r="L13" t="n">
-        <v>41.31449705935852</v>
+        <v>23.78584854180562</v>
       </c>
       <c r="M13" t="inlineStr">
         <is>
@@ -2193,26 +2411,24 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Saúde - UBS, consultas, exames básicos, acesso SUS</t>
+          <t>Saúde - Doenças crônicas, cuidado do idoso, acesso</t>
         </is>
       </c>
       <c r="G14" t="n">
         <v>1</v>
       </c>
       <c r="H14" t="n">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="I14" t="n">
-        <v>6374</v>
+        <v>0</v>
       </c>
       <c r="J14" t="n">
-        <v>44118</v>
-      </c>
-      <c r="K14" t="n">
-        <v>144.4761775239132</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="K14" t="inlineStr"/>
       <c r="L14" t="n">
-        <v>38.64669859940581</v>
+        <v>0</v>
       </c>
       <c r="M14" t="inlineStr">
         <is>
@@ -2248,26 +2464,26 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Saúde - UBS, consultas, exames básicos, acesso SUS</t>
+          <t>Saúde - Doenças crônicas, cuidado do idoso, acesso</t>
         </is>
       </c>
       <c r="G15" t="n">
         <v>2</v>
       </c>
       <c r="H15" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="I15" t="n">
-        <v>3266</v>
+        <v>5633</v>
       </c>
       <c r="J15" t="n">
-        <v>19250</v>
+        <v>35281</v>
       </c>
       <c r="K15" t="n">
-        <v>169.6623376623376</v>
+        <v>159.6610073410617</v>
       </c>
       <c r="L15" t="n">
-        <v>19.80234038683078</v>
+        <v>34.15388346571272</v>
       </c>
       <c r="M15" t="inlineStr">
         <is>
@@ -2303,26 +2519,26 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Saúde - UBS, consultas, exames básicos, acesso SUS</t>
+          <t>Saúde - Doenças crônicas, cuidado do idoso, acesso</t>
         </is>
       </c>
       <c r="G16" t="n">
         <v>3</v>
       </c>
       <c r="H16" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="I16" t="n">
-        <v>2308</v>
+        <v>4046</v>
       </c>
       <c r="J16" t="n">
-        <v>11017</v>
+        <v>23400</v>
       </c>
       <c r="K16" t="n">
-        <v>209.4944177180721</v>
+        <v>172.9059829059829</v>
       </c>
       <c r="L16" t="n">
-        <v>13.99381555811556</v>
+        <v>24.53161947492876</v>
       </c>
       <c r="M16" t="inlineStr">
         <is>
@@ -2358,26 +2574,26 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Saúde - UBS, consultas, exames básicos, acesso SUS</t>
+          <t>Saúde - Doenças crônicas, cuidado do idoso, acesso</t>
         </is>
       </c>
       <c r="G17" t="n">
         <v>4</v>
       </c>
       <c r="H17" t="n">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="I17" t="n">
-        <v>4545</v>
+        <v>6814</v>
       </c>
       <c r="J17" t="n">
-        <v>22013</v>
+        <v>37717</v>
       </c>
       <c r="K17" t="n">
-        <v>206.4689047381093</v>
+        <v>180.6612402895246</v>
       </c>
       <c r="L17" t="n">
-        <v>27.55714545564785</v>
+        <v>41.31449705935852</v>
       </c>
       <c r="M17" t="inlineStr">
         <is>
@@ -2393,7 +2609,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>salto</t>
+          <t>itu</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -2413,26 +2629,26 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Assistência Social - Proteção social, seguridade, assistência, rede pública</t>
+          <t>Saúde - UBS, consultas, exames básicos, acesso SUS</t>
         </is>
       </c>
       <c r="G18" t="n">
         <v>1</v>
       </c>
       <c r="H18" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="I18" t="n">
-        <v>314</v>
+        <v>6374</v>
       </c>
       <c r="J18" t="n">
-        <v>24918</v>
+        <v>44118</v>
       </c>
       <c r="K18" t="n">
-        <v>12.60133237017417</v>
+        <v>144.4761775239132</v>
       </c>
       <c r="L18" t="n">
-        <v>28.99353647276085</v>
+        <v>38.64669859940581</v>
       </c>
       <c r="M18" t="inlineStr">
         <is>
@@ -2448,7 +2664,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>salto</t>
+          <t>itu</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -2468,7 +2684,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Assistência Social - Proteção social, seguridade, assistência, rede pública</t>
+          <t>Saúde - UBS, consultas, exames básicos, acesso SUS</t>
         </is>
       </c>
       <c r="G19" t="n">
@@ -2478,16 +2694,16 @@
         <v>8</v>
       </c>
       <c r="I19" t="n">
-        <v>251</v>
+        <v>3266</v>
       </c>
       <c r="J19" t="n">
-        <v>18295</v>
+        <v>19250</v>
       </c>
       <c r="K19" t="n">
-        <v>13.71959551790107</v>
+        <v>169.6623376623376</v>
       </c>
       <c r="L19" t="n">
-        <v>23.17636195752539</v>
+        <v>19.80234038683078</v>
       </c>
       <c r="M19" t="inlineStr">
         <is>
@@ -2503,7 +2719,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>salto</t>
+          <t>itu</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -2523,26 +2739,26 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Assistência Social - Proteção social, seguridade, assistência, rede pública</t>
+          <t>Saúde - UBS, consultas, exames básicos, acesso SUS</t>
         </is>
       </c>
       <c r="G20" t="n">
         <v>3</v>
       </c>
       <c r="H20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I20" t="n">
-        <v>221</v>
+        <v>2308</v>
       </c>
       <c r="J20" t="n">
-        <v>14214</v>
+        <v>11017</v>
       </c>
       <c r="K20" t="n">
-        <v>15.54805121710989</v>
+        <v>209.4944177180721</v>
       </c>
       <c r="L20" t="n">
-        <v>20.40627885503232</v>
+        <v>13.99381555811556</v>
       </c>
       <c r="M20" t="inlineStr">
         <is>
@@ -2558,7 +2774,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>salto</t>
+          <t>itu</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -2578,26 +2794,26 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Assistência Social - Proteção social, seguridade, assistência, rede pública</t>
+          <t>Saúde - UBS, consultas, exames básicos, acesso SUS</t>
         </is>
       </c>
       <c r="G21" t="n">
         <v>4</v>
       </c>
       <c r="H21" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="I21" t="n">
-        <v>297</v>
+        <v>4545</v>
       </c>
       <c r="J21" t="n">
-        <v>17333</v>
+        <v>22013</v>
       </c>
       <c r="K21" t="n">
-        <v>17.13494490278659</v>
+        <v>206.4689047381093</v>
       </c>
       <c r="L21" t="n">
-        <v>27.42382271468144</v>
+        <v>27.55714545564785</v>
       </c>
       <c r="M21" t="inlineStr">
         <is>
@@ -2633,26 +2849,26 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Religião e Valores - Religiosidade, valores morais, costumes, família</t>
+          <t>Assistência Social - Proteção social, seguridade, assistência, rede pública</t>
         </is>
       </c>
       <c r="G22" t="n">
         <v>1</v>
       </c>
       <c r="H22" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="I22" t="n">
-        <v>301</v>
+        <v>314</v>
       </c>
       <c r="J22" t="n">
-        <v>20374</v>
+        <v>24918</v>
       </c>
       <c r="K22" t="n">
-        <v>14.77373122607245</v>
+        <v>12.60133237017417</v>
       </c>
       <c r="L22" t="n">
-        <v>27.79316712834719</v>
+        <v>28.99353647276085</v>
       </c>
       <c r="M22" t="inlineStr">
         <is>
@@ -2688,26 +2904,26 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Religião e Valores - Religiosidade, valores morais, costumes, família</t>
+          <t>Assistência Social - Proteção social, seguridade, assistência, rede pública</t>
         </is>
       </c>
       <c r="G23" t="n">
         <v>2</v>
       </c>
       <c r="H23" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="I23" t="n">
-        <v>210</v>
+        <v>251</v>
       </c>
       <c r="J23" t="n">
-        <v>16286</v>
+        <v>18295</v>
       </c>
       <c r="K23" t="n">
-        <v>12.89451062262066</v>
+        <v>13.71959551790107</v>
       </c>
       <c r="L23" t="n">
-        <v>19.39058171745152</v>
+        <v>23.17636195752539</v>
       </c>
       <c r="M23" t="inlineStr">
         <is>
@@ -2743,26 +2959,26 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Religião e Valores - Religiosidade, valores morais, costumes, família</t>
+          <t>Assistência Social - Proteção social, seguridade, assistência, rede pública</t>
         </is>
       </c>
       <c r="G24" t="n">
         <v>3</v>
       </c>
       <c r="H24" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="I24" t="n">
-        <v>317</v>
+        <v>221</v>
       </c>
       <c r="J24" t="n">
-        <v>21370</v>
+        <v>14214</v>
       </c>
       <c r="K24" t="n">
-        <v>14.83387927000468</v>
+        <v>15.54805121710989</v>
       </c>
       <c r="L24" t="n">
-        <v>29.27054478301016</v>
+        <v>20.40627885503232</v>
       </c>
       <c r="M24" t="inlineStr">
         <is>
@@ -2798,7 +3014,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Religião e Valores - Religiosidade, valores morais, costumes, família</t>
+          <t>Assistência Social - Proteção social, seguridade, assistência, rede pública</t>
         </is>
       </c>
       <c r="G25" t="n">
@@ -2808,16 +3024,16 @@
         <v>9</v>
       </c>
       <c r="I25" t="n">
-        <v>255</v>
+        <v>297</v>
       </c>
       <c r="J25" t="n">
-        <v>16730</v>
+        <v>17333</v>
       </c>
       <c r="K25" t="n">
-        <v>15.24208009563658</v>
+        <v>17.13494490278659</v>
       </c>
       <c r="L25" t="n">
-        <v>23.54570637119114</v>
+        <v>27.42382271468144</v>
       </c>
       <c r="M25" t="inlineStr">
         <is>
@@ -2853,26 +3069,26 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Saúde - Doenças crônicas, cuidado do idoso, acesso</t>
+          <t>Comportamento Político - Qualidade de gestão, eficiência, entrega de serviços</t>
         </is>
       </c>
       <c r="G26" t="n">
         <v>1</v>
       </c>
       <c r="H26" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="I26" t="n">
-        <v>127</v>
+        <v>202</v>
       </c>
       <c r="J26" t="n">
-        <v>7202</v>
+        <v>14966</v>
       </c>
       <c r="K26" t="n">
-        <v>17.63399055817828</v>
+        <v>13.49726045703595</v>
       </c>
       <c r="L26" t="n">
-        <v>11.72668513388735</v>
+        <v>18.65189289012004</v>
       </c>
       <c r="M26" t="inlineStr">
         <is>
@@ -2908,26 +3124,26 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Saúde - Doenças crônicas, cuidado do idoso, acesso</t>
+          <t>Comportamento Político - Qualidade de gestão, eficiência, entrega de serviços</t>
         </is>
       </c>
       <c r="G27" t="n">
         <v>2</v>
       </c>
       <c r="H27" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="I27" t="n">
-        <v>243</v>
+        <v>447</v>
       </c>
       <c r="J27" t="n">
-        <v>20059</v>
+        <v>30113</v>
       </c>
       <c r="K27" t="n">
-        <v>12.1142629243731</v>
+        <v>14.84408727127819</v>
       </c>
       <c r="L27" t="n">
-        <v>22.4376731301939</v>
+        <v>41.27423822714682</v>
       </c>
       <c r="M27" t="inlineStr">
         <is>
@@ -2963,26 +3179,26 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Saúde - Doenças crônicas, cuidado do idoso, acesso</t>
+          <t>Comportamento Político - Qualidade de gestão, eficiência, entrega de serviços</t>
         </is>
       </c>
       <c r="G28" t="n">
         <v>3</v>
       </c>
       <c r="H28" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="I28" t="n">
-        <v>362</v>
+        <v>336</v>
       </c>
       <c r="J28" t="n">
-        <v>24063</v>
+        <v>22414</v>
       </c>
       <c r="K28" t="n">
-        <v>15.04384324481569</v>
+        <v>14.99063085571518</v>
       </c>
       <c r="L28" t="n">
-        <v>33.42566943674976</v>
+        <v>31.02493074792244</v>
       </c>
       <c r="M28" t="inlineStr">
         <is>
@@ -3018,26 +3234,26 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Saúde - Doenças crônicas, cuidado do idoso, acesso</t>
+          <t>Comportamento Político - Qualidade de gestão, eficiência, entrega de serviços</t>
         </is>
       </c>
       <c r="G29" t="n">
         <v>4</v>
       </c>
       <c r="H29" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="I29" t="n">
-        <v>351</v>
+        <v>98</v>
       </c>
       <c r="J29" t="n">
-        <v>23436</v>
+        <v>7267</v>
       </c>
       <c r="K29" t="n">
-        <v>14.97695852534562</v>
+        <v>13.48561992569148</v>
       </c>
       <c r="L29" t="n">
-        <v>32.40997229916898</v>
+        <v>9.04893813481071</v>
       </c>
       <c r="M29" t="inlineStr">
         <is>
@@ -3073,26 +3289,26 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Saúde - UBS, consultas, exames básicos, acesso SUS</t>
+          <t>Religião e Valores - Religiosidade, valores morais, costumes, família</t>
         </is>
       </c>
       <c r="G30" t="n">
         <v>1</v>
       </c>
       <c r="H30" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="I30" t="n">
-        <v>314</v>
+        <v>301</v>
       </c>
       <c r="J30" t="n">
-        <v>24918</v>
+        <v>20374</v>
       </c>
       <c r="K30" t="n">
-        <v>12.60133237017417</v>
+        <v>14.77373122607245</v>
       </c>
       <c r="L30" t="n">
-        <v>28.99353647276085</v>
+        <v>27.79316712834719</v>
       </c>
       <c r="M30" t="inlineStr">
         <is>
@@ -3128,26 +3344,26 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Saúde - UBS, consultas, exames básicos, acesso SUS</t>
+          <t>Religião e Valores - Religiosidade, valores morais, costumes, família</t>
         </is>
       </c>
       <c r="G31" t="n">
         <v>2</v>
       </c>
       <c r="H31" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="I31" t="n">
-        <v>251</v>
+        <v>210</v>
       </c>
       <c r="J31" t="n">
-        <v>18295</v>
+        <v>16286</v>
       </c>
       <c r="K31" t="n">
-        <v>13.71959551790107</v>
+        <v>12.89451062262066</v>
       </c>
       <c r="L31" t="n">
-        <v>23.17636195752539</v>
+        <v>19.39058171745152</v>
       </c>
       <c r="M31" t="inlineStr">
         <is>
@@ -3183,26 +3399,26 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Saúde - UBS, consultas, exames básicos, acesso SUS</t>
+          <t>Religião e Valores - Religiosidade, valores morais, costumes, família</t>
         </is>
       </c>
       <c r="G32" t="n">
         <v>3</v>
       </c>
       <c r="H32" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="I32" t="n">
-        <v>221</v>
+        <v>317</v>
       </c>
       <c r="J32" t="n">
-        <v>14214</v>
+        <v>21370</v>
       </c>
       <c r="K32" t="n">
-        <v>15.54805121710989</v>
+        <v>14.83387927000468</v>
       </c>
       <c r="L32" t="n">
-        <v>20.40627885503232</v>
+        <v>29.27054478301016</v>
       </c>
       <c r="M32" t="inlineStr">
         <is>
@@ -3238,7 +3454,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Saúde - UBS, consultas, exames básicos, acesso SUS</t>
+          <t>Religião e Valores - Religiosidade, valores morais, costumes, família</t>
         </is>
       </c>
       <c r="G33" t="n">
@@ -3248,18 +3464,458 @@
         <v>9</v>
       </c>
       <c r="I33" t="n">
+        <v>255</v>
+      </c>
+      <c r="J33" t="n">
+        <v>16730</v>
+      </c>
+      <c r="K33" t="n">
+        <v>15.24208009563658</v>
+      </c>
+      <c r="L33" t="n">
+        <v>23.54570637119114</v>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>votos por mil</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>salto</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>RITA DE CASSIA TRINCA PASSOS</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>cidade_inteira</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Saúde - Doenças crônicas, cuidado do idoso, acesso</t>
+        </is>
+      </c>
+      <c r="G34" t="n">
+        <v>1</v>
+      </c>
+      <c r="H34" t="n">
+        <v>3</v>
+      </c>
+      <c r="I34" t="n">
+        <v>127</v>
+      </c>
+      <c r="J34" t="n">
+        <v>7202</v>
+      </c>
+      <c r="K34" t="n">
+        <v>17.63399055817828</v>
+      </c>
+      <c r="L34" t="n">
+        <v>11.72668513388735</v>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>votos por mil</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>salto</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>RITA DE CASSIA TRINCA PASSOS</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>cidade_inteira</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Saúde - Doenças crônicas, cuidado do idoso, acesso</t>
+        </is>
+      </c>
+      <c r="G35" t="n">
+        <v>2</v>
+      </c>
+      <c r="H35" t="n">
+        <v>8</v>
+      </c>
+      <c r="I35" t="n">
+        <v>243</v>
+      </c>
+      <c r="J35" t="n">
+        <v>20059</v>
+      </c>
+      <c r="K35" t="n">
+        <v>12.1142629243731</v>
+      </c>
+      <c r="L35" t="n">
+        <v>22.4376731301939</v>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>votos por mil</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>salto</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>RITA DE CASSIA TRINCA PASSOS</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>cidade_inteira</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Saúde - Doenças crônicas, cuidado do idoso, acesso</t>
+        </is>
+      </c>
+      <c r="G36" t="n">
+        <v>3</v>
+      </c>
+      <c r="H36" t="n">
+        <v>12</v>
+      </c>
+      <c r="I36" t="n">
+        <v>362</v>
+      </c>
+      <c r="J36" t="n">
+        <v>24063</v>
+      </c>
+      <c r="K36" t="n">
+        <v>15.04384324481569</v>
+      </c>
+      <c r="L36" t="n">
+        <v>33.42566943674976</v>
+      </c>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>votos por mil</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>salto</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>RITA DE CASSIA TRINCA PASSOS</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>cidade_inteira</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Saúde - Doenças crônicas, cuidado do idoso, acesso</t>
+        </is>
+      </c>
+      <c r="G37" t="n">
+        <v>4</v>
+      </c>
+      <c r="H37" t="n">
+        <v>9</v>
+      </c>
+      <c r="I37" t="n">
+        <v>351</v>
+      </c>
+      <c r="J37" t="n">
+        <v>23436</v>
+      </c>
+      <c r="K37" t="n">
+        <v>14.97695852534562</v>
+      </c>
+      <c r="L37" t="n">
+        <v>32.40997229916898</v>
+      </c>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>votos por mil</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>salto</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>RITA DE CASSIA TRINCA PASSOS</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>cidade_inteira</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Saúde - UBS, consultas, exames básicos, acesso SUS</t>
+        </is>
+      </c>
+      <c r="G38" t="n">
+        <v>1</v>
+      </c>
+      <c r="H38" t="n">
+        <v>10</v>
+      </c>
+      <c r="I38" t="n">
+        <v>314</v>
+      </c>
+      <c r="J38" t="n">
+        <v>24918</v>
+      </c>
+      <c r="K38" t="n">
+        <v>12.60133237017417</v>
+      </c>
+      <c r="L38" t="n">
+        <v>28.99353647276085</v>
+      </c>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>votos por mil</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>salto</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>RITA DE CASSIA TRINCA PASSOS</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>cidade_inteira</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Saúde - UBS, consultas, exames básicos, acesso SUS</t>
+        </is>
+      </c>
+      <c r="G39" t="n">
+        <v>2</v>
+      </c>
+      <c r="H39" t="n">
+        <v>8</v>
+      </c>
+      <c r="I39" t="n">
+        <v>251</v>
+      </c>
+      <c r="J39" t="n">
+        <v>18295</v>
+      </c>
+      <c r="K39" t="n">
+        <v>13.71959551790107</v>
+      </c>
+      <c r="L39" t="n">
+        <v>23.17636195752539</v>
+      </c>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>votos por mil</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>salto</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>RITA DE CASSIA TRINCA PASSOS</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>cidade_inteira</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Saúde - UBS, consultas, exames básicos, acesso SUS</t>
+        </is>
+      </c>
+      <c r="G40" t="n">
+        <v>3</v>
+      </c>
+      <c r="H40" t="n">
+        <v>5</v>
+      </c>
+      <c r="I40" t="n">
+        <v>221</v>
+      </c>
+      <c r="J40" t="n">
+        <v>14214</v>
+      </c>
+      <c r="K40" t="n">
+        <v>15.54805121710989</v>
+      </c>
+      <c r="L40" t="n">
+        <v>20.40627885503232</v>
+      </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>votos por mil</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>salto</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>RITA DE CASSIA TRINCA PASSOS</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>cidade_inteira</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Saúde - UBS, consultas, exames básicos, acesso SUS</t>
+        </is>
+      </c>
+      <c r="G41" t="n">
+        <v>4</v>
+      </c>
+      <c r="H41" t="n">
+        <v>9</v>
+      </c>
+      <c r="I41" t="n">
         <v>297</v>
       </c>
-      <c r="J33" t="n">
+      <c r="J41" t="n">
         <v>17333</v>
       </c>
-      <c r="K33" t="n">
+      <c r="K41" t="n">
         <v>17.13494490278659</v>
       </c>
-      <c r="L33" t="n">
+      <c r="L41" t="n">
         <v>27.42382271468144</v>
       </c>
-      <c r="M33" t="inlineStr">
+      <c r="M41" t="inlineStr">
         <is>
           <t>votos por mil</t>
         </is>

</xml_diff>

<commit_message>
Publica mapas XG-AE mapa_aderencia 2026-07-02 16:34:01
</commit_message>
<xml_diff>
--- a/mapas2/mapa_aderencia_xg_aderencia_eleitoral.xlsx
+++ b/mapas2/mapa_aderencia_xg_aderencia_eleitoral.xlsx
@@ -580,12 +580,12 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>RITA DE CASSIA TRINCA PASSOS</t>
+          <t>ROGERIO NOGUEIRA LOPES CRUZ</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>DEPUTADO FEDERAL</t>
+          <t>DEPUTADO ESTADUAL</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -600,37 +600,37 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Assistência Social - Proteção social, seguridade, assistência, rede pública</t>
+          <t>Proteção Animal - Proteção animal, bem-estar, resgate, políticas pets</t>
         </is>
       </c>
       <c r="I2" t="n">
         <v>1</v>
       </c>
       <c r="J2" t="n">
-        <v>71.77251483095174</v>
+        <v>43.76961846968661</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Aderência positiva moderada</t>
+          <t>Relação inversa moderada</t>
         </is>
       </c>
       <c r="L2" t="n">
-        <v>0.596922741358306</v>
+        <v>-0.2266143280393914</v>
       </c>
       <c r="M2" t="n">
-        <v>79.84613706791531</v>
+        <v>38.66928359803043</v>
       </c>
       <c r="N2" t="n">
-        <v>1.206765869092601</v>
+        <v>1.09404096406401</v>
       </c>
       <c r="O2" t="n">
-        <v>56.7786449623051</v>
+        <v>53.24166894561949</v>
       </c>
       <c r="P2" t="n">
-        <v>171.0927612606071</v>
+        <v>50.32344697494485</v>
       </c>
       <c r="Q2" t="n">
-        <v>206.4689047381093</v>
+        <v>55.05591244349274</v>
       </c>
       <c r="R2" t="inlineStr">
         <is>
@@ -641,7 +641,7 @@
         <v>36</v>
       </c>
       <c r="T2" t="n">
-        <v>16493</v>
+        <v>4722</v>
       </c>
       <c r="U2" t="n">
         <v>0</v>
@@ -661,12 +661,12 @@
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>C:\Users\guilh\Trabalho\Relatórios Alisson\Documentos gerais\Git\2\dataquadri\mapas2\mapa_aderencia_rita_itu_sp_2022_assistencia_social_protecao_social_seguridade_assistencia_rede_publica_cidade_inteira.html</t>
+          <t>C:\Users\guilh\Trabalho\Relatórios Alisson\Documentos gerais\Git\2\dataquadri\mapas2\mapa_aderencia_rogerio_itu_sp_2022_protecao_animal_protecao_animal_bem_estar_resgate_politicas_pets_cidade_inteira.html</t>
         </is>
       </c>
       <c r="Z2" t="inlineStr">
         <is>
-          <t>https://quadrifygit.github.io/dataquadri/mapas2/mapa_aderencia_rita_itu_sp_2022_assistencia_social_protecao_social_seguridade_assistencia_rede_publica_cidade_inteira.html</t>
+          <t>https://quadrifygit.github.io/dataquadri/mapas2/mapa_aderencia_rogerio_itu_sp_2022_protecao_animal_protecao_animal_bem_estar_resgate_politicas_pets_cidade_inteira.html</t>
         </is>
       </c>
     </row>
@@ -688,12 +688,12 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>RITA DE CASSIA TRINCA PASSOS</t>
+          <t>ROGERIO NOGUEIRA LOPES CRUZ</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>DEPUTADO FEDERAL</t>
+          <t>DEPUTADO ESTADUAL</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -708,37 +708,37 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Saúde - UBS, consultas, exames básicos, acesso SUS</t>
+          <t>Comportamento Político - Qualidade de gestão, eficiência, entrega de serviços</t>
         </is>
       </c>
       <c r="I3" t="n">
         <v>2</v>
       </c>
       <c r="J3" t="n">
-        <v>71.53817501445646</v>
+        <v>42.73191145739839</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Aderência positiva moderada</t>
+          <t>Relação inversa moderada</t>
         </is>
       </c>
       <c r="L3" t="n">
-        <v>0.5897122854661436</v>
+        <v>-0.2353698816227315</v>
       </c>
       <c r="M3" t="n">
-        <v>79.48561427330718</v>
+        <v>38.23150591886343</v>
       </c>
       <c r="N3" t="n">
-        <v>1.206765869092601</v>
+        <v>1.030677011112459</v>
       </c>
       <c r="O3" t="n">
-        <v>56.7786449623051</v>
+        <v>51.08980745753475</v>
       </c>
       <c r="P3" t="n">
-        <v>171.0927612606071</v>
+        <v>50.32344697494485</v>
       </c>
       <c r="Q3" t="n">
-        <v>206.4689047381093</v>
+        <v>51.86721991701245</v>
       </c>
       <c r="R3" t="inlineStr">
         <is>
@@ -749,7 +749,7 @@
         <v>36</v>
       </c>
       <c r="T3" t="n">
-        <v>16493</v>
+        <v>4722</v>
       </c>
       <c r="U3" t="n">
         <v>0</v>
@@ -769,12 +769,12 @@
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>C:\Users\guilh\Trabalho\Relatórios Alisson\Documentos gerais\Git\2\dataquadri\mapas2\mapa_aderencia_rita_itu_sp_2022_saude_ubs_consultas_exames_basicos_acesso_sus_cidade_inteira.html</t>
+          <t>C:\Users\guilh\Trabalho\Relatórios Alisson\Documentos gerais\Git\2\dataquadri\mapas2\mapa_aderencia_rogerio_itu_sp_2022_comportamento_politico_qualidade_de_gestao_eficiencia_entrega_de_servicos_cidade_inteira.html</t>
         </is>
       </c>
       <c r="Z3" t="inlineStr">
         <is>
-          <t>https://quadrifygit.github.io/dataquadri/mapas2/mapa_aderencia_rita_itu_sp_2022_saude_ubs_consultas_exames_basicos_acesso_sus_cidade_inteira.html</t>
+          <t>https://quadrifygit.github.io/dataquadri/mapas2/mapa_aderencia_rogerio_itu_sp_2022_comportamento_politico_qualidade_de_gestao_eficiencia_entrega_de_servicos_cidade_inteira.html</t>
         </is>
       </c>
     </row>
@@ -796,12 +796,12 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>RITA DE CASSIA TRINCA PASSOS</t>
+          <t>ROGERIO NOGUEIRA LOPES CRUZ</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>DEPUTADO FEDERAL</t>
+          <t>DEPUTADO ESTADUAL</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -816,37 +816,37 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Religião e Valores - Religiosidade, valores morais, costumes, família</t>
+          <t>Mobilidade e Acessibilidade - Transporte, calçadas, acesso a serviços, mobilidade</t>
         </is>
       </c>
       <c r="I4" t="n">
         <v>3</v>
       </c>
       <c r="J4" t="n">
-        <v>69.63056526675756</v>
+        <v>34.71562985569617</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Aderência positiva moderada</t>
+          <t>Relação inversa moderada</t>
         </is>
       </c>
       <c r="L4" t="n">
-        <v>0.5279083778190369</v>
+        <v>-0.2866156217134576</v>
       </c>
       <c r="M4" t="n">
-        <v>76.39541889095185</v>
+        <v>35.66921891432712</v>
       </c>
       <c r="N4" t="n">
-        <v>1.216461471554447</v>
+        <v>0.6232086443536621</v>
       </c>
       <c r="O4" t="n">
-        <v>57.06726567896817</v>
+        <v>32.94467874681013</v>
       </c>
       <c r="P4" t="n">
-        <v>171.0927612606071</v>
+        <v>50.32344697494485</v>
       </c>
       <c r="Q4" t="n">
-        <v>208.1277521353918</v>
+        <v>31.36200716845878</v>
       </c>
       <c r="R4" t="inlineStr">
         <is>
@@ -857,7 +857,7 @@
         <v>36</v>
       </c>
       <c r="T4" t="n">
-        <v>16493</v>
+        <v>4722</v>
       </c>
       <c r="U4" t="n">
         <v>0</v>
@@ -877,12 +877,12 @@
       </c>
       <c r="Y4" t="inlineStr">
         <is>
-          <t>C:\Users\guilh\Trabalho\Relatórios Alisson\Documentos gerais\Git\2\dataquadri\mapas2\mapa_aderencia_rita_itu_sp_2022_religiao_e_valores_religiosidade_valores_morais_costumes_familia_cidade_inteira.html</t>
+          <t>C:\Users\guilh\Trabalho\Relatórios Alisson\Documentos gerais\Git\2\dataquadri\mapas2\mapa_aderencia_rogerio_itu_sp_2022_mobilidade_e_acessibilidade_transporte_calcadas_acesso_a_servicos_mobilidade_cidade_inteira.html</t>
         </is>
       </c>
       <c r="Z4" t="inlineStr">
         <is>
-          <t>https://quadrifygit.github.io/dataquadri/mapas2/mapa_aderencia_rita_itu_sp_2022_religiao_e_valores_religiosidade_valores_morais_costumes_familia_cidade_inteira.html</t>
+          <t>https://quadrifygit.github.io/dataquadri/mapas2/mapa_aderencia_rogerio_itu_sp_2022_mobilidade_e_acessibilidade_transporte_calcadas_acesso_a_servicos_mobilidade_cidade_inteira.html</t>
         </is>
       </c>
     </row>
@@ -904,12 +904,12 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>RITA DE CASSIA TRINCA PASSOS</t>
+          <t>ROGERIO NOGUEIRA LOPES CRUZ</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>DEPUTADO FEDERAL</t>
+          <t>DEPUTADO ESTADUAL</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -924,37 +924,37 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Saúde - Doenças crônicas, cuidado do idoso, acesso</t>
+          <t>Saúde - UBS, consultas, exames básicos, acesso SUS</t>
         </is>
       </c>
       <c r="I5" t="n">
         <v>4</v>
       </c>
       <c r="J5" t="n">
-        <v>58.94742612227699</v>
+        <v>28.76619148168748</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Relação fraca ou neutra</t>
+          <t>Forte relação inversa</t>
         </is>
       </c>
       <c r="L5" t="n">
-        <v>0.2541685701987265</v>
+        <v>-0.5567502013876867</v>
       </c>
       <c r="M5" t="n">
-        <v>62.70842850993632</v>
+        <v>22.16248993061566</v>
       </c>
       <c r="N5" t="n">
-        <v>1.055925680072127</v>
+        <v>0.7798174513384127</v>
       </c>
       <c r="O5" t="n">
-        <v>51.96270740233822</v>
+        <v>41.03020864796372</v>
       </c>
       <c r="P5" t="n">
-        <v>171.0927612606071</v>
+        <v>50.32344697494485</v>
       </c>
       <c r="Q5" t="n">
-        <v>180.6612402895246</v>
+        <v>39.24310216256525</v>
       </c>
       <c r="R5" t="inlineStr">
         <is>
@@ -965,7 +965,7 @@
         <v>36</v>
       </c>
       <c r="T5" t="n">
-        <v>16493</v>
+        <v>4722</v>
       </c>
       <c r="U5" t="n">
         <v>0</v>
@@ -985,12 +985,12 @@
       </c>
       <c r="Y5" t="inlineStr">
         <is>
-          <t>C:\Users\guilh\Trabalho\Relatórios Alisson\Documentos gerais\Git\2\dataquadri\mapas2\mapa_aderencia_rita_itu_sp_2022_saude_doencas_cronicas_cuidado_do_idoso_acesso_cidade_inteira.html</t>
+          <t>C:\Users\guilh\Trabalho\Relatórios Alisson\Documentos gerais\Git\2\dataquadri\mapas2\mapa_aderencia_rogerio_itu_sp_2022_saude_ubs_consultas_exames_basicos_acesso_sus_cidade_inteira.html</t>
         </is>
       </c>
       <c r="Z5" t="inlineStr">
         <is>
-          <t>https://quadrifygit.github.io/dataquadri/mapas2/mapa_aderencia_rita_itu_sp_2022_saude_doencas_cronicas_cuidado_do_idoso_acesso_cidade_inteira.html</t>
+          <t>https://quadrifygit.github.io/dataquadri/mapas2/mapa_aderencia_rogerio_itu_sp_2022_saude_ubs_consultas_exames_basicos_acesso_sus_cidade_inteira.html</t>
         </is>
       </c>
     </row>
@@ -1012,12 +1012,12 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>RITA DE CASSIA TRINCA PASSOS</t>
+          <t>ROGERIO NOGUEIRA LOPES CRUZ</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>DEPUTADO FEDERAL</t>
+          <t>DEPUTADO ESTADUAL</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -1032,37 +1032,37 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Comportamento Político - Qualidade de gestão, eficiência, entrega de serviços</t>
+          <t>Assistência Social - Proteção social, seguridade, assistência, rede pública</t>
         </is>
       </c>
       <c r="I6" t="n">
         <v>5</v>
       </c>
       <c r="J6" t="n">
-        <v>41.94822057230441</v>
+        <v>28.69923724840312</v>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Relação inversa moderada</t>
+          <t>Forte relação inversa</t>
         </is>
       </c>
       <c r="L6" t="n">
-        <v>-0.1709908111569954</v>
+        <v>-0.5588103316425902</v>
       </c>
       <c r="M6" t="n">
-        <v>41.45045944215023</v>
+        <v>22.05948341787049</v>
       </c>
       <c r="N6" t="n">
-        <v>0.8206877726483239</v>
+        <v>0.7798174513384127</v>
       </c>
       <c r="O6" t="n">
-        <v>42.8726340997336</v>
+        <v>41.03020864796372</v>
       </c>
       <c r="P6" t="n">
-        <v>171.0927612606071</v>
+        <v>50.32344697494485</v>
       </c>
       <c r="Q6" t="n">
-        <v>140.4137371552191</v>
+        <v>39.24310216256525</v>
       </c>
       <c r="R6" t="inlineStr">
         <is>
@@ -1073,7 +1073,7 @@
         <v>36</v>
       </c>
       <c r="T6" t="n">
-        <v>16493</v>
+        <v>4722</v>
       </c>
       <c r="U6" t="n">
         <v>0</v>
@@ -1093,12 +1093,12 @@
       </c>
       <c r="Y6" t="inlineStr">
         <is>
-          <t>C:\Users\guilh\Trabalho\Relatórios Alisson\Documentos gerais\Git\2\dataquadri\mapas2\mapa_aderencia_rita_itu_sp_2022_comportamento_politico_qualidade_de_gestao_eficiencia_entrega_de_servicos_cidade_inteira.html</t>
+          <t>C:\Users\guilh\Trabalho\Relatórios Alisson\Documentos gerais\Git\2\dataquadri\mapas2\mapa_aderencia_rogerio_itu_sp_2022_assistencia_social_protecao_social_seguridade_assistencia_rede_publica_cidade_inteira.html</t>
         </is>
       </c>
       <c r="Z6" t="inlineStr">
         <is>
-          <t>https://quadrifygit.github.io/dataquadri/mapas2/mapa_aderencia_rita_itu_sp_2022_comportamento_politico_qualidade_de_gestao_eficiencia_entrega_de_servicos_cidade_inteira.html</t>
+          <t>https://quadrifygit.github.io/dataquadri/mapas2/mapa_aderencia_rogerio_itu_sp_2022_assistencia_social_protecao_social_seguridade_assistencia_rede_publica_cidade_inteira.html</t>
         </is>
       </c>
     </row>
@@ -1120,12 +1120,12 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>RITA DE CASSIA TRINCA PASSOS</t>
+          <t>ROGERIO NOGUEIRA LOPES CRUZ</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>DEPUTADO FEDERAL</t>
+          <t>DEPUTADO ESTADUAL</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -1140,14 +1140,14 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Saúde - UBS, consultas, exames básicos, acesso SUS</t>
+          <t>Mobilidade e Acessibilidade - Transporte, calçadas, acesso a serviços, mobilidade</t>
         </is>
       </c>
       <c r="I7" t="n">
         <v>1</v>
       </c>
       <c r="J7" t="n">
-        <v>66.65348872129978</v>
+        <v>63.30874465234245</v>
       </c>
       <c r="K7" t="inlineStr">
         <is>
@@ -1155,22 +1155,22 @@
         </is>
       </c>
       <c r="L7" t="n">
-        <v>0.4471947495393861</v>
+        <v>0.4167583705219454</v>
       </c>
       <c r="M7" t="n">
-        <v>72.35973747696931</v>
+        <v>70.83791852609727</v>
       </c>
       <c r="N7" t="n">
-        <v>1.182833315726986</v>
+        <v>0.9814860902605079</v>
       </c>
       <c r="O7" t="n">
-        <v>56.05616960362779</v>
+        <v>49.32599317251208</v>
       </c>
       <c r="P7" t="n">
-        <v>14.48635634028892</v>
+        <v>240.4783054321831</v>
       </c>
       <c r="Q7" t="n">
-        <v>17.13494490278659</v>
+        <v>236.0261117911057</v>
       </c>
       <c r="R7" t="inlineStr">
         <is>
@@ -1181,7 +1181,7 @@
         <v>32</v>
       </c>
       <c r="T7" t="n">
-        <v>1083</v>
+        <v>17597</v>
       </c>
       <c r="U7" t="n">
         <v>0</v>
@@ -1201,12 +1201,12 @@
       </c>
       <c r="Y7" t="inlineStr">
         <is>
-          <t>C:\Users\guilh\Trabalho\Relatórios Alisson\Documentos gerais\Git\2\dataquadri\mapas2\mapa_aderencia_rita_salto_sp_2022_saude_ubs_consultas_exames_basicos_acesso_sus_cidade_inteira.html</t>
+          <t>C:\Users\guilh\Trabalho\Relatórios Alisson\Documentos gerais\Git\2\dataquadri\mapas2\mapa_aderencia_rogerio_salto_sp_2022_mobilidade_e_acessibilidade_transporte_calcadas_acesso_a_servicos_mobilidade_cidade_inteira.html</t>
         </is>
       </c>
       <c r="Z7" t="inlineStr">
         <is>
-          <t>https://quadrifygit.github.io/dataquadri/mapas2/mapa_aderencia_rita_salto_sp_2022_saude_ubs_consultas_exames_basicos_acesso_sus_cidade_inteira.html</t>
+          <t>https://quadrifygit.github.io/dataquadri/mapas2/mapa_aderencia_rogerio_salto_sp_2022_mobilidade_e_acessibilidade_transporte_calcadas_acesso_a_servicos_mobilidade_cidade_inteira.html</t>
         </is>
       </c>
     </row>
@@ -1228,12 +1228,12 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>RITA DE CASSIA TRINCA PASSOS</t>
+          <t>ROGERIO NOGUEIRA LOPES CRUZ</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>DEPUTADO FEDERAL</t>
+          <t>DEPUTADO ESTADUAL</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -1255,7 +1255,7 @@
         <v>2</v>
       </c>
       <c r="J8" t="n">
-        <v>66.21252792890854</v>
+        <v>60.40720914054178</v>
       </c>
       <c r="K8" t="inlineStr">
         <is>
@@ -1263,22 +1263,22 @@
         </is>
       </c>
       <c r="L8" t="n">
-        <v>0.4336267251581173</v>
+        <v>0.321048793129752</v>
       </c>
       <c r="M8" t="n">
-        <v>71.68133625790587</v>
+        <v>66.05243965648761</v>
       </c>
       <c r="N8" t="n">
-        <v>1.182833315726986</v>
+        <v>0.9978731832195397</v>
       </c>
       <c r="O8" t="n">
-        <v>56.05616960362779</v>
+        <v>49.9232096109281</v>
       </c>
       <c r="P8" t="n">
-        <v>14.48635634028892</v>
+        <v>240.4783054321831</v>
       </c>
       <c r="Q8" t="n">
-        <v>17.13494490278659</v>
+        <v>239.9668521368533</v>
       </c>
       <c r="R8" t="inlineStr">
         <is>
@@ -1289,7 +1289,7 @@
         <v>32</v>
       </c>
       <c r="T8" t="n">
-        <v>1083</v>
+        <v>17597</v>
       </c>
       <c r="U8" t="n">
         <v>0</v>
@@ -1309,12 +1309,12 @@
       </c>
       <c r="Y8" t="inlineStr">
         <is>
-          <t>C:\Users\guilh\Trabalho\Relatórios Alisson\Documentos gerais\Git\2\dataquadri\mapas2\mapa_aderencia_rita_salto_sp_2022_assistencia_social_protecao_social_seguridade_assistencia_rede_publica_cidade_inteira.html</t>
+          <t>C:\Users\guilh\Trabalho\Relatórios Alisson\Documentos gerais\Git\2\dataquadri\mapas2\mapa_aderencia_rogerio_salto_sp_2022_assistencia_social_protecao_social_seguridade_assistencia_rede_publica_cidade_inteira.html</t>
         </is>
       </c>
       <c r="Z8" t="inlineStr">
         <is>
-          <t>https://quadrifygit.github.io/dataquadri/mapas2/mapa_aderencia_rita_salto_sp_2022_assistencia_social_protecao_social_seguridade_assistencia_rede_publica_cidade_inteira.html</t>
+          <t>https://quadrifygit.github.io/dataquadri/mapas2/mapa_aderencia_rogerio_salto_sp_2022_assistencia_social_protecao_social_seguridade_assistencia_rede_publica_cidade_inteira.html</t>
         </is>
       </c>
     </row>
@@ -1336,12 +1336,12 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>RITA DE CASSIA TRINCA PASSOS</t>
+          <t>ROGERIO NOGUEIRA LOPES CRUZ</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>DEPUTADO FEDERAL</t>
+          <t>DEPUTADO ESTADUAL</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -1356,37 +1356,37 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Saúde - Doenças crônicas, cuidado do idoso, acesso</t>
+          <t>Saúde - UBS, consultas, exames básicos, acesso SUS</t>
         </is>
       </c>
       <c r="I9" t="n">
         <v>3</v>
       </c>
       <c r="J9" t="n">
-        <v>54.93134641137685</v>
+        <v>60.29994840725742</v>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>Relação fraca ou neutra</t>
+          <t>Aderência positiva moderada</t>
         </is>
       </c>
       <c r="L9" t="n">
-        <v>0.1387972223867631</v>
+        <v>0.3177484628748488</v>
       </c>
       <c r="M9" t="n">
-        <v>56.93986111933815</v>
+        <v>65.88742314374244</v>
       </c>
       <c r="N9" t="n">
-        <v>1.033866499865964</v>
+        <v>0.9978731832195397</v>
       </c>
       <c r="O9" t="n">
-        <v>51.20124766802015</v>
+        <v>49.9232096109281</v>
       </c>
       <c r="P9" t="n">
-        <v>14.48635634028892</v>
+        <v>240.4783054321831</v>
       </c>
       <c r="Q9" t="n">
-        <v>14.97695852534562</v>
+        <v>239.9668521368533</v>
       </c>
       <c r="R9" t="inlineStr">
         <is>
@@ -1397,7 +1397,7 @@
         <v>32</v>
       </c>
       <c r="T9" t="n">
-        <v>1083</v>
+        <v>17597</v>
       </c>
       <c r="U9" t="n">
         <v>0</v>
@@ -1417,12 +1417,12 @@
       </c>
       <c r="Y9" t="inlineStr">
         <is>
-          <t>C:\Users\guilh\Trabalho\Relatórios Alisson\Documentos gerais\Git\2\dataquadri\mapas2\mapa_aderencia_rita_salto_sp_2022_saude_doencas_cronicas_cuidado_do_idoso_acesso_cidade_inteira.html</t>
+          <t>C:\Users\guilh\Trabalho\Relatórios Alisson\Documentos gerais\Git\2\dataquadri\mapas2\mapa_aderencia_rogerio_salto_sp_2022_saude_ubs_consultas_exames_basicos_acesso_sus_cidade_inteira.html</t>
         </is>
       </c>
       <c r="Z9" t="inlineStr">
         <is>
-          <t>https://quadrifygit.github.io/dataquadri/mapas2/mapa_aderencia_rita_salto_sp_2022_saude_doencas_cronicas_cuidado_do_idoso_acesso_cidade_inteira.html</t>
+          <t>https://quadrifygit.github.io/dataquadri/mapas2/mapa_aderencia_rogerio_salto_sp_2022_saude_ubs_consultas_exames_basicos_acesso_sus_cidade_inteira.html</t>
         </is>
       </c>
     </row>
@@ -1444,12 +1444,12 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>RITA DE CASSIA TRINCA PASSOS</t>
+          <t>ROGERIO NOGUEIRA LOPES CRUZ</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>DEPUTADO FEDERAL</t>
+          <t>DEPUTADO ESTADUAL</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -1464,14 +1464,14 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Religião e Valores - Religiosidade, valores morais, costumes, família</t>
+          <t>Comportamento Político - Qualidade de gestão, eficiência, entrega de serviços</t>
         </is>
       </c>
       <c r="I10" t="n">
         <v>4</v>
       </c>
       <c r="J10" t="n">
-        <v>53.79421781101134</v>
+        <v>55.6793858563519</v>
       </c>
       <c r="K10" t="inlineStr">
         <is>
@@ -1479,22 +1479,22 @@
         </is>
       </c>
       <c r="L10" t="n">
-        <v>0.09699303915798903</v>
+        <v>0.1762009652756663</v>
       </c>
       <c r="M10" t="n">
-        <v>54.84965195789945</v>
+        <v>58.81004826378331</v>
       </c>
       <c r="N10" t="n">
-        <v>1.052167966712642</v>
+        <v>0.9962722475706126</v>
       </c>
       <c r="O10" t="n">
-        <v>51.83412582393341</v>
+        <v>49.86529852826499</v>
       </c>
       <c r="P10" t="n">
-        <v>14.48635634028892</v>
+        <v>240.4783054321831</v>
       </c>
       <c r="Q10" t="n">
-        <v>15.24208009563658</v>
+        <v>239.5818618448934</v>
       </c>
       <c r="R10" t="inlineStr">
         <is>
@@ -1505,7 +1505,7 @@
         <v>32</v>
       </c>
       <c r="T10" t="n">
-        <v>1083</v>
+        <v>17597</v>
       </c>
       <c r="U10" t="n">
         <v>0</v>
@@ -1525,12 +1525,12 @@
       </c>
       <c r="Y10" t="inlineStr">
         <is>
-          <t>C:\Users\guilh\Trabalho\Relatórios Alisson\Documentos gerais\Git\2\dataquadri\mapas2\mapa_aderencia_rita_salto_sp_2022_religiao_e_valores_religiosidade_valores_morais_costumes_familia_cidade_inteira.html</t>
+          <t>C:\Users\guilh\Trabalho\Relatórios Alisson\Documentos gerais\Git\2\dataquadri\mapas2\mapa_aderencia_rogerio_salto_sp_2022_comportamento_politico_qualidade_de_gestao_eficiencia_entrega_de_servicos_cidade_inteira.html</t>
         </is>
       </c>
       <c r="Z10" t="inlineStr">
         <is>
-          <t>https://quadrifygit.github.io/dataquadri/mapas2/mapa_aderencia_rita_salto_sp_2022_religiao_e_valores_religiosidade_valores_morais_costumes_familia_cidade_inteira.html</t>
+          <t>https://quadrifygit.github.io/dataquadri/mapas2/mapa_aderencia_rogerio_salto_sp_2022_comportamento_politico_qualidade_de_gestao_eficiencia_entrega_de_servicos_cidade_inteira.html</t>
         </is>
       </c>
     </row>
@@ -1552,12 +1552,12 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>RITA DE CASSIA TRINCA PASSOS</t>
+          <t>ROGERIO NOGUEIRA LOPES CRUZ</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>DEPUTADO FEDERAL</t>
+          <t>DEPUTADO ESTADUAL</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -1572,14 +1572,14 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Comportamento Político - Qualidade de gestão, eficiência, entrega de serviços</t>
+          <t>Proteção Animal - Proteção animal, bem-estar, resgate, políticas pets</t>
         </is>
       </c>
       <c r="I11" t="n">
         <v>5</v>
       </c>
       <c r="J11" t="n">
-        <v>53.27357156732022</v>
+        <v>53.43884739138753</v>
       </c>
       <c r="K11" t="inlineStr">
         <is>
@@ -1587,22 +1587,22 @@
         </is>
       </c>
       <c r="L11" t="n">
-        <v>0.1285295282603976</v>
+        <v>0.09479281898805356</v>
       </c>
       <c r="M11" t="n">
-        <v>56.42647641301988</v>
+        <v>54.73964094940268</v>
       </c>
       <c r="N11" t="n">
-        <v>0.9309186940394231</v>
+        <v>1.028772167187943</v>
       </c>
       <c r="O11" t="n">
-        <v>47.41817685387798</v>
+        <v>51.02308792650224</v>
       </c>
       <c r="P11" t="n">
-        <v>14.48635634028892</v>
+        <v>240.4783054321831</v>
       </c>
       <c r="Q11" t="n">
-        <v>13.48561992569148</v>
+        <v>247.3973874411511</v>
       </c>
       <c r="R11" t="inlineStr">
         <is>
@@ -1613,7 +1613,7 @@
         <v>32</v>
       </c>
       <c r="T11" t="n">
-        <v>1083</v>
+        <v>17597</v>
       </c>
       <c r="U11" t="n">
         <v>0</v>
@@ -1633,12 +1633,12 @@
       </c>
       <c r="Y11" t="inlineStr">
         <is>
-          <t>C:\Users\guilh\Trabalho\Relatórios Alisson\Documentos gerais\Git\2\dataquadri\mapas2\mapa_aderencia_rita_salto_sp_2022_comportamento_politico_qualidade_de_gestao_eficiencia_entrega_de_servicos_cidade_inteira.html</t>
+          <t>C:\Users\guilh\Trabalho\Relatórios Alisson\Documentos gerais\Git\2\dataquadri\mapas2\mapa_aderencia_rogerio_salto_sp_2022_protecao_animal_protecao_animal_bem_estar_resgate_politicas_pets_cidade_inteira.html</t>
         </is>
       </c>
       <c r="Z11" t="inlineStr">
         <is>
-          <t>https://quadrifygit.github.io/dataquadri/mapas2/mapa_aderencia_rita_salto_sp_2022_comportamento_politico_qualidade_de_gestao_eficiencia_entrega_de_servicos_cidade_inteira.html</t>
+          <t>https://quadrifygit.github.io/dataquadri/mapas2/mapa_aderencia_rogerio_salto_sp_2022_protecao_animal_protecao_animal_bem_estar_resgate_politicas_pets_cidade_inteira.html</t>
         </is>
       </c>
     </row>
@@ -1741,7 +1741,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>RITA DE CASSIA TRINCA PASSOS</t>
+          <t>ROGERIO NOGUEIRA LOPES CRUZ</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -1761,16 +1761,16 @@
         <v>14</v>
       </c>
       <c r="I2" t="n">
-        <v>6374</v>
+        <v>2445</v>
       </c>
       <c r="J2" t="n">
-        <v>44118</v>
+        <v>43069</v>
       </c>
       <c r="K2" t="n">
-        <v>144.4761775239132</v>
+        <v>56.76937008056839</v>
       </c>
       <c r="L2" t="n">
-        <v>38.64669859940581</v>
+        <v>51.77890724269377</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
@@ -1796,7 +1796,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>RITA DE CASSIA TRINCA PASSOS</t>
+          <t>ROGERIO NOGUEIRA LOPES CRUZ</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -1816,16 +1816,16 @@
         <v>8</v>
       </c>
       <c r="I3" t="n">
-        <v>3266</v>
+        <v>966</v>
       </c>
       <c r="J3" t="n">
-        <v>19250</v>
+        <v>18608</v>
       </c>
       <c r="K3" t="n">
-        <v>169.6623376623376</v>
+        <v>51.91315563198624</v>
       </c>
       <c r="L3" t="n">
-        <v>19.80234038683078</v>
+        <v>20.4574332909784</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>
@@ -1851,7 +1851,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>RITA DE CASSIA TRINCA PASSOS</t>
+          <t>ROGERIO NOGUEIRA LOPES CRUZ</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -1871,16 +1871,16 @@
         <v>4</v>
       </c>
       <c r="I4" t="n">
-        <v>2308</v>
+        <v>469</v>
       </c>
       <c r="J4" t="n">
-        <v>11017</v>
+        <v>10700</v>
       </c>
       <c r="K4" t="n">
-        <v>209.4944177180721</v>
+        <v>43.83177570093458</v>
       </c>
       <c r="L4" t="n">
-        <v>13.99381555811556</v>
+        <v>9.932232105040237</v>
       </c>
       <c r="M4" t="inlineStr">
         <is>
@@ -1906,7 +1906,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>RITA DE CASSIA TRINCA PASSOS</t>
+          <t>ROGERIO NOGUEIRA LOPES CRUZ</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -1926,16 +1926,16 @@
         <v>10</v>
       </c>
       <c r="I5" t="n">
-        <v>4545</v>
+        <v>842</v>
       </c>
       <c r="J5" t="n">
-        <v>22013</v>
+        <v>21456</v>
       </c>
       <c r="K5" t="n">
-        <v>206.4689047381093</v>
+        <v>39.24310216256525</v>
       </c>
       <c r="L5" t="n">
-        <v>27.55714545564785</v>
+        <v>17.83142736128759</v>
       </c>
       <c r="M5" t="inlineStr">
         <is>
@@ -1961,7 +1961,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>RITA DE CASSIA TRINCA PASSOS</t>
+          <t>ROGERIO NOGUEIRA LOPES CRUZ</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -1981,16 +1981,16 @@
         <v>1</v>
       </c>
       <c r="I6" t="n">
-        <v>411</v>
+        <v>179</v>
       </c>
       <c r="J6" t="n">
-        <v>2386</v>
+        <v>2311</v>
       </c>
       <c r="K6" t="n">
-        <v>172.254819782062</v>
+        <v>77.45564690610125</v>
       </c>
       <c r="L6" t="n">
-        <v>2.491966288728551</v>
+        <v>3.790766624311733</v>
       </c>
       <c r="M6" t="inlineStr">
         <is>
@@ -2016,7 +2016,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>RITA DE CASSIA TRINCA PASSOS</t>
+          <t>ROGERIO NOGUEIRA LOPES CRUZ</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -2036,16 +2036,16 @@
         <v>16</v>
       </c>
       <c r="I7" t="n">
-        <v>8843</v>
+        <v>2246</v>
       </c>
       <c r="J7" t="n">
-        <v>47466</v>
+        <v>46189</v>
       </c>
       <c r="K7" t="n">
-        <v>186.3017739013188</v>
+        <v>48.62629630431488</v>
       </c>
       <c r="L7" t="n">
-        <v>53.61668586673134</v>
+        <v>47.56459127488352</v>
       </c>
       <c r="M7" t="inlineStr">
         <is>
@@ -2071,7 +2071,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>RITA DE CASSIA TRINCA PASSOS</t>
+          <t>ROGERIO NOGUEIRA LOPES CRUZ</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -2091,16 +2091,16 @@
         <v>10</v>
       </c>
       <c r="I8" t="n">
-        <v>5162</v>
+        <v>1547</v>
       </c>
       <c r="J8" t="n">
-        <v>31754</v>
+        <v>30873</v>
       </c>
       <c r="K8" t="n">
-        <v>162.562196888581</v>
+        <v>50.10850905321802</v>
       </c>
       <c r="L8" t="n">
-        <v>31.29812647789971</v>
+        <v>32.76154171961034</v>
       </c>
       <c r="M8" t="inlineStr">
         <is>
@@ -2126,7 +2126,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>RITA DE CASSIA TRINCA PASSOS</t>
+          <t>ROGERIO NOGUEIRA LOPES CRUZ</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -2146,16 +2146,16 @@
         <v>9</v>
       </c>
       <c r="I9" t="n">
-        <v>2077</v>
+        <v>750</v>
       </c>
       <c r="J9" t="n">
-        <v>14792</v>
+        <v>14460</v>
       </c>
       <c r="K9" t="n">
-        <v>140.4137371552191</v>
+        <v>51.86721991701245</v>
       </c>
       <c r="L9" t="n">
-        <v>12.59322136664039</v>
+        <v>15.88310038119441</v>
       </c>
       <c r="M9" t="inlineStr">
         <is>
@@ -2181,7 +2181,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>RITA DE CASSIA TRINCA PASSOS</t>
+          <t>ROGERIO NOGUEIRA LOPES CRUZ</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -2191,26 +2191,26 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Religião e Valores - Religiosidade, valores morais, costumes, família</t>
+          <t>Mobilidade e Acessibilidade - Transporte, calçadas, acesso a serviços, mobilidade</t>
         </is>
       </c>
       <c r="G10" t="n">
         <v>1</v>
       </c>
       <c r="H10" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="I10" t="n">
-        <v>5282</v>
+        <v>2149</v>
       </c>
       <c r="J10" t="n">
-        <v>37231</v>
+        <v>40283</v>
       </c>
       <c r="K10" t="n">
-        <v>141.8710214606108</v>
+        <v>53.3475659707569</v>
       </c>
       <c r="L10" t="n">
-        <v>32.02570787606864</v>
+        <v>45.51037695891571</v>
       </c>
       <c r="M10" t="inlineStr">
         <is>
@@ -2236,7 +2236,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>RITA DE CASSIA TRINCA PASSOS</t>
+          <t>ROGERIO NOGUEIRA LOPES CRUZ</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -2246,26 +2246,26 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Religião e Valores - Religiosidade, valores morais, costumes, família</t>
+          <t>Mobilidade e Acessibilidade - Transporte, calçadas, acesso a serviços, mobilidade</t>
         </is>
       </c>
       <c r="G11" t="n">
         <v>2</v>
       </c>
       <c r="H11" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="I11" t="n">
-        <v>4714</v>
+        <v>1154</v>
       </c>
       <c r="J11" t="n">
-        <v>27516</v>
+        <v>20731</v>
       </c>
       <c r="K11" t="n">
-        <v>171.3185055967437</v>
+        <v>55.66542858521056</v>
       </c>
       <c r="L11" t="n">
-        <v>28.58182259140241</v>
+        <v>24.43879711986446</v>
       </c>
       <c r="M11" t="inlineStr">
         <is>
@@ -2291,7 +2291,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>RITA DE CASSIA TRINCA PASSOS</t>
+          <t>ROGERIO NOGUEIRA LOPES CRUZ</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -2301,26 +2301,26 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Religião e Valores - Religiosidade, valores morais, costumes, família</t>
+          <t>Mobilidade e Acessibilidade - Transporte, calçadas, acesso a serviços, mobilidade</t>
         </is>
       </c>
       <c r="G12" t="n">
         <v>3</v>
       </c>
       <c r="H12" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="I12" t="n">
-        <v>2574</v>
+        <v>1314</v>
       </c>
       <c r="J12" t="n">
-        <v>12802</v>
+        <v>29471</v>
       </c>
       <c r="K12" t="n">
-        <v>201.0623340103109</v>
+        <v>44.58620338637983</v>
       </c>
       <c r="L12" t="n">
-        <v>15.60662099072334</v>
+        <v>27.82719186785261</v>
       </c>
       <c r="M12" t="inlineStr">
         <is>
@@ -2346,7 +2346,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>RITA DE CASSIA TRINCA PASSOS</t>
+          <t>ROGERIO NOGUEIRA LOPES CRUZ</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -2356,26 +2356,26 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Religião e Valores - Religiosidade, valores morais, costumes, família</t>
+          <t>Mobilidade e Acessibilidade - Transporte, calçadas, acesso a serviços, mobilidade</t>
         </is>
       </c>
       <c r="G13" t="n">
         <v>4</v>
       </c>
       <c r="H13" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="I13" t="n">
-        <v>3923</v>
+        <v>105</v>
       </c>
       <c r="J13" t="n">
-        <v>18849</v>
+        <v>3348</v>
       </c>
       <c r="K13" t="n">
-        <v>208.1277521353918</v>
+        <v>31.36200716845878</v>
       </c>
       <c r="L13" t="n">
-        <v>23.78584854180562</v>
+        <v>2.223634053367217</v>
       </c>
       <c r="M13" t="inlineStr">
         <is>
@@ -2401,7 +2401,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>RITA DE CASSIA TRINCA PASSOS</t>
+          <t>ROGERIO NOGUEIRA LOPES CRUZ</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -2411,24 +2411,26 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Saúde - Doenças crônicas, cuidado do idoso, acesso</t>
+          <t>Proteção Animal - Proteção animal, bem-estar, resgate, políticas pets</t>
         </is>
       </c>
       <c r="G14" t="n">
         <v>1</v>
       </c>
       <c r="H14" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="I14" t="n">
-        <v>0</v>
+        <v>1130</v>
       </c>
       <c r="J14" t="n">
-        <v>0</v>
-      </c>
-      <c r="K14" t="inlineStr"/>
+        <v>20098</v>
+      </c>
+      <c r="K14" t="n">
+        <v>56.2244999502438</v>
+      </c>
       <c r="L14" t="n">
-        <v>0</v>
+        <v>23.93053790766625</v>
       </c>
       <c r="M14" t="inlineStr">
         <is>
@@ -2454,7 +2456,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>RITA DE CASSIA TRINCA PASSOS</t>
+          <t>ROGERIO NOGUEIRA LOPES CRUZ</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -2464,26 +2466,26 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Saúde - Doenças crônicas, cuidado do idoso, acesso</t>
+          <t>Proteção Animal - Proteção animal, bem-estar, resgate, políticas pets</t>
         </is>
       </c>
       <c r="G15" t="n">
         <v>2</v>
       </c>
       <c r="H15" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="I15" t="n">
-        <v>5633</v>
+        <v>904</v>
       </c>
       <c r="J15" t="n">
-        <v>35281</v>
+        <v>18629</v>
       </c>
       <c r="K15" t="n">
-        <v>159.6610073410617</v>
+        <v>48.52649095496269</v>
       </c>
       <c r="L15" t="n">
-        <v>34.15388346571272</v>
+        <v>19.14443032613299</v>
       </c>
       <c r="M15" t="inlineStr">
         <is>
@@ -2509,7 +2511,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>RITA DE CASSIA TRINCA PASSOS</t>
+          <t>ROGERIO NOGUEIRA LOPES CRUZ</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -2519,26 +2521,26 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Saúde - Doenças crônicas, cuidado do idoso, acesso</t>
+          <t>Proteção Animal - Proteção animal, bem-estar, resgate, políticas pets</t>
         </is>
       </c>
       <c r="G16" t="n">
         <v>3</v>
       </c>
       <c r="H16" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="I16" t="n">
-        <v>4046</v>
+        <v>1531</v>
       </c>
       <c r="J16" t="n">
-        <v>23400</v>
+        <v>34091</v>
       </c>
       <c r="K16" t="n">
-        <v>172.9059829059829</v>
+        <v>44.90921357543046</v>
       </c>
       <c r="L16" t="n">
-        <v>24.53161947492876</v>
+        <v>32.42270224481152</v>
       </c>
       <c r="M16" t="inlineStr">
         <is>
@@ -2564,7 +2566,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>RITA DE CASSIA TRINCA PASSOS</t>
+          <t>ROGERIO NOGUEIRA LOPES CRUZ</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -2574,26 +2576,26 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Saúde - Doenças crônicas, cuidado do idoso, acesso</t>
+          <t>Proteção Animal - Proteção animal, bem-estar, resgate, políticas pets</t>
         </is>
       </c>
       <c r="G17" t="n">
         <v>4</v>
       </c>
       <c r="H17" t="n">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="I17" t="n">
-        <v>6814</v>
+        <v>1157</v>
       </c>
       <c r="J17" t="n">
-        <v>37717</v>
+        <v>21015</v>
       </c>
       <c r="K17" t="n">
-        <v>180.6612402895246</v>
+        <v>55.05591244349274</v>
       </c>
       <c r="L17" t="n">
-        <v>41.31449705935852</v>
+        <v>24.50232952138924</v>
       </c>
       <c r="M17" t="inlineStr">
         <is>
@@ -2619,7 +2621,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>RITA DE CASSIA TRINCA PASSOS</t>
+          <t>ROGERIO NOGUEIRA LOPES CRUZ</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -2639,16 +2641,16 @@
         <v>14</v>
       </c>
       <c r="I18" t="n">
-        <v>6374</v>
+        <v>2445</v>
       </c>
       <c r="J18" t="n">
-        <v>44118</v>
+        <v>43069</v>
       </c>
       <c r="K18" t="n">
-        <v>144.4761775239132</v>
+        <v>56.76937008056839</v>
       </c>
       <c r="L18" t="n">
-        <v>38.64669859940581</v>
+        <v>51.77890724269377</v>
       </c>
       <c r="M18" t="inlineStr">
         <is>
@@ -2674,7 +2676,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>RITA DE CASSIA TRINCA PASSOS</t>
+          <t>ROGERIO NOGUEIRA LOPES CRUZ</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -2694,16 +2696,16 @@
         <v>8</v>
       </c>
       <c r="I19" t="n">
-        <v>3266</v>
+        <v>966</v>
       </c>
       <c r="J19" t="n">
-        <v>19250</v>
+        <v>18608</v>
       </c>
       <c r="K19" t="n">
-        <v>169.6623376623376</v>
+        <v>51.91315563198624</v>
       </c>
       <c r="L19" t="n">
-        <v>19.80234038683078</v>
+        <v>20.4574332909784</v>
       </c>
       <c r="M19" t="inlineStr">
         <is>
@@ -2729,7 +2731,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>RITA DE CASSIA TRINCA PASSOS</t>
+          <t>ROGERIO NOGUEIRA LOPES CRUZ</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -2749,16 +2751,16 @@
         <v>4</v>
       </c>
       <c r="I20" t="n">
-        <v>2308</v>
+        <v>469</v>
       </c>
       <c r="J20" t="n">
-        <v>11017</v>
+        <v>10700</v>
       </c>
       <c r="K20" t="n">
-        <v>209.4944177180721</v>
+        <v>43.83177570093458</v>
       </c>
       <c r="L20" t="n">
-        <v>13.99381555811556</v>
+        <v>9.932232105040237</v>
       </c>
       <c r="M20" t="inlineStr">
         <is>
@@ -2784,7 +2786,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>RITA DE CASSIA TRINCA PASSOS</t>
+          <t>ROGERIO NOGUEIRA LOPES CRUZ</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -2804,16 +2806,16 @@
         <v>10</v>
       </c>
       <c r="I21" t="n">
-        <v>4545</v>
+        <v>842</v>
       </c>
       <c r="J21" t="n">
-        <v>22013</v>
+        <v>21456</v>
       </c>
       <c r="K21" t="n">
-        <v>206.4689047381093</v>
+        <v>39.24310216256525</v>
       </c>
       <c r="L21" t="n">
-        <v>27.55714545564785</v>
+        <v>17.83142736128759</v>
       </c>
       <c r="M21" t="inlineStr">
         <is>
@@ -2839,7 +2841,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>RITA DE CASSIA TRINCA PASSOS</t>
+          <t>ROGERIO NOGUEIRA LOPES CRUZ</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -2859,16 +2861,16 @@
         <v>10</v>
       </c>
       <c r="I22" t="n">
-        <v>314</v>
+        <v>5411</v>
       </c>
       <c r="J22" t="n">
-        <v>24918</v>
+        <v>24471</v>
       </c>
       <c r="K22" t="n">
-        <v>12.60133237017417</v>
+        <v>221.1188754035389</v>
       </c>
       <c r="L22" t="n">
-        <v>28.99353647276085</v>
+        <v>30.74955958402</v>
       </c>
       <c r="M22" t="inlineStr">
         <is>
@@ -2894,7 +2896,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>RITA DE CASSIA TRINCA PASSOS</t>
+          <t>ROGERIO NOGUEIRA LOPES CRUZ</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -2914,16 +2916,16 @@
         <v>8</v>
       </c>
       <c r="I23" t="n">
-        <v>251</v>
+        <v>4640</v>
       </c>
       <c r="J23" t="n">
-        <v>18295</v>
+        <v>17952</v>
       </c>
       <c r="K23" t="n">
-        <v>13.71959551790107</v>
+        <v>258.4670231729056</v>
       </c>
       <c r="L23" t="n">
-        <v>23.17636195752539</v>
+        <v>26.36813093140876</v>
       </c>
       <c r="M23" t="inlineStr">
         <is>
@@ -2949,7 +2951,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>RITA DE CASSIA TRINCA PASSOS</t>
+          <t>ROGERIO NOGUEIRA LOPES CRUZ</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -2969,16 +2971,16 @@
         <v>5</v>
       </c>
       <c r="I24" t="n">
-        <v>221</v>
+        <v>3492</v>
       </c>
       <c r="J24" t="n">
-        <v>14214</v>
+        <v>13858</v>
       </c>
       <c r="K24" t="n">
-        <v>15.54805121710989</v>
+        <v>251.9844133352576</v>
       </c>
       <c r="L24" t="n">
-        <v>20.40627885503232</v>
+        <v>19.84429164062056</v>
       </c>
       <c r="M24" t="inlineStr">
         <is>
@@ -3004,7 +3006,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>RITA DE CASSIA TRINCA PASSOS</t>
+          <t>ROGERIO NOGUEIRA LOPES CRUZ</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -3024,16 +3026,16 @@
         <v>9</v>
       </c>
       <c r="I25" t="n">
-        <v>297</v>
+        <v>4054</v>
       </c>
       <c r="J25" t="n">
-        <v>17333</v>
+        <v>16894</v>
       </c>
       <c r="K25" t="n">
-        <v>17.13494490278659</v>
+        <v>239.9668521368533</v>
       </c>
       <c r="L25" t="n">
-        <v>27.42382271468144</v>
+        <v>23.03801784395067</v>
       </c>
       <c r="M25" t="inlineStr">
         <is>
@@ -3059,7 +3061,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>RITA DE CASSIA TRINCA PASSOS</t>
+          <t>ROGERIO NOGUEIRA LOPES CRUZ</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -3079,16 +3081,16 @@
         <v>5</v>
       </c>
       <c r="I26" t="n">
-        <v>202</v>
+        <v>3212</v>
       </c>
       <c r="J26" t="n">
-        <v>14966</v>
+        <v>14760</v>
       </c>
       <c r="K26" t="n">
-        <v>13.49726045703595</v>
+        <v>217.6151761517615</v>
       </c>
       <c r="L26" t="n">
-        <v>18.65189289012004</v>
+        <v>18.25311132579417</v>
       </c>
       <c r="M26" t="inlineStr">
         <is>
@@ -3114,7 +3116,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>RITA DE CASSIA TRINCA PASSOS</t>
+          <t>ROGERIO NOGUEIRA LOPES CRUZ</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -3134,16 +3136,16 @@
         <v>12</v>
       </c>
       <c r="I27" t="n">
-        <v>447</v>
+        <v>7153</v>
       </c>
       <c r="J27" t="n">
-        <v>30113</v>
+        <v>29390</v>
       </c>
       <c r="K27" t="n">
-        <v>14.84408727127819</v>
+        <v>243.3821027560395</v>
       </c>
       <c r="L27" t="n">
-        <v>41.27423822714682</v>
+        <v>40.64897425697562</v>
       </c>
       <c r="M27" t="inlineStr">
         <is>
@@ -3169,7 +3171,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>RITA DE CASSIA TRINCA PASSOS</t>
+          <t>ROGERIO NOGUEIRA LOPES CRUZ</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -3189,16 +3191,16 @@
         <v>10</v>
       </c>
       <c r="I28" t="n">
-        <v>336</v>
+        <v>5536</v>
       </c>
       <c r="J28" t="n">
-        <v>22414</v>
+        <v>21946</v>
       </c>
       <c r="K28" t="n">
-        <v>14.99063085571518</v>
+        <v>252.255536316413</v>
       </c>
       <c r="L28" t="n">
-        <v>31.02493074792244</v>
+        <v>31.45990793885322</v>
       </c>
       <c r="M28" t="inlineStr">
         <is>
@@ -3224,7 +3226,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>RITA DE CASSIA TRINCA PASSOS</t>
+          <t>ROGERIO NOGUEIRA LOPES CRUZ</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -3244,16 +3246,16 @@
         <v>5</v>
       </c>
       <c r="I29" t="n">
-        <v>98</v>
+        <v>1696</v>
       </c>
       <c r="J29" t="n">
-        <v>7267</v>
+        <v>7079</v>
       </c>
       <c r="K29" t="n">
-        <v>13.48561992569148</v>
+        <v>239.5818618448934</v>
       </c>
       <c r="L29" t="n">
-        <v>9.04893813481071</v>
+        <v>9.638006478376997</v>
       </c>
       <c r="M29" t="inlineStr">
         <is>
@@ -3279,7 +3281,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>RITA DE CASSIA TRINCA PASSOS</t>
+          <t>ROGERIO NOGUEIRA LOPES CRUZ</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -3289,26 +3291,26 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Religião e Valores - Religiosidade, valores morais, costumes, família</t>
+          <t>Mobilidade e Acessibilidade - Transporte, calçadas, acesso a serviços, mobilidade</t>
         </is>
       </c>
       <c r="G30" t="n">
         <v>1</v>
       </c>
       <c r="H30" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="I30" t="n">
-        <v>301</v>
+        <v>4983</v>
       </c>
       <c r="J30" t="n">
-        <v>20374</v>
+        <v>22743</v>
       </c>
       <c r="K30" t="n">
-        <v>14.77373122607245</v>
+        <v>219.1003825352856</v>
       </c>
       <c r="L30" t="n">
-        <v>27.79316712834719</v>
+        <v>28.31732681707109</v>
       </c>
       <c r="M30" t="inlineStr">
         <is>
@@ -3334,7 +3336,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>RITA DE CASSIA TRINCA PASSOS</t>
+          <t>ROGERIO NOGUEIRA LOPES CRUZ</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -3344,26 +3346,26 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Religião e Valores - Religiosidade, valores morais, costumes, família</t>
+          <t>Mobilidade e Acessibilidade - Transporte, calçadas, acesso a serviços, mobilidade</t>
         </is>
       </c>
       <c r="G31" t="n">
         <v>2</v>
       </c>
       <c r="H31" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I31" t="n">
-        <v>210</v>
+        <v>4834</v>
       </c>
       <c r="J31" t="n">
-        <v>16286</v>
+        <v>19745</v>
       </c>
       <c r="K31" t="n">
-        <v>12.89451062262066</v>
+        <v>244.8214737908331</v>
       </c>
       <c r="L31" t="n">
-        <v>19.39058171745152</v>
+        <v>27.4705915781099</v>
       </c>
       <c r="M31" t="inlineStr">
         <is>
@@ -3389,7 +3391,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>RITA DE CASSIA TRINCA PASSOS</t>
+          <t>ROGERIO NOGUEIRA LOPES CRUZ</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -3399,26 +3401,26 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Religião e Valores - Religiosidade, valores morais, costumes, família</t>
+          <t>Mobilidade e Acessibilidade - Transporte, calçadas, acesso a serviços, mobilidade</t>
         </is>
       </c>
       <c r="G32" t="n">
         <v>3</v>
       </c>
       <c r="H32" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="I32" t="n">
-        <v>317</v>
+        <v>6623</v>
       </c>
       <c r="J32" t="n">
-        <v>21370</v>
+        <v>25785</v>
       </c>
       <c r="K32" t="n">
-        <v>14.83387927000468</v>
+        <v>256.854760519682</v>
       </c>
       <c r="L32" t="n">
-        <v>29.27054478301016</v>
+        <v>37.63709723248281</v>
       </c>
       <c r="M32" t="inlineStr">
         <is>
@@ -3444,7 +3446,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>RITA DE CASSIA TRINCA PASSOS</t>
+          <t>ROGERIO NOGUEIRA LOPES CRUZ</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -3454,26 +3456,26 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Religião e Valores - Religiosidade, valores morais, costumes, família</t>
+          <t>Mobilidade e Acessibilidade - Transporte, calçadas, acesso a serviços, mobilidade</t>
         </is>
       </c>
       <c r="G33" t="n">
         <v>4</v>
       </c>
       <c r="H33" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="I33" t="n">
-        <v>255</v>
+        <v>1157</v>
       </c>
       <c r="J33" t="n">
-        <v>16730</v>
+        <v>4902</v>
       </c>
       <c r="K33" t="n">
-        <v>15.24208009563658</v>
+        <v>236.0261117911057</v>
       </c>
       <c r="L33" t="n">
-        <v>23.54570637119114</v>
+        <v>6.574984372336194</v>
       </c>
       <c r="M33" t="inlineStr">
         <is>
@@ -3499,7 +3501,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>RITA DE CASSIA TRINCA PASSOS</t>
+          <t>ROGERIO NOGUEIRA LOPES CRUZ</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -3509,26 +3511,26 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Saúde - Doenças crônicas, cuidado do idoso, acesso</t>
+          <t>Proteção Animal - Proteção animal, bem-estar, resgate, políticas pets</t>
         </is>
       </c>
       <c r="G34" t="n">
         <v>1</v>
       </c>
       <c r="H34" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="I34" t="n">
-        <v>127</v>
+        <v>5330</v>
       </c>
       <c r="J34" t="n">
-        <v>7202</v>
+        <v>21963</v>
       </c>
       <c r="K34" t="n">
-        <v>17.63399055817828</v>
+        <v>242.6808723762692</v>
       </c>
       <c r="L34" t="n">
-        <v>11.72668513388735</v>
+        <v>30.28925385008808</v>
       </c>
       <c r="M34" t="inlineStr">
         <is>
@@ -3554,7 +3556,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>RITA DE CASSIA TRINCA PASSOS</t>
+          <t>ROGERIO NOGUEIRA LOPES CRUZ</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -3564,26 +3566,26 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Saúde - Doenças crônicas, cuidado do idoso, acesso</t>
+          <t>Proteção Animal - Proteção animal, bem-estar, resgate, políticas pets</t>
         </is>
       </c>
       <c r="G35" t="n">
         <v>2</v>
       </c>
       <c r="H35" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="I35" t="n">
-        <v>243</v>
+        <v>5165</v>
       </c>
       <c r="J35" t="n">
-        <v>20059</v>
+        <v>22551</v>
       </c>
       <c r="K35" t="n">
-        <v>12.1142629243731</v>
+        <v>229.0364063677886</v>
       </c>
       <c r="L35" t="n">
-        <v>22.4376731301939</v>
+        <v>29.35159402170824</v>
       </c>
       <c r="M35" t="inlineStr">
         <is>
@@ -3609,7 +3611,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>RITA DE CASSIA TRINCA PASSOS</t>
+          <t>ROGERIO NOGUEIRA LOPES CRUZ</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -3619,26 +3621,26 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Saúde - Doenças crônicas, cuidado do idoso, acesso</t>
+          <t>Proteção Animal - Proteção animal, bem-estar, resgate, políticas pets</t>
         </is>
       </c>
       <c r="G36" t="n">
         <v>3</v>
       </c>
       <c r="H36" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="I36" t="n">
-        <v>362</v>
+        <v>3371</v>
       </c>
       <c r="J36" t="n">
-        <v>24063</v>
+        <v>13580</v>
       </c>
       <c r="K36" t="n">
-        <v>15.04384324481569</v>
+        <v>248.2326951399116</v>
       </c>
       <c r="L36" t="n">
-        <v>33.42566943674976</v>
+        <v>19.15667443314201</v>
       </c>
       <c r="M36" t="inlineStr">
         <is>
@@ -3664,7 +3666,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>RITA DE CASSIA TRINCA PASSOS</t>
+          <t>ROGERIO NOGUEIRA LOPES CRUZ</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -3674,26 +3676,26 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Saúde - Doenças crônicas, cuidado do idoso, acesso</t>
+          <t>Proteção Animal - Proteção animal, bem-estar, resgate, políticas pets</t>
         </is>
       </c>
       <c r="G37" t="n">
         <v>4</v>
       </c>
       <c r="H37" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="I37" t="n">
-        <v>351</v>
+        <v>3731</v>
       </c>
       <c r="J37" t="n">
-        <v>23436</v>
+        <v>15081</v>
       </c>
       <c r="K37" t="n">
-        <v>14.97695852534562</v>
+        <v>247.3973874411511</v>
       </c>
       <c r="L37" t="n">
-        <v>32.40997229916898</v>
+        <v>21.20247769506166</v>
       </c>
       <c r="M37" t="inlineStr">
         <is>
@@ -3719,7 +3721,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>RITA DE CASSIA TRINCA PASSOS</t>
+          <t>ROGERIO NOGUEIRA LOPES CRUZ</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -3739,16 +3741,16 @@
         <v>10</v>
       </c>
       <c r="I38" t="n">
-        <v>314</v>
+        <v>5411</v>
       </c>
       <c r="J38" t="n">
-        <v>24918</v>
+        <v>24471</v>
       </c>
       <c r="K38" t="n">
-        <v>12.60133237017417</v>
+        <v>221.1188754035389</v>
       </c>
       <c r="L38" t="n">
-        <v>28.99353647276085</v>
+        <v>30.74955958402</v>
       </c>
       <c r="M38" t="inlineStr">
         <is>
@@ -3774,7 +3776,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>RITA DE CASSIA TRINCA PASSOS</t>
+          <t>ROGERIO NOGUEIRA LOPES CRUZ</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -3794,16 +3796,16 @@
         <v>8</v>
       </c>
       <c r="I39" t="n">
-        <v>251</v>
+        <v>4640</v>
       </c>
       <c r="J39" t="n">
-        <v>18295</v>
+        <v>17952</v>
       </c>
       <c r="K39" t="n">
-        <v>13.71959551790107</v>
+        <v>258.4670231729056</v>
       </c>
       <c r="L39" t="n">
-        <v>23.17636195752539</v>
+        <v>26.36813093140876</v>
       </c>
       <c r="M39" t="inlineStr">
         <is>
@@ -3829,7 +3831,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>RITA DE CASSIA TRINCA PASSOS</t>
+          <t>ROGERIO NOGUEIRA LOPES CRUZ</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -3849,16 +3851,16 @@
         <v>5</v>
       </c>
       <c r="I40" t="n">
-        <v>221</v>
+        <v>3492</v>
       </c>
       <c r="J40" t="n">
-        <v>14214</v>
+        <v>13858</v>
       </c>
       <c r="K40" t="n">
-        <v>15.54805121710989</v>
+        <v>251.9844133352576</v>
       </c>
       <c r="L40" t="n">
-        <v>20.40627885503232</v>
+        <v>19.84429164062056</v>
       </c>
       <c r="M40" t="inlineStr">
         <is>
@@ -3884,7 +3886,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>RITA DE CASSIA TRINCA PASSOS</t>
+          <t>ROGERIO NOGUEIRA LOPES CRUZ</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -3904,16 +3906,16 @@
         <v>9</v>
       </c>
       <c r="I41" t="n">
-        <v>297</v>
+        <v>4054</v>
       </c>
       <c r="J41" t="n">
-        <v>17333</v>
+        <v>16894</v>
       </c>
       <c r="K41" t="n">
-        <v>17.13494490278659</v>
+        <v>239.9668521368533</v>
       </c>
       <c r="L41" t="n">
-        <v>27.42382271468144</v>
+        <v>23.03801784395067</v>
       </c>
       <c r="M41" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Publica mapas XG-AE mapa_aderencia 2026-07-02 16:39:37
</commit_message>
<xml_diff>
--- a/mapas2/mapa_aderencia_xg_aderencia_eleitoral.xlsx
+++ b/mapas2/mapa_aderencia_xg_aderencia_eleitoral.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z11"/>
+  <dimension ref="A1:Z15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -600,37 +600,37 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Proteção Animal - Proteção animal, bem-estar, resgate, políticas pets</t>
+          <t>Bem-Estar e Serviços - Qualidade do bairro, serviços, segurança, lazer</t>
         </is>
       </c>
       <c r="I2" t="n">
         <v>1</v>
       </c>
       <c r="J2" t="n">
-        <v>43.76961846968661</v>
+        <v>62.46992594531096</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Relação inversa moderada</t>
+          <t>Aderência positiva moderada</t>
         </is>
       </c>
       <c r="L2" t="n">
-        <v>-0.2266143280393914</v>
+        <v>0.3512522084610567</v>
       </c>
       <c r="M2" t="n">
-        <v>38.66928359803043</v>
+        <v>67.56261042305283</v>
       </c>
       <c r="N2" t="n">
-        <v>1.09404096406401</v>
+        <v>1.087099002984713</v>
       </c>
       <c r="O2" t="n">
-        <v>53.24166894561949</v>
+        <v>53.01208334379036</v>
       </c>
       <c r="P2" t="n">
         <v>50.32344697494485</v>
       </c>
       <c r="Q2" t="n">
-        <v>55.05591244349274</v>
+        <v>54.7065690332166</v>
       </c>
       <c r="R2" t="inlineStr">
         <is>
@@ -661,12 +661,12 @@
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>C:\Users\guilh\Trabalho\Relatórios Alisson\Documentos gerais\Git\2\dataquadri\mapas2\mapa_aderencia_rogerio_itu_sp_2022_protecao_animal_protecao_animal_bem_estar_resgate_politicas_pets_cidade_inteira.html</t>
+          <t>C:\Users\guilh\Trabalho\Relatórios Alisson\Documentos gerais\Git\2\dataquadri\mapas2\mapa_aderencia_rogerio_itu_sp_2022_bem_estar_e_servicos_qualidade_do_bairro_servicos_seguranca_lazer_cidade_inteira.html</t>
         </is>
       </c>
       <c r="Z2" t="inlineStr">
         <is>
-          <t>https://quadrifygit.github.io/dataquadri/mapas2/mapa_aderencia_rogerio_itu_sp_2022_protecao_animal_protecao_animal_bem_estar_resgate_politicas_pets_cidade_inteira.html</t>
+          <t>https://quadrifygit.github.io/dataquadri/mapas2/mapa_aderencia_rogerio_itu_sp_2022_bem_estar_e_servicos_qualidade_do_bairro_servicos_seguranca_lazer_cidade_inteira.html</t>
         </is>
       </c>
     </row>
@@ -708,14 +708,14 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Comportamento Político - Qualidade de gestão, eficiência, entrega de serviços</t>
+          <t>Proteção Animal - Proteção animal, bem-estar, resgate, políticas pets</t>
         </is>
       </c>
       <c r="I3" t="n">
         <v>2</v>
       </c>
       <c r="J3" t="n">
-        <v>42.73191145739839</v>
+        <v>43.76961846968661</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
@@ -723,22 +723,22 @@
         </is>
       </c>
       <c r="L3" t="n">
-        <v>-0.2353698816227315</v>
+        <v>-0.2266143280393914</v>
       </c>
       <c r="M3" t="n">
-        <v>38.23150591886343</v>
+        <v>38.66928359803043</v>
       </c>
       <c r="N3" t="n">
-        <v>1.030677011112459</v>
+        <v>1.09404096406401</v>
       </c>
       <c r="O3" t="n">
-        <v>51.08980745753475</v>
+        <v>53.24166894561949</v>
       </c>
       <c r="P3" t="n">
         <v>50.32344697494485</v>
       </c>
       <c r="Q3" t="n">
-        <v>51.86721991701245</v>
+        <v>55.05591244349274</v>
       </c>
       <c r="R3" t="inlineStr">
         <is>
@@ -769,12 +769,12 @@
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>C:\Users\guilh\Trabalho\Relatórios Alisson\Documentos gerais\Git\2\dataquadri\mapas2\mapa_aderencia_rogerio_itu_sp_2022_comportamento_politico_qualidade_de_gestao_eficiencia_entrega_de_servicos_cidade_inteira.html</t>
+          <t>C:\Users\guilh\Trabalho\Relatórios Alisson\Documentos gerais\Git\2\dataquadri\mapas2\mapa_aderencia_rogerio_itu_sp_2022_protecao_animal_protecao_animal_bem_estar_resgate_politicas_pets_cidade_inteira.html</t>
         </is>
       </c>
       <c r="Z3" t="inlineStr">
         <is>
-          <t>https://quadrifygit.github.io/dataquadri/mapas2/mapa_aderencia_rogerio_itu_sp_2022_comportamento_politico_qualidade_de_gestao_eficiencia_entrega_de_servicos_cidade_inteira.html</t>
+          <t>https://quadrifygit.github.io/dataquadri/mapas2/mapa_aderencia_rogerio_itu_sp_2022_protecao_animal_protecao_animal_bem_estar_resgate_politicas_pets_cidade_inteira.html</t>
         </is>
       </c>
     </row>
@@ -816,14 +816,14 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Mobilidade e Acessibilidade - Transporte, calçadas, acesso a serviços, mobilidade</t>
+          <t>Comportamento Político - Qualidade de gestão, eficiência, entrega de serviços</t>
         </is>
       </c>
       <c r="I4" t="n">
         <v>3</v>
       </c>
       <c r="J4" t="n">
-        <v>34.71562985569617</v>
+        <v>42.73191145739839</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
@@ -831,22 +831,22 @@
         </is>
       </c>
       <c r="L4" t="n">
-        <v>-0.2866156217134576</v>
+        <v>-0.2353698816227315</v>
       </c>
       <c r="M4" t="n">
-        <v>35.66921891432712</v>
+        <v>38.23150591886343</v>
       </c>
       <c r="N4" t="n">
-        <v>0.6232086443536621</v>
+        <v>1.030677011112459</v>
       </c>
       <c r="O4" t="n">
-        <v>32.94467874681013</v>
+        <v>51.08980745753475</v>
       </c>
       <c r="P4" t="n">
         <v>50.32344697494485</v>
       </c>
       <c r="Q4" t="n">
-        <v>31.36200716845878</v>
+        <v>51.86721991701245</v>
       </c>
       <c r="R4" t="inlineStr">
         <is>
@@ -877,12 +877,12 @@
       </c>
       <c r="Y4" t="inlineStr">
         <is>
-          <t>C:\Users\guilh\Trabalho\Relatórios Alisson\Documentos gerais\Git\2\dataquadri\mapas2\mapa_aderencia_rogerio_itu_sp_2022_mobilidade_e_acessibilidade_transporte_calcadas_acesso_a_servicos_mobilidade_cidade_inteira.html</t>
+          <t>C:\Users\guilh\Trabalho\Relatórios Alisson\Documentos gerais\Git\2\dataquadri\mapas2\mapa_aderencia_rogerio_itu_sp_2022_comportamento_politico_qualidade_de_gestao_eficiencia_entrega_de_servicos_cidade_inteira.html</t>
         </is>
       </c>
       <c r="Z4" t="inlineStr">
         <is>
-          <t>https://quadrifygit.github.io/dataquadri/mapas2/mapa_aderencia_rogerio_itu_sp_2022_mobilidade_e_acessibilidade_transporte_calcadas_acesso_a_servicos_mobilidade_cidade_inteira.html</t>
+          <t>https://quadrifygit.github.io/dataquadri/mapas2/mapa_aderencia_rogerio_itu_sp_2022_comportamento_politico_qualidade_de_gestao_eficiencia_entrega_de_servicos_cidade_inteira.html</t>
         </is>
       </c>
     </row>
@@ -924,37 +924,37 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Saúde - UBS, consultas, exames básicos, acesso SUS</t>
+          <t>Bem-Estar e Serviços - Busca por qualidade de vida, serviços, lazer</t>
         </is>
       </c>
       <c r="I5" t="n">
         <v>4</v>
       </c>
       <c r="J5" t="n">
-        <v>28.76619148168748</v>
+        <v>36.72918203727596</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Forte relação inversa</t>
+          <t>Relação inversa moderada</t>
         </is>
       </c>
       <c r="L5" t="n">
-        <v>-0.5567502013876867</v>
+        <v>-0.3321960036031988</v>
       </c>
       <c r="M5" t="n">
-        <v>22.16248993061566</v>
+        <v>33.39019981984006</v>
       </c>
       <c r="N5" t="n">
-        <v>0.7798174513384127</v>
+        <v>0.821997528058819</v>
       </c>
       <c r="O5" t="n">
-        <v>41.03020864796372</v>
+        <v>42.93014901251406</v>
       </c>
       <c r="P5" t="n">
         <v>50.32344697494485</v>
       </c>
       <c r="Q5" t="n">
-        <v>39.24310216256525</v>
+        <v>41.36574901680372</v>
       </c>
       <c r="R5" t="inlineStr">
         <is>
@@ -985,12 +985,12 @@
       </c>
       <c r="Y5" t="inlineStr">
         <is>
-          <t>C:\Users\guilh\Trabalho\Relatórios Alisson\Documentos gerais\Git\2\dataquadri\mapas2\mapa_aderencia_rogerio_itu_sp_2022_saude_ubs_consultas_exames_basicos_acesso_sus_cidade_inteira.html</t>
+          <t>C:\Users\guilh\Trabalho\Relatórios Alisson\Documentos gerais\Git\2\dataquadri\mapas2\mapa_aderencia_rogerio_itu_sp_2022_bem_estar_e_servicos_busca_por_qualidade_de_vida_servicos_lazer_cidade_inteira.html</t>
         </is>
       </c>
       <c r="Z5" t="inlineStr">
         <is>
-          <t>https://quadrifygit.github.io/dataquadri/mapas2/mapa_aderencia_rogerio_itu_sp_2022_saude_ubs_consultas_exames_basicos_acesso_sus_cidade_inteira.html</t>
+          <t>https://quadrifygit.github.io/dataquadri/mapas2/mapa_aderencia_rogerio_itu_sp_2022_bem_estar_e_servicos_busca_por_qualidade_de_vida_servicos_lazer_cidade_inteira.html</t>
         </is>
       </c>
     </row>
@@ -1032,37 +1032,37 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Assistência Social - Proteção social, seguridade, assistência, rede pública</t>
+          <t>Mobilidade e Acessibilidade - Transporte, calçadas, acesso a serviços, mobilidade</t>
         </is>
       </c>
       <c r="I6" t="n">
         <v>5</v>
       </c>
       <c r="J6" t="n">
-        <v>28.69923724840312</v>
+        <v>34.71562985569617</v>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Forte relação inversa</t>
+          <t>Relação inversa moderada</t>
         </is>
       </c>
       <c r="L6" t="n">
-        <v>-0.5588103316425902</v>
+        <v>-0.2866156217134576</v>
       </c>
       <c r="M6" t="n">
-        <v>22.05948341787049</v>
+        <v>35.66921891432712</v>
       </c>
       <c r="N6" t="n">
-        <v>0.7798174513384127</v>
+        <v>0.6232086443536621</v>
       </c>
       <c r="O6" t="n">
-        <v>41.03020864796372</v>
+        <v>32.94467874681013</v>
       </c>
       <c r="P6" t="n">
         <v>50.32344697494485</v>
       </c>
       <c r="Q6" t="n">
-        <v>39.24310216256525</v>
+        <v>31.36200716845878</v>
       </c>
       <c r="R6" t="inlineStr">
         <is>
@@ -1093,12 +1093,12 @@
       </c>
       <c r="Y6" t="inlineStr">
         <is>
-          <t>C:\Users\guilh\Trabalho\Relatórios Alisson\Documentos gerais\Git\2\dataquadri\mapas2\mapa_aderencia_rogerio_itu_sp_2022_assistencia_social_protecao_social_seguridade_assistencia_rede_publica_cidade_inteira.html</t>
+          <t>C:\Users\guilh\Trabalho\Relatórios Alisson\Documentos gerais\Git\2\dataquadri\mapas2\mapa_aderencia_rogerio_itu_sp_2022_mobilidade_e_acessibilidade_transporte_calcadas_acesso_a_servicos_mobilidade_cidade_inteira.html</t>
         </is>
       </c>
       <c r="Z6" t="inlineStr">
         <is>
-          <t>https://quadrifygit.github.io/dataquadri/mapas2/mapa_aderencia_rogerio_itu_sp_2022_assistencia_social_protecao_social_seguridade_assistencia_rede_publica_cidade_inteira.html</t>
+          <t>https://quadrifygit.github.io/dataquadri/mapas2/mapa_aderencia_rogerio_itu_sp_2022_mobilidade_e_acessibilidade_transporte_calcadas_acesso_a_servicos_mobilidade_cidade_inteira.html</t>
         </is>
       </c>
     </row>
@@ -1110,7 +1110,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>salto</t>
+          <t>itu</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1140,37 +1140,37 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Mobilidade e Acessibilidade - Transporte, calçadas, acesso a serviços, mobilidade</t>
+          <t>Saúde - UBS, consultas, exames básicos, acesso SUS</t>
         </is>
       </c>
       <c r="I7" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="J7" t="n">
-        <v>63.30874465234245</v>
+        <v>28.76619148168748</v>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Aderência positiva moderada</t>
+          <t>Forte relação inversa</t>
         </is>
       </c>
       <c r="L7" t="n">
-        <v>0.4167583705219454</v>
+        <v>-0.5567502013876867</v>
       </c>
       <c r="M7" t="n">
-        <v>70.83791852609727</v>
+        <v>22.16248993061566</v>
       </c>
       <c r="N7" t="n">
-        <v>0.9814860902605079</v>
+        <v>0.7798174513384127</v>
       </c>
       <c r="O7" t="n">
-        <v>49.32599317251208</v>
+        <v>41.03020864796372</v>
       </c>
       <c r="P7" t="n">
-        <v>240.4783054321831</v>
+        <v>50.32344697494485</v>
       </c>
       <c r="Q7" t="n">
-        <v>236.0261117911057</v>
+        <v>39.24310216256525</v>
       </c>
       <c r="R7" t="inlineStr">
         <is>
@@ -1178,10 +1178,10 @@
         </is>
       </c>
       <c r="S7" t="n">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="T7" t="n">
-        <v>17597</v>
+        <v>4722</v>
       </c>
       <c r="U7" t="n">
         <v>0</v>
@@ -1201,12 +1201,12 @@
       </c>
       <c r="Y7" t="inlineStr">
         <is>
-          <t>C:\Users\guilh\Trabalho\Relatórios Alisson\Documentos gerais\Git\2\dataquadri\mapas2\mapa_aderencia_rogerio_salto_sp_2022_mobilidade_e_acessibilidade_transporte_calcadas_acesso_a_servicos_mobilidade_cidade_inteira.html</t>
+          <t>C:\Users\guilh\Trabalho\Relatórios Alisson\Documentos gerais\Git\2\dataquadri\mapas2\mapa_aderencia_rogerio_itu_sp_2022_saude_ubs_consultas_exames_basicos_acesso_sus_cidade_inteira.html</t>
         </is>
       </c>
       <c r="Z7" t="inlineStr">
         <is>
-          <t>https://quadrifygit.github.io/dataquadri/mapas2/mapa_aderencia_rogerio_salto_sp_2022_mobilidade_e_acessibilidade_transporte_calcadas_acesso_a_servicos_mobilidade_cidade_inteira.html</t>
+          <t>https://quadrifygit.github.io/dataquadri/mapas2/mapa_aderencia_rogerio_itu_sp_2022_saude_ubs_consultas_exames_basicos_acesso_sus_cidade_inteira.html</t>
         </is>
       </c>
     </row>
@@ -1218,7 +1218,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>salto</t>
+          <t>itu</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1252,33 +1252,33 @@
         </is>
       </c>
       <c r="I8" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="J8" t="n">
-        <v>60.40720914054178</v>
+        <v>28.69923724840312</v>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>Aderência positiva moderada</t>
+          <t>Forte relação inversa</t>
         </is>
       </c>
       <c r="L8" t="n">
-        <v>0.321048793129752</v>
+        <v>-0.5588103316425902</v>
       </c>
       <c r="M8" t="n">
-        <v>66.05243965648761</v>
+        <v>22.05948341787049</v>
       </c>
       <c r="N8" t="n">
-        <v>0.9978731832195397</v>
+        <v>0.7798174513384127</v>
       </c>
       <c r="O8" t="n">
-        <v>49.9232096109281</v>
+        <v>41.03020864796372</v>
       </c>
       <c r="P8" t="n">
-        <v>240.4783054321831</v>
+        <v>50.32344697494485</v>
       </c>
       <c r="Q8" t="n">
-        <v>239.9668521368533</v>
+        <v>39.24310216256525</v>
       </c>
       <c r="R8" t="inlineStr">
         <is>
@@ -1286,10 +1286,10 @@
         </is>
       </c>
       <c r="S8" t="n">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="T8" t="n">
-        <v>17597</v>
+        <v>4722</v>
       </c>
       <c r="U8" t="n">
         <v>0</v>
@@ -1309,12 +1309,12 @@
       </c>
       <c r="Y8" t="inlineStr">
         <is>
-          <t>C:\Users\guilh\Trabalho\Relatórios Alisson\Documentos gerais\Git\2\dataquadri\mapas2\mapa_aderencia_rogerio_salto_sp_2022_assistencia_social_protecao_social_seguridade_assistencia_rede_publica_cidade_inteira.html</t>
+          <t>C:\Users\guilh\Trabalho\Relatórios Alisson\Documentos gerais\Git\2\dataquadri\mapas2\mapa_aderencia_rogerio_itu_sp_2022_assistencia_social_protecao_social_seguridade_assistencia_rede_publica_cidade_inteira.html</t>
         </is>
       </c>
       <c r="Z8" t="inlineStr">
         <is>
-          <t>https://quadrifygit.github.io/dataquadri/mapas2/mapa_aderencia_rogerio_salto_sp_2022_assistencia_social_protecao_social_seguridade_assistencia_rede_publica_cidade_inteira.html</t>
+          <t>https://quadrifygit.github.io/dataquadri/mapas2/mapa_aderencia_rogerio_itu_sp_2022_assistencia_social_protecao_social_seguridade_assistencia_rede_publica_cidade_inteira.html</t>
         </is>
       </c>
     </row>
@@ -1356,14 +1356,14 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Saúde - UBS, consultas, exames básicos, acesso SUS</t>
+          <t>Mobilidade e Acessibilidade - Transporte, calçadas, acesso a serviços, mobilidade</t>
         </is>
       </c>
       <c r="I9" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J9" t="n">
-        <v>60.29994840725742</v>
+        <v>63.30874465234245</v>
       </c>
       <c r="K9" t="inlineStr">
         <is>
@@ -1371,22 +1371,22 @@
         </is>
       </c>
       <c r="L9" t="n">
-        <v>0.3177484628748488</v>
+        <v>0.4167583705219454</v>
       </c>
       <c r="M9" t="n">
-        <v>65.88742314374244</v>
+        <v>70.83791852609727</v>
       </c>
       <c r="N9" t="n">
-        <v>0.9978731832195397</v>
+        <v>0.9814860902605079</v>
       </c>
       <c r="O9" t="n">
-        <v>49.9232096109281</v>
+        <v>49.32599317251208</v>
       </c>
       <c r="P9" t="n">
         <v>240.4783054321831</v>
       </c>
       <c r="Q9" t="n">
-        <v>239.9668521368533</v>
+        <v>236.0261117911057</v>
       </c>
       <c r="R9" t="inlineStr">
         <is>
@@ -1417,12 +1417,12 @@
       </c>
       <c r="Y9" t="inlineStr">
         <is>
-          <t>C:\Users\guilh\Trabalho\Relatórios Alisson\Documentos gerais\Git\2\dataquadri\mapas2\mapa_aderencia_rogerio_salto_sp_2022_saude_ubs_consultas_exames_basicos_acesso_sus_cidade_inteira.html</t>
+          <t>C:\Users\guilh\Trabalho\Relatórios Alisson\Documentos gerais\Git\2\dataquadri\mapas2\mapa_aderencia_rogerio_salto_sp_2022_mobilidade_e_acessibilidade_transporte_calcadas_acesso_a_servicos_mobilidade_cidade_inteira.html</t>
         </is>
       </c>
       <c r="Z9" t="inlineStr">
         <is>
-          <t>https://quadrifygit.github.io/dataquadri/mapas2/mapa_aderencia_rogerio_salto_sp_2022_saude_ubs_consultas_exames_basicos_acesso_sus_cidade_inteira.html</t>
+          <t>https://quadrifygit.github.io/dataquadri/mapas2/mapa_aderencia_rogerio_salto_sp_2022_mobilidade_e_acessibilidade_transporte_calcadas_acesso_a_servicos_mobilidade_cidade_inteira.html</t>
         </is>
       </c>
     </row>
@@ -1464,37 +1464,37 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Comportamento Político - Qualidade de gestão, eficiência, entrega de serviços</t>
+          <t>Bem-Estar e Serviços - Busca por qualidade de vida, serviços, lazer</t>
         </is>
       </c>
       <c r="I10" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J10" t="n">
-        <v>55.6793858563519</v>
+        <v>62.58152253016321</v>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>Relação fraca ou neutra</t>
+          <t>Aderência positiva moderada</t>
         </is>
       </c>
       <c r="L10" t="n">
-        <v>0.1762009652756663</v>
+        <v>0.3712871536766121</v>
       </c>
       <c r="M10" t="n">
-        <v>58.81004826378331</v>
+        <v>68.56435768383061</v>
       </c>
       <c r="N10" t="n">
-        <v>0.9962722475706126</v>
+        <v>1.041614703086268</v>
       </c>
       <c r="O10" t="n">
-        <v>49.86529852826499</v>
+        <v>51.47054295906663</v>
       </c>
       <c r="P10" t="n">
         <v>240.4783054321831</v>
       </c>
       <c r="Q10" t="n">
-        <v>239.5818618448934</v>
+        <v>250.4857387114324</v>
       </c>
       <c r="R10" t="inlineStr">
         <is>
@@ -1525,12 +1525,12 @@
       </c>
       <c r="Y10" t="inlineStr">
         <is>
-          <t>C:\Users\guilh\Trabalho\Relatórios Alisson\Documentos gerais\Git\2\dataquadri\mapas2\mapa_aderencia_rogerio_salto_sp_2022_comportamento_politico_qualidade_de_gestao_eficiencia_entrega_de_servicos_cidade_inteira.html</t>
+          <t>C:\Users\guilh\Trabalho\Relatórios Alisson\Documentos gerais\Git\2\dataquadri\mapas2\mapa_aderencia_rogerio_salto_sp_2022_bem_estar_e_servicos_busca_por_qualidade_de_vida_servicos_lazer_cidade_inteira.html</t>
         </is>
       </c>
       <c r="Z10" t="inlineStr">
         <is>
-          <t>https://quadrifygit.github.io/dataquadri/mapas2/mapa_aderencia_rogerio_salto_sp_2022_comportamento_politico_qualidade_de_gestao_eficiencia_entrega_de_servicos_cidade_inteira.html</t>
+          <t>https://quadrifygit.github.io/dataquadri/mapas2/mapa_aderencia_rogerio_salto_sp_2022_bem_estar_e_servicos_busca_por_qualidade_de_vida_servicos_lazer_cidade_inteira.html</t>
         </is>
       </c>
     </row>
@@ -1572,37 +1572,37 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Proteção Animal - Proteção animal, bem-estar, resgate, políticas pets</t>
+          <t>Assistência Social - Proteção social, seguridade, assistência, rede pública</t>
         </is>
       </c>
       <c r="I11" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J11" t="n">
-        <v>53.43884739138753</v>
+        <v>60.40720914054178</v>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>Relação fraca ou neutra</t>
+          <t>Aderência positiva moderada</t>
         </is>
       </c>
       <c r="L11" t="n">
-        <v>0.09479281898805356</v>
+        <v>0.321048793129752</v>
       </c>
       <c r="M11" t="n">
-        <v>54.73964094940268</v>
+        <v>66.05243965648761</v>
       </c>
       <c r="N11" t="n">
-        <v>1.028772167187943</v>
+        <v>0.9978731832195397</v>
       </c>
       <c r="O11" t="n">
-        <v>51.02308792650224</v>
+        <v>49.9232096109281</v>
       </c>
       <c r="P11" t="n">
         <v>240.4783054321831</v>
       </c>
       <c r="Q11" t="n">
-        <v>247.3973874411511</v>
+        <v>239.9668521368533</v>
       </c>
       <c r="R11" t="inlineStr">
         <is>
@@ -1633,12 +1633,444 @@
       </c>
       <c r="Y11" t="inlineStr">
         <is>
+          <t>C:\Users\guilh\Trabalho\Relatórios Alisson\Documentos gerais\Git\2\dataquadri\mapas2\mapa_aderencia_rogerio_salto_sp_2022_assistencia_social_protecao_social_seguridade_assistencia_rede_publica_cidade_inteira.html</t>
+        </is>
+      </c>
+      <c r="Z11" t="inlineStr">
+        <is>
+          <t>https://quadrifygit.github.io/dataquadri/mapas2/mapa_aderencia_rogerio_salto_sp_2022_assistencia_social_protecao_social_seguridade_assistencia_rede_publica_cidade_inteira.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>salto</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>ROGERIO NOGUEIRA LOPES CRUZ</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>DEPUTADO ESTADUAL</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>cidade_inteira</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Saúde - UBS, consultas, exames básicos, acesso SUS</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
+        <v>4</v>
+      </c>
+      <c r="J12" t="n">
+        <v>60.29994840725742</v>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>Aderência positiva moderada</t>
+        </is>
+      </c>
+      <c r="L12" t="n">
+        <v>0.3177484628748488</v>
+      </c>
+      <c r="M12" t="n">
+        <v>65.88742314374244</v>
+      </c>
+      <c r="N12" t="n">
+        <v>0.9978731832195397</v>
+      </c>
+      <c r="O12" t="n">
+        <v>49.9232096109281</v>
+      </c>
+      <c r="P12" t="n">
+        <v>240.4783054321831</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>239.9668521368533</v>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>votos por mil</t>
+        </is>
+      </c>
+      <c r="S12" t="n">
+        <v>32</v>
+      </c>
+      <c r="T12" t="n">
+        <v>17597</v>
+      </c>
+      <c r="U12" t="n">
+        <v>0</v>
+      </c>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="W12" t="inlineStr">
+        <is>
+          <t>Total de votos do cargo/turno no local</t>
+        </is>
+      </c>
+      <c r="X12" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y12" t="inlineStr">
+        <is>
+          <t>C:\Users\guilh\Trabalho\Relatórios Alisson\Documentos gerais\Git\2\dataquadri\mapas2\mapa_aderencia_rogerio_salto_sp_2022_saude_ubs_consultas_exames_basicos_acesso_sus_cidade_inteira.html</t>
+        </is>
+      </c>
+      <c r="Z12" t="inlineStr">
+        <is>
+          <t>https://quadrifygit.github.io/dataquadri/mapas2/mapa_aderencia_rogerio_salto_sp_2022_saude_ubs_consultas_exames_basicos_acesso_sus_cidade_inteira.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>salto</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>ROGERIO NOGUEIRA LOPES CRUZ</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>DEPUTADO ESTADUAL</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>cidade_inteira</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Comportamento Político - Qualidade de gestão, eficiência, entrega de serviços</t>
+        </is>
+      </c>
+      <c r="I13" t="n">
+        <v>5</v>
+      </c>
+      <c r="J13" t="n">
+        <v>55.6793858563519</v>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>Relação fraca ou neutra</t>
+        </is>
+      </c>
+      <c r="L13" t="n">
+        <v>0.1762009652756663</v>
+      </c>
+      <c r="M13" t="n">
+        <v>58.81004826378331</v>
+      </c>
+      <c r="N13" t="n">
+        <v>0.9962722475706126</v>
+      </c>
+      <c r="O13" t="n">
+        <v>49.86529852826499</v>
+      </c>
+      <c r="P13" t="n">
+        <v>240.4783054321831</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>239.5818618448934</v>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>votos por mil</t>
+        </is>
+      </c>
+      <c r="S13" t="n">
+        <v>32</v>
+      </c>
+      <c r="T13" t="n">
+        <v>17597</v>
+      </c>
+      <c r="U13" t="n">
+        <v>0</v>
+      </c>
+      <c r="V13" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="W13" t="inlineStr">
+        <is>
+          <t>Total de votos do cargo/turno no local</t>
+        </is>
+      </c>
+      <c r="X13" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y13" t="inlineStr">
+        <is>
+          <t>C:\Users\guilh\Trabalho\Relatórios Alisson\Documentos gerais\Git\2\dataquadri\mapas2\mapa_aderencia_rogerio_salto_sp_2022_comportamento_politico_qualidade_de_gestao_eficiencia_entrega_de_servicos_cidade_inteira.html</t>
+        </is>
+      </c>
+      <c r="Z13" t="inlineStr">
+        <is>
+          <t>https://quadrifygit.github.io/dataquadri/mapas2/mapa_aderencia_rogerio_salto_sp_2022_comportamento_politico_qualidade_de_gestao_eficiencia_entrega_de_servicos_cidade_inteira.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>salto</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>ROGERIO NOGUEIRA LOPES CRUZ</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>DEPUTADO ESTADUAL</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>cidade_inteira</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Proteção Animal - Proteção animal, bem-estar, resgate, políticas pets</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
+        <v>6</v>
+      </c>
+      <c r="J14" t="n">
+        <v>53.43884739138753</v>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>Relação fraca ou neutra</t>
+        </is>
+      </c>
+      <c r="L14" t="n">
+        <v>0.09479281898805356</v>
+      </c>
+      <c r="M14" t="n">
+        <v>54.73964094940268</v>
+      </c>
+      <c r="N14" t="n">
+        <v>1.028772167187943</v>
+      </c>
+      <c r="O14" t="n">
+        <v>51.02308792650224</v>
+      </c>
+      <c r="P14" t="n">
+        <v>240.4783054321831</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>247.3973874411511</v>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>votos por mil</t>
+        </is>
+      </c>
+      <c r="S14" t="n">
+        <v>32</v>
+      </c>
+      <c r="T14" t="n">
+        <v>17597</v>
+      </c>
+      <c r="U14" t="n">
+        <v>0</v>
+      </c>
+      <c r="V14" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="W14" t="inlineStr">
+        <is>
+          <t>Total de votos do cargo/turno no local</t>
+        </is>
+      </c>
+      <c r="X14" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y14" t="inlineStr">
+        <is>
           <t>C:\Users\guilh\Trabalho\Relatórios Alisson\Documentos gerais\Git\2\dataquadri\mapas2\mapa_aderencia_rogerio_salto_sp_2022_protecao_animal_protecao_animal_bem_estar_resgate_politicas_pets_cidade_inteira.html</t>
         </is>
       </c>
-      <c r="Z11" t="inlineStr">
+      <c r="Z14" t="inlineStr">
         <is>
           <t>https://quadrifygit.github.io/dataquadri/mapas2/mapa_aderencia_rogerio_salto_sp_2022_protecao_animal_protecao_animal_bem_estar_resgate_politicas_pets_cidade_inteira.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>salto</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>ROGERIO NOGUEIRA LOPES CRUZ</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>DEPUTADO ESTADUAL</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>cidade_inteira</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Bem-Estar e Serviços - Qualidade do bairro, serviços, segurança, lazer</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
+        <v>7</v>
+      </c>
+      <c r="J15" t="n">
+        <v>51.6473882332125</v>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>Relação fraca ou neutra</t>
+        </is>
+      </c>
+      <c r="L15" t="n">
+        <v>0.05592226265252676</v>
+      </c>
+      <c r="M15" t="n">
+        <v>52.79611313262635</v>
+      </c>
+      <c r="N15" t="n">
+        <v>0.9866167459431195</v>
+      </c>
+      <c r="O15" t="n">
+        <v>49.51404199144392</v>
+      </c>
+      <c r="P15" t="n">
+        <v>240.4783054321831</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>237.2599231754161</v>
+      </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>votos por mil</t>
+        </is>
+      </c>
+      <c r="S15" t="n">
+        <v>32</v>
+      </c>
+      <c r="T15" t="n">
+        <v>17597</v>
+      </c>
+      <c r="U15" t="n">
+        <v>0</v>
+      </c>
+      <c r="V15" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="W15" t="inlineStr">
+        <is>
+          <t>Total de votos do cargo/turno no local</t>
+        </is>
+      </c>
+      <c r="X15" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y15" t="inlineStr">
+        <is>
+          <t>C:\Users\guilh\Trabalho\Relatórios Alisson\Documentos gerais\Git\2\dataquadri\mapas2\mapa_aderencia_rogerio_salto_sp_2022_bem_estar_e_servicos_qualidade_do_bairro_servicos_seguranca_lazer_cidade_inteira.html</t>
+        </is>
+      </c>
+      <c r="Z15" t="inlineStr">
+        <is>
+          <t>https://quadrifygit.github.io/dataquadri/mapas2/mapa_aderencia_rogerio_salto_sp_2022_bem_estar_e_servicos_qualidade_do_bairro_servicos_seguranca_lazer_cidade_inteira.html</t>
         </is>
       </c>
     </row>
@@ -1653,7 +2085,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M41"/>
+  <dimension ref="A1:M57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1971,26 +2403,26 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Comportamento Político - Qualidade de gestão, eficiência, entrega de serviços</t>
+          <t>Bem-Estar e Serviços - Busca por qualidade de vida, serviços, lazer</t>
         </is>
       </c>
       <c r="G6" t="n">
         <v>1</v>
       </c>
       <c r="H6" t="n">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="I6" t="n">
-        <v>179</v>
+        <v>2175</v>
       </c>
       <c r="J6" t="n">
-        <v>2311</v>
+        <v>40684</v>
       </c>
       <c r="K6" t="n">
-        <v>77.45564690610125</v>
+        <v>53.46081997836988</v>
       </c>
       <c r="L6" t="n">
-        <v>3.790766624311733</v>
+        <v>46.06099110546379</v>
       </c>
       <c r="M6" t="inlineStr">
         <is>
@@ -2026,26 +2458,26 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Comportamento Político - Qualidade de gestão, eficiência, entrega de serviços</t>
+          <t>Bem-Estar e Serviços - Busca por qualidade de vida, serviços, lazer</t>
         </is>
       </c>
       <c r="G7" t="n">
         <v>2</v>
       </c>
       <c r="H7" t="n">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="I7" t="n">
-        <v>2246</v>
+        <v>814</v>
       </c>
       <c r="J7" t="n">
-        <v>46189</v>
+        <v>13655</v>
       </c>
       <c r="K7" t="n">
-        <v>48.62629630431488</v>
+        <v>59.61186378615891</v>
       </c>
       <c r="L7" t="n">
-        <v>47.56459127488352</v>
+        <v>17.23845828038966</v>
       </c>
       <c r="M7" t="inlineStr">
         <is>
@@ -2081,26 +2513,26 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Comportamento Político - Qualidade de gestão, eficiência, entrega de serviços</t>
+          <t>Bem-Estar e Serviços - Busca por qualidade de vida, serviços, lazer</t>
         </is>
       </c>
       <c r="G8" t="n">
         <v>3</v>
       </c>
       <c r="H8" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="I8" t="n">
-        <v>1547</v>
+        <v>576</v>
       </c>
       <c r="J8" t="n">
-        <v>30873</v>
+        <v>11524</v>
       </c>
       <c r="K8" t="n">
-        <v>50.10850905321802</v>
+        <v>49.98264491496008</v>
       </c>
       <c r="L8" t="n">
-        <v>32.76154171961034</v>
+        <v>12.19822109275731</v>
       </c>
       <c r="M8" t="inlineStr">
         <is>
@@ -2136,26 +2568,26 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Comportamento Político - Qualidade de gestão, eficiência, entrega de serviços</t>
+          <t>Bem-Estar e Serviços - Busca por qualidade de vida, serviços, lazer</t>
         </is>
       </c>
       <c r="G9" t="n">
         <v>4</v>
       </c>
       <c r="H9" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="I9" t="n">
-        <v>750</v>
+        <v>1157</v>
       </c>
       <c r="J9" t="n">
-        <v>14460</v>
+        <v>27970</v>
       </c>
       <c r="K9" t="n">
-        <v>51.86721991701245</v>
+        <v>41.36574901680372</v>
       </c>
       <c r="L9" t="n">
-        <v>15.88310038119441</v>
+        <v>24.50232952138924</v>
       </c>
       <c r="M9" t="inlineStr">
         <is>
@@ -2191,26 +2623,26 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Mobilidade e Acessibilidade - Transporte, calçadas, acesso a serviços, mobilidade</t>
+          <t>Bem-Estar e Serviços - Qualidade do bairro, serviços, segurança, lazer</t>
         </is>
       </c>
       <c r="G10" t="n">
         <v>1</v>
       </c>
       <c r="H10" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="I10" t="n">
-        <v>2149</v>
+        <v>13</v>
       </c>
       <c r="J10" t="n">
-        <v>40283</v>
+        <v>251</v>
       </c>
       <c r="K10" t="n">
-        <v>53.3475659707569</v>
+        <v>51.79282868525897</v>
       </c>
       <c r="L10" t="n">
-        <v>45.51037695891571</v>
+        <v>0.2753070732740364</v>
       </c>
       <c r="M10" t="inlineStr">
         <is>
@@ -2246,26 +2678,26 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Mobilidade e Acessibilidade - Transporte, calçadas, acesso a serviços, mobilidade</t>
+          <t>Bem-Estar e Serviços - Qualidade do bairro, serviços, segurança, lazer</t>
         </is>
       </c>
       <c r="G11" t="n">
         <v>2</v>
       </c>
       <c r="H11" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="I11" t="n">
-        <v>1154</v>
+        <v>869</v>
       </c>
       <c r="J11" t="n">
-        <v>20731</v>
+        <v>22532</v>
       </c>
       <c r="K11" t="n">
-        <v>55.66542858521056</v>
+        <v>38.56737085034617</v>
       </c>
       <c r="L11" t="n">
-        <v>24.43879711986446</v>
+        <v>18.40321897501059</v>
       </c>
       <c r="M11" t="inlineStr">
         <is>
@@ -2301,26 +2733,26 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Mobilidade e Acessibilidade - Transporte, calçadas, acesso a serviços, mobilidade</t>
+          <t>Bem-Estar e Serviços - Qualidade do bairro, serviços, segurança, lazer</t>
         </is>
       </c>
       <c r="G12" t="n">
         <v>3</v>
       </c>
       <c r="H12" t="n">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="I12" t="n">
-        <v>1314</v>
+        <v>2809</v>
       </c>
       <c r="J12" t="n">
-        <v>29471</v>
+        <v>52204</v>
       </c>
       <c r="K12" t="n">
-        <v>44.58620338637983</v>
+        <v>53.80813730748601</v>
       </c>
       <c r="L12" t="n">
-        <v>27.82719186785261</v>
+        <v>59.48750529436679</v>
       </c>
       <c r="M12" t="inlineStr">
         <is>
@@ -2356,26 +2788,26 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Mobilidade e Acessibilidade - Transporte, calçadas, acesso a serviços, mobilidade</t>
+          <t>Bem-Estar e Serviços - Qualidade do bairro, serviços, segurança, lazer</t>
         </is>
       </c>
       <c r="G13" t="n">
         <v>4</v>
       </c>
       <c r="H13" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="I13" t="n">
-        <v>105</v>
+        <v>1031</v>
       </c>
       <c r="J13" t="n">
-        <v>3348</v>
+        <v>18846</v>
       </c>
       <c r="K13" t="n">
-        <v>31.36200716845878</v>
+        <v>54.7065690332166</v>
       </c>
       <c r="L13" t="n">
-        <v>2.223634053367217</v>
+        <v>21.83396865734858</v>
       </c>
       <c r="M13" t="inlineStr">
         <is>
@@ -2411,26 +2843,26 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Proteção Animal - Proteção animal, bem-estar, resgate, políticas pets</t>
+          <t>Comportamento Político - Qualidade de gestão, eficiência, entrega de serviços</t>
         </is>
       </c>
       <c r="G14" t="n">
         <v>1</v>
       </c>
       <c r="H14" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="I14" t="n">
-        <v>1130</v>
+        <v>179</v>
       </c>
       <c r="J14" t="n">
-        <v>20098</v>
+        <v>2311</v>
       </c>
       <c r="K14" t="n">
-        <v>56.2244999502438</v>
+        <v>77.45564690610125</v>
       </c>
       <c r="L14" t="n">
-        <v>23.93053790766625</v>
+        <v>3.790766624311733</v>
       </c>
       <c r="M14" t="inlineStr">
         <is>
@@ -2466,26 +2898,26 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Proteção Animal - Proteção animal, bem-estar, resgate, políticas pets</t>
+          <t>Comportamento Político - Qualidade de gestão, eficiência, entrega de serviços</t>
         </is>
       </c>
       <c r="G15" t="n">
         <v>2</v>
       </c>
       <c r="H15" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="I15" t="n">
-        <v>904</v>
+        <v>2246</v>
       </c>
       <c r="J15" t="n">
-        <v>18629</v>
+        <v>46189</v>
       </c>
       <c r="K15" t="n">
-        <v>48.52649095496269</v>
+        <v>48.62629630431488</v>
       </c>
       <c r="L15" t="n">
-        <v>19.14443032613299</v>
+        <v>47.56459127488352</v>
       </c>
       <c r="M15" t="inlineStr">
         <is>
@@ -2521,26 +2953,26 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Proteção Animal - Proteção animal, bem-estar, resgate, políticas pets</t>
+          <t>Comportamento Político - Qualidade de gestão, eficiência, entrega de serviços</t>
         </is>
       </c>
       <c r="G16" t="n">
         <v>3</v>
       </c>
       <c r="H16" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="I16" t="n">
-        <v>1531</v>
+        <v>1547</v>
       </c>
       <c r="J16" t="n">
-        <v>34091</v>
+        <v>30873</v>
       </c>
       <c r="K16" t="n">
-        <v>44.90921357543046</v>
+        <v>50.10850905321802</v>
       </c>
       <c r="L16" t="n">
-        <v>32.42270224481152</v>
+        <v>32.76154171961034</v>
       </c>
       <c r="M16" t="inlineStr">
         <is>
@@ -2576,26 +3008,26 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Proteção Animal - Proteção animal, bem-estar, resgate, políticas pets</t>
+          <t>Comportamento Político - Qualidade de gestão, eficiência, entrega de serviços</t>
         </is>
       </c>
       <c r="G17" t="n">
         <v>4</v>
       </c>
       <c r="H17" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="I17" t="n">
-        <v>1157</v>
+        <v>750</v>
       </c>
       <c r="J17" t="n">
-        <v>21015</v>
+        <v>14460</v>
       </c>
       <c r="K17" t="n">
-        <v>55.05591244349274</v>
+        <v>51.86721991701245</v>
       </c>
       <c r="L17" t="n">
-        <v>24.50232952138924</v>
+        <v>15.88310038119441</v>
       </c>
       <c r="M17" t="inlineStr">
         <is>
@@ -2631,26 +3063,26 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Saúde - UBS, consultas, exames básicos, acesso SUS</t>
+          <t>Mobilidade e Acessibilidade - Transporte, calçadas, acesso a serviços, mobilidade</t>
         </is>
       </c>
       <c r="G18" t="n">
         <v>1</v>
       </c>
       <c r="H18" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="I18" t="n">
-        <v>2445</v>
+        <v>2149</v>
       </c>
       <c r="J18" t="n">
-        <v>43069</v>
+        <v>40283</v>
       </c>
       <c r="K18" t="n">
-        <v>56.76937008056839</v>
+        <v>53.3475659707569</v>
       </c>
       <c r="L18" t="n">
-        <v>51.77890724269377</v>
+        <v>45.51037695891571</v>
       </c>
       <c r="M18" t="inlineStr">
         <is>
@@ -2686,7 +3118,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Saúde - UBS, consultas, exames básicos, acesso SUS</t>
+          <t>Mobilidade e Acessibilidade - Transporte, calçadas, acesso a serviços, mobilidade</t>
         </is>
       </c>
       <c r="G19" t="n">
@@ -2696,16 +3128,16 @@
         <v>8</v>
       </c>
       <c r="I19" t="n">
-        <v>966</v>
+        <v>1154</v>
       </c>
       <c r="J19" t="n">
-        <v>18608</v>
+        <v>20731</v>
       </c>
       <c r="K19" t="n">
-        <v>51.91315563198624</v>
+        <v>55.66542858521056</v>
       </c>
       <c r="L19" t="n">
-        <v>20.4574332909784</v>
+        <v>24.43879711986446</v>
       </c>
       <c r="M19" t="inlineStr">
         <is>
@@ -2741,26 +3173,26 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Saúde - UBS, consultas, exames básicos, acesso SUS</t>
+          <t>Mobilidade e Acessibilidade - Transporte, calçadas, acesso a serviços, mobilidade</t>
         </is>
       </c>
       <c r="G20" t="n">
         <v>3</v>
       </c>
       <c r="H20" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="I20" t="n">
-        <v>469</v>
+        <v>1314</v>
       </c>
       <c r="J20" t="n">
-        <v>10700</v>
+        <v>29471</v>
       </c>
       <c r="K20" t="n">
-        <v>43.83177570093458</v>
+        <v>44.58620338637983</v>
       </c>
       <c r="L20" t="n">
-        <v>9.932232105040237</v>
+        <v>27.82719186785261</v>
       </c>
       <c r="M20" t="inlineStr">
         <is>
@@ -2796,26 +3228,26 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Saúde - UBS, consultas, exames básicos, acesso SUS</t>
+          <t>Mobilidade e Acessibilidade - Transporte, calçadas, acesso a serviços, mobilidade</t>
         </is>
       </c>
       <c r="G21" t="n">
         <v>4</v>
       </c>
       <c r="H21" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="I21" t="n">
-        <v>842</v>
+        <v>105</v>
       </c>
       <c r="J21" t="n">
-        <v>21456</v>
+        <v>3348</v>
       </c>
       <c r="K21" t="n">
-        <v>39.24310216256525</v>
+        <v>31.36200716845878</v>
       </c>
       <c r="L21" t="n">
-        <v>17.83142736128759</v>
+        <v>2.223634053367217</v>
       </c>
       <c r="M21" t="inlineStr">
         <is>
@@ -2831,7 +3263,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>salto</t>
+          <t>itu</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -2851,26 +3283,26 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Assistência Social - Proteção social, seguridade, assistência, rede pública</t>
+          <t>Proteção Animal - Proteção animal, bem-estar, resgate, políticas pets</t>
         </is>
       </c>
       <c r="G22" t="n">
         <v>1</v>
       </c>
       <c r="H22" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="I22" t="n">
-        <v>5411</v>
+        <v>1130</v>
       </c>
       <c r="J22" t="n">
-        <v>24471</v>
+        <v>20098</v>
       </c>
       <c r="K22" t="n">
-        <v>221.1188754035389</v>
+        <v>56.2244999502438</v>
       </c>
       <c r="L22" t="n">
-        <v>30.74955958402</v>
+        <v>23.93053790766625</v>
       </c>
       <c r="M22" t="inlineStr">
         <is>
@@ -2886,7 +3318,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>salto</t>
+          <t>itu</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -2906,7 +3338,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Assistência Social - Proteção social, seguridade, assistência, rede pública</t>
+          <t>Proteção Animal - Proteção animal, bem-estar, resgate, políticas pets</t>
         </is>
       </c>
       <c r="G23" t="n">
@@ -2916,16 +3348,16 @@
         <v>8</v>
       </c>
       <c r="I23" t="n">
-        <v>4640</v>
+        <v>904</v>
       </c>
       <c r="J23" t="n">
-        <v>17952</v>
+        <v>18629</v>
       </c>
       <c r="K23" t="n">
-        <v>258.4670231729056</v>
+        <v>48.52649095496269</v>
       </c>
       <c r="L23" t="n">
-        <v>26.36813093140876</v>
+        <v>19.14443032613299</v>
       </c>
       <c r="M23" t="inlineStr">
         <is>
@@ -2941,7 +3373,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>salto</t>
+          <t>itu</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -2961,26 +3393,26 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Assistência Social - Proteção social, seguridade, assistência, rede pública</t>
+          <t>Proteção Animal - Proteção animal, bem-estar, resgate, políticas pets</t>
         </is>
       </c>
       <c r="G24" t="n">
         <v>3</v>
       </c>
       <c r="H24" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="I24" t="n">
-        <v>3492</v>
+        <v>1531</v>
       </c>
       <c r="J24" t="n">
-        <v>13858</v>
+        <v>34091</v>
       </c>
       <c r="K24" t="n">
-        <v>251.9844133352576</v>
+        <v>44.90921357543046</v>
       </c>
       <c r="L24" t="n">
-        <v>19.84429164062056</v>
+        <v>32.42270224481152</v>
       </c>
       <c r="M24" t="inlineStr">
         <is>
@@ -2996,7 +3428,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>salto</t>
+          <t>itu</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -3016,26 +3448,26 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Assistência Social - Proteção social, seguridade, assistência, rede pública</t>
+          <t>Proteção Animal - Proteção animal, bem-estar, resgate, políticas pets</t>
         </is>
       </c>
       <c r="G25" t="n">
         <v>4</v>
       </c>
       <c r="H25" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="I25" t="n">
-        <v>4054</v>
+        <v>1157</v>
       </c>
       <c r="J25" t="n">
-        <v>16894</v>
+        <v>21015</v>
       </c>
       <c r="K25" t="n">
-        <v>239.9668521368533</v>
+        <v>55.05591244349274</v>
       </c>
       <c r="L25" t="n">
-        <v>23.03801784395067</v>
+        <v>24.50232952138924</v>
       </c>
       <c r="M25" t="inlineStr">
         <is>
@@ -3051,7 +3483,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>salto</t>
+          <t>itu</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -3071,26 +3503,26 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Comportamento Político - Qualidade de gestão, eficiência, entrega de serviços</t>
+          <t>Saúde - UBS, consultas, exames básicos, acesso SUS</t>
         </is>
       </c>
       <c r="G26" t="n">
         <v>1</v>
       </c>
       <c r="H26" t="n">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="I26" t="n">
-        <v>3212</v>
+        <v>2445</v>
       </c>
       <c r="J26" t="n">
-        <v>14760</v>
+        <v>43069</v>
       </c>
       <c r="K26" t="n">
-        <v>217.6151761517615</v>
+        <v>56.76937008056839</v>
       </c>
       <c r="L26" t="n">
-        <v>18.25311132579417</v>
+        <v>51.77890724269377</v>
       </c>
       <c r="M26" t="inlineStr">
         <is>
@@ -3106,7 +3538,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>salto</t>
+          <t>itu</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -3126,26 +3558,26 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Comportamento Político - Qualidade de gestão, eficiência, entrega de serviços</t>
+          <t>Saúde - UBS, consultas, exames básicos, acesso SUS</t>
         </is>
       </c>
       <c r="G27" t="n">
         <v>2</v>
       </c>
       <c r="H27" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="I27" t="n">
-        <v>7153</v>
+        <v>966</v>
       </c>
       <c r="J27" t="n">
-        <v>29390</v>
+        <v>18608</v>
       </c>
       <c r="K27" t="n">
-        <v>243.3821027560395</v>
+        <v>51.91315563198624</v>
       </c>
       <c r="L27" t="n">
-        <v>40.64897425697562</v>
+        <v>20.4574332909784</v>
       </c>
       <c r="M27" t="inlineStr">
         <is>
@@ -3161,7 +3593,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>salto</t>
+          <t>itu</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -3181,26 +3613,26 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Comportamento Político - Qualidade de gestão, eficiência, entrega de serviços</t>
+          <t>Saúde - UBS, consultas, exames básicos, acesso SUS</t>
         </is>
       </c>
       <c r="G28" t="n">
         <v>3</v>
       </c>
       <c r="H28" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="I28" t="n">
-        <v>5536</v>
+        <v>469</v>
       </c>
       <c r="J28" t="n">
-        <v>21946</v>
+        <v>10700</v>
       </c>
       <c r="K28" t="n">
-        <v>252.255536316413</v>
+        <v>43.83177570093458</v>
       </c>
       <c r="L28" t="n">
-        <v>31.45990793885322</v>
+        <v>9.932232105040237</v>
       </c>
       <c r="M28" t="inlineStr">
         <is>
@@ -3216,7 +3648,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>salto</t>
+          <t>itu</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -3236,26 +3668,26 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Comportamento Político - Qualidade de gestão, eficiência, entrega de serviços</t>
+          <t>Saúde - UBS, consultas, exames básicos, acesso SUS</t>
         </is>
       </c>
       <c r="G29" t="n">
         <v>4</v>
       </c>
       <c r="H29" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="I29" t="n">
-        <v>1696</v>
+        <v>842</v>
       </c>
       <c r="J29" t="n">
-        <v>7079</v>
+        <v>21456</v>
       </c>
       <c r="K29" t="n">
-        <v>239.5818618448934</v>
+        <v>39.24310216256525</v>
       </c>
       <c r="L29" t="n">
-        <v>9.638006478376997</v>
+        <v>17.83142736128759</v>
       </c>
       <c r="M29" t="inlineStr">
         <is>
@@ -3291,26 +3723,26 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Mobilidade e Acessibilidade - Transporte, calçadas, acesso a serviços, mobilidade</t>
+          <t>Assistência Social - Proteção social, seguridade, assistência, rede pública</t>
         </is>
       </c>
       <c r="G30" t="n">
         <v>1</v>
       </c>
       <c r="H30" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="I30" t="n">
-        <v>4983</v>
+        <v>5411</v>
       </c>
       <c r="J30" t="n">
-        <v>22743</v>
+        <v>24471</v>
       </c>
       <c r="K30" t="n">
-        <v>219.1003825352856</v>
+        <v>221.1188754035389</v>
       </c>
       <c r="L30" t="n">
-        <v>28.31732681707109</v>
+        <v>30.74955958402</v>
       </c>
       <c r="M30" t="inlineStr">
         <is>
@@ -3346,26 +3778,26 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Mobilidade e Acessibilidade - Transporte, calçadas, acesso a serviços, mobilidade</t>
+          <t>Assistência Social - Proteção social, seguridade, assistência, rede pública</t>
         </is>
       </c>
       <c r="G31" t="n">
         <v>2</v>
       </c>
       <c r="H31" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="I31" t="n">
-        <v>4834</v>
+        <v>4640</v>
       </c>
       <c r="J31" t="n">
-        <v>19745</v>
+        <v>17952</v>
       </c>
       <c r="K31" t="n">
-        <v>244.8214737908331</v>
+        <v>258.4670231729056</v>
       </c>
       <c r="L31" t="n">
-        <v>27.4705915781099</v>
+        <v>26.36813093140876</v>
       </c>
       <c r="M31" t="inlineStr">
         <is>
@@ -3401,26 +3833,26 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Mobilidade e Acessibilidade - Transporte, calçadas, acesso a serviços, mobilidade</t>
+          <t>Assistência Social - Proteção social, seguridade, assistência, rede pública</t>
         </is>
       </c>
       <c r="G32" t="n">
         <v>3</v>
       </c>
       <c r="H32" t="n">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="I32" t="n">
-        <v>6623</v>
+        <v>3492</v>
       </c>
       <c r="J32" t="n">
-        <v>25785</v>
+        <v>13858</v>
       </c>
       <c r="K32" t="n">
-        <v>256.854760519682</v>
+        <v>251.9844133352576</v>
       </c>
       <c r="L32" t="n">
-        <v>37.63709723248281</v>
+        <v>19.84429164062056</v>
       </c>
       <c r="M32" t="inlineStr">
         <is>
@@ -3456,26 +3888,26 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Mobilidade e Acessibilidade - Transporte, calçadas, acesso a serviços, mobilidade</t>
+          <t>Assistência Social - Proteção social, seguridade, assistência, rede pública</t>
         </is>
       </c>
       <c r="G33" t="n">
         <v>4</v>
       </c>
       <c r="H33" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="I33" t="n">
-        <v>1157</v>
+        <v>4054</v>
       </c>
       <c r="J33" t="n">
-        <v>4902</v>
+        <v>16894</v>
       </c>
       <c r="K33" t="n">
-        <v>236.0261117911057</v>
+        <v>239.9668521368533</v>
       </c>
       <c r="L33" t="n">
-        <v>6.574984372336194</v>
+        <v>23.03801784395067</v>
       </c>
       <c r="M33" t="inlineStr">
         <is>
@@ -3511,7 +3943,7 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Proteção Animal - Proteção animal, bem-estar, resgate, políticas pets</t>
+          <t>Bem-Estar e Serviços - Busca por qualidade de vida, serviços, lazer</t>
         </is>
       </c>
       <c r="G34" t="n">
@@ -3521,16 +3953,16 @@
         <v>8</v>
       </c>
       <c r="I34" t="n">
-        <v>5330</v>
+        <v>4075</v>
       </c>
       <c r="J34" t="n">
-        <v>21963</v>
+        <v>18517</v>
       </c>
       <c r="K34" t="n">
-        <v>242.6808723762692</v>
+        <v>220.0680455797375</v>
       </c>
       <c r="L34" t="n">
-        <v>30.28925385008808</v>
+        <v>23.15735636756265</v>
       </c>
       <c r="M34" t="inlineStr">
         <is>
@@ -3566,26 +3998,26 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Proteção Animal - Proteção animal, bem-estar, resgate, políticas pets</t>
+          <t>Bem-Estar e Serviços - Busca por qualidade de vida, serviços, lazer</t>
         </is>
       </c>
       <c r="G35" t="n">
         <v>2</v>
       </c>
       <c r="H35" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="I35" t="n">
-        <v>5165</v>
+        <v>4938</v>
       </c>
       <c r="J35" t="n">
-        <v>22551</v>
+        <v>20661</v>
       </c>
       <c r="K35" t="n">
-        <v>229.0364063677886</v>
+        <v>239.0010164077247</v>
       </c>
       <c r="L35" t="n">
-        <v>29.35159402170824</v>
+        <v>28.06160140933114</v>
       </c>
       <c r="M35" t="inlineStr">
         <is>
@@ -3621,26 +4053,26 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Proteção Animal - Proteção animal, bem-estar, resgate, políticas pets</t>
+          <t>Bem-Estar e Serviços - Busca por qualidade de vida, serviços, lazer</t>
         </is>
       </c>
       <c r="G36" t="n">
         <v>3</v>
       </c>
       <c r="H36" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="I36" t="n">
-        <v>3371</v>
+        <v>5361</v>
       </c>
       <c r="J36" t="n">
-        <v>13580</v>
+        <v>21130</v>
       </c>
       <c r="K36" t="n">
-        <v>248.2326951399116</v>
+        <v>253.7150970184572</v>
       </c>
       <c r="L36" t="n">
-        <v>19.15667443314201</v>
+        <v>30.46542024208672</v>
       </c>
       <c r="M36" t="inlineStr">
         <is>
@@ -3676,26 +4108,26 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Proteção Animal - Proteção animal, bem-estar, resgate, políticas pets</t>
+          <t>Bem-Estar e Serviços - Busca por qualidade de vida, serviços, lazer</t>
         </is>
       </c>
       <c r="G37" t="n">
         <v>4</v>
       </c>
       <c r="H37" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I37" t="n">
-        <v>3731</v>
+        <v>3223</v>
       </c>
       <c r="J37" t="n">
-        <v>15081</v>
+        <v>12867</v>
       </c>
       <c r="K37" t="n">
-        <v>247.3973874411511</v>
+        <v>250.4857387114324</v>
       </c>
       <c r="L37" t="n">
-        <v>21.20247769506166</v>
+        <v>18.31562198101949</v>
       </c>
       <c r="M37" t="inlineStr">
         <is>
@@ -3731,26 +4163,26 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Saúde - UBS, consultas, exames básicos, acesso SUS</t>
+          <t>Bem-Estar e Serviços - Qualidade do bairro, serviços, segurança, lazer</t>
         </is>
       </c>
       <c r="G38" t="n">
         <v>1</v>
       </c>
       <c r="H38" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="I38" t="n">
-        <v>5411</v>
+        <v>4213</v>
       </c>
       <c r="J38" t="n">
-        <v>24471</v>
+        <v>17547</v>
       </c>
       <c r="K38" t="n">
-        <v>221.1188754035389</v>
+        <v>240.0980224539807</v>
       </c>
       <c r="L38" t="n">
-        <v>30.74955958402</v>
+        <v>23.94158095129852</v>
       </c>
       <c r="M38" t="inlineStr">
         <is>
@@ -3786,26 +4218,26 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Saúde - UBS, consultas, exames básicos, acesso SUS</t>
+          <t>Bem-Estar e Serviços - Qualidade do bairro, serviços, segurança, lazer</t>
         </is>
       </c>
       <c r="G39" t="n">
         <v>2</v>
       </c>
       <c r="H39" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="I39" t="n">
-        <v>4640</v>
+        <v>2502</v>
       </c>
       <c r="J39" t="n">
-        <v>17952</v>
+        <v>10764</v>
       </c>
       <c r="K39" t="n">
-        <v>258.4670231729056</v>
+        <v>232.4414715719064</v>
       </c>
       <c r="L39" t="n">
-        <v>26.36813093140876</v>
+        <v>14.21833267034154</v>
       </c>
       <c r="M39" t="inlineStr">
         <is>
@@ -3841,26 +4273,26 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Saúde - UBS, consultas, exames básicos, acesso SUS</t>
+          <t>Bem-Estar e Serviços - Qualidade do bairro, serviços, segurança, lazer</t>
         </is>
       </c>
       <c r="G40" t="n">
         <v>3</v>
       </c>
       <c r="H40" t="n">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="I40" t="n">
-        <v>3492</v>
+        <v>7176</v>
       </c>
       <c r="J40" t="n">
-        <v>13858</v>
+        <v>29244</v>
       </c>
       <c r="K40" t="n">
-        <v>251.9844133352576</v>
+        <v>245.3836684448092</v>
       </c>
       <c r="L40" t="n">
-        <v>19.84429164062056</v>
+        <v>40.77967835426493</v>
       </c>
       <c r="M40" t="inlineStr">
         <is>
@@ -3896,28 +4328,908 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Saúde - UBS, consultas, exames básicos, acesso SUS</t>
+          <t>Bem-Estar e Serviços - Qualidade do bairro, serviços, segurança, lazer</t>
         </is>
       </c>
       <c r="G41" t="n">
         <v>4</v>
       </c>
       <c r="H41" t="n">
+        <v>8</v>
+      </c>
+      <c r="I41" t="n">
+        <v>3706</v>
+      </c>
+      <c r="J41" t="n">
+        <v>15620</v>
+      </c>
+      <c r="K41" t="n">
+        <v>237.2599231754161</v>
+      </c>
+      <c r="L41" t="n">
+        <v>21.06040802409502</v>
+      </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>votos por mil</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>salto</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>ROGERIO NOGUEIRA LOPES CRUZ</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>cidade_inteira</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Comportamento Político - Qualidade de gestão, eficiência, entrega de serviços</t>
+        </is>
+      </c>
+      <c r="G42" t="n">
+        <v>1</v>
+      </c>
+      <c r="H42" t="n">
+        <v>5</v>
+      </c>
+      <c r="I42" t="n">
+        <v>3212</v>
+      </c>
+      <c r="J42" t="n">
+        <v>14760</v>
+      </c>
+      <c r="K42" t="n">
+        <v>217.6151761517615</v>
+      </c>
+      <c r="L42" t="n">
+        <v>18.25311132579417</v>
+      </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>votos por mil</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>salto</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>ROGERIO NOGUEIRA LOPES CRUZ</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>cidade_inteira</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Comportamento Político - Qualidade de gestão, eficiência, entrega de serviços</t>
+        </is>
+      </c>
+      <c r="G43" t="n">
+        <v>2</v>
+      </c>
+      <c r="H43" t="n">
+        <v>12</v>
+      </c>
+      <c r="I43" t="n">
+        <v>7153</v>
+      </c>
+      <c r="J43" t="n">
+        <v>29390</v>
+      </c>
+      <c r="K43" t="n">
+        <v>243.3821027560395</v>
+      </c>
+      <c r="L43" t="n">
+        <v>40.64897425697562</v>
+      </c>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>votos por mil</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>salto</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>ROGERIO NOGUEIRA LOPES CRUZ</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>cidade_inteira</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Comportamento Político - Qualidade de gestão, eficiência, entrega de serviços</t>
+        </is>
+      </c>
+      <c r="G44" t="n">
+        <v>3</v>
+      </c>
+      <c r="H44" t="n">
+        <v>10</v>
+      </c>
+      <c r="I44" t="n">
+        <v>5536</v>
+      </c>
+      <c r="J44" t="n">
+        <v>21946</v>
+      </c>
+      <c r="K44" t="n">
+        <v>252.255536316413</v>
+      </c>
+      <c r="L44" t="n">
+        <v>31.45990793885322</v>
+      </c>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>votos por mil</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>salto</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>ROGERIO NOGUEIRA LOPES CRUZ</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>cidade_inteira</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Comportamento Político - Qualidade de gestão, eficiência, entrega de serviços</t>
+        </is>
+      </c>
+      <c r="G45" t="n">
+        <v>4</v>
+      </c>
+      <c r="H45" t="n">
+        <v>5</v>
+      </c>
+      <c r="I45" t="n">
+        <v>1696</v>
+      </c>
+      <c r="J45" t="n">
+        <v>7079</v>
+      </c>
+      <c r="K45" t="n">
+        <v>239.5818618448934</v>
+      </c>
+      <c r="L45" t="n">
+        <v>9.638006478376997</v>
+      </c>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>votos por mil</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>salto</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>ROGERIO NOGUEIRA LOPES CRUZ</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>cidade_inteira</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Mobilidade e Acessibilidade - Transporte, calçadas, acesso a serviços, mobilidade</t>
+        </is>
+      </c>
+      <c r="G46" t="n">
+        <v>1</v>
+      </c>
+      <c r="H46" t="n">
+        <v>11</v>
+      </c>
+      <c r="I46" t="n">
+        <v>4983</v>
+      </c>
+      <c r="J46" t="n">
+        <v>22743</v>
+      </c>
+      <c r="K46" t="n">
+        <v>219.1003825352856</v>
+      </c>
+      <c r="L46" t="n">
+        <v>28.31732681707109</v>
+      </c>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>votos por mil</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>salto</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>ROGERIO NOGUEIRA LOPES CRUZ</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>cidade_inteira</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Mobilidade e Acessibilidade - Transporte, calçadas, acesso a serviços, mobilidade</t>
+        </is>
+      </c>
+      <c r="G47" t="n">
+        <v>2</v>
+      </c>
+      <c r="H47" t="n">
+        <v>7</v>
+      </c>
+      <c r="I47" t="n">
+        <v>4834</v>
+      </c>
+      <c r="J47" t="n">
+        <v>19745</v>
+      </c>
+      <c r="K47" t="n">
+        <v>244.8214737908331</v>
+      </c>
+      <c r="L47" t="n">
+        <v>27.4705915781099</v>
+      </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>votos por mil</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>salto</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>ROGERIO NOGUEIRA LOPES CRUZ</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>cidade_inteira</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Mobilidade e Acessibilidade - Transporte, calçadas, acesso a serviços, mobilidade</t>
+        </is>
+      </c>
+      <c r="G48" t="n">
+        <v>3</v>
+      </c>
+      <c r="H48" t="n">
+        <v>11</v>
+      </c>
+      <c r="I48" t="n">
+        <v>6623</v>
+      </c>
+      <c r="J48" t="n">
+        <v>25785</v>
+      </c>
+      <c r="K48" t="n">
+        <v>256.854760519682</v>
+      </c>
+      <c r="L48" t="n">
+        <v>37.63709723248281</v>
+      </c>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>votos por mil</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>salto</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>ROGERIO NOGUEIRA LOPES CRUZ</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>cidade_inteira</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Mobilidade e Acessibilidade - Transporte, calçadas, acesso a serviços, mobilidade</t>
+        </is>
+      </c>
+      <c r="G49" t="n">
+        <v>4</v>
+      </c>
+      <c r="H49" t="n">
+        <v>3</v>
+      </c>
+      <c r="I49" t="n">
+        <v>1157</v>
+      </c>
+      <c r="J49" t="n">
+        <v>4902</v>
+      </c>
+      <c r="K49" t="n">
+        <v>236.0261117911057</v>
+      </c>
+      <c r="L49" t="n">
+        <v>6.574984372336194</v>
+      </c>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>votos por mil</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>salto</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>ROGERIO NOGUEIRA LOPES CRUZ</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>cidade_inteira</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Proteção Animal - Proteção animal, bem-estar, resgate, políticas pets</t>
+        </is>
+      </c>
+      <c r="G50" t="n">
+        <v>1</v>
+      </c>
+      <c r="H50" t="n">
+        <v>8</v>
+      </c>
+      <c r="I50" t="n">
+        <v>5330</v>
+      </c>
+      <c r="J50" t="n">
+        <v>21963</v>
+      </c>
+      <c r="K50" t="n">
+        <v>242.6808723762692</v>
+      </c>
+      <c r="L50" t="n">
+        <v>30.28925385008808</v>
+      </c>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>votos por mil</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>salto</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>ROGERIO NOGUEIRA LOPES CRUZ</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>cidade_inteira</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Proteção Animal - Proteção animal, bem-estar, resgate, políticas pets</t>
+        </is>
+      </c>
+      <c r="G51" t="n">
+        <v>2</v>
+      </c>
+      <c r="H51" t="n">
+        <v>10</v>
+      </c>
+      <c r="I51" t="n">
+        <v>5165</v>
+      </c>
+      <c r="J51" t="n">
+        <v>22551</v>
+      </c>
+      <c r="K51" t="n">
+        <v>229.0364063677886</v>
+      </c>
+      <c r="L51" t="n">
+        <v>29.35159402170824</v>
+      </c>
+      <c r="M51" t="inlineStr">
+        <is>
+          <t>votos por mil</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>salto</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>ROGERIO NOGUEIRA LOPES CRUZ</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>cidade_inteira</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>Proteção Animal - Proteção animal, bem-estar, resgate, políticas pets</t>
+        </is>
+      </c>
+      <c r="G52" t="n">
+        <v>3</v>
+      </c>
+      <c r="H52" t="n">
+        <v>8</v>
+      </c>
+      <c r="I52" t="n">
+        <v>3371</v>
+      </c>
+      <c r="J52" t="n">
+        <v>13580</v>
+      </c>
+      <c r="K52" t="n">
+        <v>248.2326951399116</v>
+      </c>
+      <c r="L52" t="n">
+        <v>19.15667443314201</v>
+      </c>
+      <c r="M52" t="inlineStr">
+        <is>
+          <t>votos por mil</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>salto</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>ROGERIO NOGUEIRA LOPES CRUZ</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>cidade_inteira</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>Proteção Animal - Proteção animal, bem-estar, resgate, políticas pets</t>
+        </is>
+      </c>
+      <c r="G53" t="n">
+        <v>4</v>
+      </c>
+      <c r="H53" t="n">
+        <v>6</v>
+      </c>
+      <c r="I53" t="n">
+        <v>3731</v>
+      </c>
+      <c r="J53" t="n">
+        <v>15081</v>
+      </c>
+      <c r="K53" t="n">
+        <v>247.3973874411511</v>
+      </c>
+      <c r="L53" t="n">
+        <v>21.20247769506166</v>
+      </c>
+      <c r="M53" t="inlineStr">
+        <is>
+          <t>votos por mil</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>salto</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>ROGERIO NOGUEIRA LOPES CRUZ</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>cidade_inteira</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>Saúde - UBS, consultas, exames básicos, acesso SUS</t>
+        </is>
+      </c>
+      <c r="G54" t="n">
+        <v>1</v>
+      </c>
+      <c r="H54" t="n">
+        <v>10</v>
+      </c>
+      <c r="I54" t="n">
+        <v>5411</v>
+      </c>
+      <c r="J54" t="n">
+        <v>24471</v>
+      </c>
+      <c r="K54" t="n">
+        <v>221.1188754035389</v>
+      </c>
+      <c r="L54" t="n">
+        <v>30.74955958402</v>
+      </c>
+      <c r="M54" t="inlineStr">
+        <is>
+          <t>votos por mil</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>salto</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>ROGERIO NOGUEIRA LOPES CRUZ</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>cidade_inteira</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>Saúde - UBS, consultas, exames básicos, acesso SUS</t>
+        </is>
+      </c>
+      <c r="G55" t="n">
+        <v>2</v>
+      </c>
+      <c r="H55" t="n">
+        <v>8</v>
+      </c>
+      <c r="I55" t="n">
+        <v>4640</v>
+      </c>
+      <c r="J55" t="n">
+        <v>17952</v>
+      </c>
+      <c r="K55" t="n">
+        <v>258.4670231729056</v>
+      </c>
+      <c r="L55" t="n">
+        <v>26.36813093140876</v>
+      </c>
+      <c r="M55" t="inlineStr">
+        <is>
+          <t>votos por mil</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>salto</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>ROGERIO NOGUEIRA LOPES CRUZ</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>cidade_inteira</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>Saúde - UBS, consultas, exames básicos, acesso SUS</t>
+        </is>
+      </c>
+      <c r="G56" t="n">
+        <v>3</v>
+      </c>
+      <c r="H56" t="n">
+        <v>5</v>
+      </c>
+      <c r="I56" t="n">
+        <v>3492</v>
+      </c>
+      <c r="J56" t="n">
+        <v>13858</v>
+      </c>
+      <c r="K56" t="n">
+        <v>251.9844133352576</v>
+      </c>
+      <c r="L56" t="n">
+        <v>19.84429164062056</v>
+      </c>
+      <c r="M56" t="inlineStr">
+        <is>
+          <t>votos por mil</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>salto</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>ROGERIO NOGUEIRA LOPES CRUZ</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>cidade_inteira</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>Saúde - UBS, consultas, exames básicos, acesso SUS</t>
+        </is>
+      </c>
+      <c r="G57" t="n">
+        <v>4</v>
+      </c>
+      <c r="H57" t="n">
         <v>9</v>
       </c>
-      <c r="I41" t="n">
+      <c r="I57" t="n">
         <v>4054</v>
       </c>
-      <c r="J41" t="n">
+      <c r="J57" t="n">
         <v>16894</v>
       </c>
-      <c r="K41" t="n">
+      <c r="K57" t="n">
         <v>239.9668521368533</v>
       </c>
-      <c r="L41" t="n">
+      <c r="L57" t="n">
         <v>23.03801784395067</v>
       </c>
-      <c r="M41" t="inlineStr">
+      <c r="M57" t="inlineStr">
         <is>
           <t>votos por mil</t>
         </is>

</xml_diff>

<commit_message>
Publica mapas XG-AE mapa_aderencia 2026-07-02 16:42:09
</commit_message>
<xml_diff>
--- a/mapas2/mapa_aderencia_xg_aderencia_eleitoral.xlsx
+++ b/mapas2/mapa_aderencia_xg_aderencia_eleitoral.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z15"/>
+  <dimension ref="A1:Z11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -816,14 +816,14 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Comportamento Político - Qualidade de gestão, eficiência, entrega de serviços</t>
+          <t>Mobilidade e Acessibilidade - Transporte, calçadas, acesso a serviços, mobilidade</t>
         </is>
       </c>
       <c r="I4" t="n">
         <v>3</v>
       </c>
       <c r="J4" t="n">
-        <v>42.73191145739839</v>
+        <v>34.71562985569617</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
@@ -831,22 +831,22 @@
         </is>
       </c>
       <c r="L4" t="n">
-        <v>-0.2353698816227315</v>
+        <v>-0.2866156217134576</v>
       </c>
       <c r="M4" t="n">
-        <v>38.23150591886343</v>
+        <v>35.66921891432712</v>
       </c>
       <c r="N4" t="n">
-        <v>1.030677011112459</v>
+        <v>0.6232086443536621</v>
       </c>
       <c r="O4" t="n">
-        <v>51.08980745753475</v>
+        <v>32.94467874681013</v>
       </c>
       <c r="P4" t="n">
         <v>50.32344697494485</v>
       </c>
       <c r="Q4" t="n">
-        <v>51.86721991701245</v>
+        <v>31.36200716845878</v>
       </c>
       <c r="R4" t="inlineStr">
         <is>
@@ -877,12 +877,12 @@
       </c>
       <c r="Y4" t="inlineStr">
         <is>
-          <t>C:\Users\guilh\Trabalho\Relatórios Alisson\Documentos gerais\Git\2\dataquadri\mapas2\mapa_aderencia_rogerio_itu_sp_2022_comportamento_politico_qualidade_de_gestao_eficiencia_entrega_de_servicos_cidade_inteira.html</t>
+          <t>C:\Users\guilh\Trabalho\Relatórios Alisson\Documentos gerais\Git\2\dataquadri\mapas2\mapa_aderencia_rogerio_itu_sp_2022_mobilidade_e_acessibilidade_transporte_calcadas_acesso_a_servicos_mobilidade_cidade_inteira.html</t>
         </is>
       </c>
       <c r="Z4" t="inlineStr">
         <is>
-          <t>https://quadrifygit.github.io/dataquadri/mapas2/mapa_aderencia_rogerio_itu_sp_2022_comportamento_politico_qualidade_de_gestao_eficiencia_entrega_de_servicos_cidade_inteira.html</t>
+          <t>https://quadrifygit.github.io/dataquadri/mapas2/mapa_aderencia_rogerio_itu_sp_2022_mobilidade_e_acessibilidade_transporte_calcadas_acesso_a_servicos_mobilidade_cidade_inteira.html</t>
         </is>
       </c>
     </row>
@@ -924,37 +924,37 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Bem-Estar e Serviços - Busca por qualidade de vida, serviços, lazer</t>
+          <t>Saúde - UBS, consultas, exames básicos, acesso SUS</t>
         </is>
       </c>
       <c r="I5" t="n">
         <v>4</v>
       </c>
       <c r="J5" t="n">
-        <v>36.72918203727596</v>
+        <v>28.76619148168748</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Relação inversa moderada</t>
+          <t>Forte relação inversa</t>
         </is>
       </c>
       <c r="L5" t="n">
-        <v>-0.3321960036031988</v>
+        <v>-0.5567502013876867</v>
       </c>
       <c r="M5" t="n">
-        <v>33.39019981984006</v>
+        <v>22.16248993061566</v>
       </c>
       <c r="N5" t="n">
-        <v>0.821997528058819</v>
+        <v>0.7798174513384127</v>
       </c>
       <c r="O5" t="n">
-        <v>42.93014901251406</v>
+        <v>41.03020864796372</v>
       </c>
       <c r="P5" t="n">
         <v>50.32344697494485</v>
       </c>
       <c r="Q5" t="n">
-        <v>41.36574901680372</v>
+        <v>39.24310216256525</v>
       </c>
       <c r="R5" t="inlineStr">
         <is>
@@ -985,12 +985,12 @@
       </c>
       <c r="Y5" t="inlineStr">
         <is>
-          <t>C:\Users\guilh\Trabalho\Relatórios Alisson\Documentos gerais\Git\2\dataquadri\mapas2\mapa_aderencia_rogerio_itu_sp_2022_bem_estar_e_servicos_busca_por_qualidade_de_vida_servicos_lazer_cidade_inteira.html</t>
+          <t>C:\Users\guilh\Trabalho\Relatórios Alisson\Documentos gerais\Git\2\dataquadri\mapas2\mapa_aderencia_rogerio_itu_sp_2022_saude_ubs_consultas_exames_basicos_acesso_sus_cidade_inteira.html</t>
         </is>
       </c>
       <c r="Z5" t="inlineStr">
         <is>
-          <t>https://quadrifygit.github.io/dataquadri/mapas2/mapa_aderencia_rogerio_itu_sp_2022_bem_estar_e_servicos_busca_por_qualidade_de_vida_servicos_lazer_cidade_inteira.html</t>
+          <t>https://quadrifygit.github.io/dataquadri/mapas2/mapa_aderencia_rogerio_itu_sp_2022_saude_ubs_consultas_exames_basicos_acesso_sus_cidade_inteira.html</t>
         </is>
       </c>
     </row>
@@ -1032,37 +1032,37 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Mobilidade e Acessibilidade - Transporte, calçadas, acesso a serviços, mobilidade</t>
+          <t>Assistência Social - Proteção social, seguridade, assistência, rede pública</t>
         </is>
       </c>
       <c r="I6" t="n">
         <v>5</v>
       </c>
       <c r="J6" t="n">
-        <v>34.71562985569617</v>
+        <v>28.69923724840312</v>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Relação inversa moderada</t>
+          <t>Forte relação inversa</t>
         </is>
       </c>
       <c r="L6" t="n">
-        <v>-0.2866156217134576</v>
+        <v>-0.5588103316425902</v>
       </c>
       <c r="M6" t="n">
-        <v>35.66921891432712</v>
+        <v>22.05948341787049</v>
       </c>
       <c r="N6" t="n">
-        <v>0.6232086443536621</v>
+        <v>0.7798174513384127</v>
       </c>
       <c r="O6" t="n">
-        <v>32.94467874681013</v>
+        <v>41.03020864796372</v>
       </c>
       <c r="P6" t="n">
         <v>50.32344697494485</v>
       </c>
       <c r="Q6" t="n">
-        <v>31.36200716845878</v>
+        <v>39.24310216256525</v>
       </c>
       <c r="R6" t="inlineStr">
         <is>
@@ -1093,12 +1093,12 @@
       </c>
       <c r="Y6" t="inlineStr">
         <is>
-          <t>C:\Users\guilh\Trabalho\Relatórios Alisson\Documentos gerais\Git\2\dataquadri\mapas2\mapa_aderencia_rogerio_itu_sp_2022_mobilidade_e_acessibilidade_transporte_calcadas_acesso_a_servicos_mobilidade_cidade_inteira.html</t>
+          <t>C:\Users\guilh\Trabalho\Relatórios Alisson\Documentos gerais\Git\2\dataquadri\mapas2\mapa_aderencia_rogerio_itu_sp_2022_assistencia_social_protecao_social_seguridade_assistencia_rede_publica_cidade_inteira.html</t>
         </is>
       </c>
       <c r="Z6" t="inlineStr">
         <is>
-          <t>https://quadrifygit.github.io/dataquadri/mapas2/mapa_aderencia_rogerio_itu_sp_2022_mobilidade_e_acessibilidade_transporte_calcadas_acesso_a_servicos_mobilidade_cidade_inteira.html</t>
+          <t>https://quadrifygit.github.io/dataquadri/mapas2/mapa_aderencia_rogerio_itu_sp_2022_assistencia_social_protecao_social_seguridade_assistencia_rede_publica_cidade_inteira.html</t>
         </is>
       </c>
     </row>
@@ -1110,7 +1110,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>itu</t>
+          <t>salto</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1140,37 +1140,37 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Saúde - UBS, consultas, exames básicos, acesso SUS</t>
+          <t>Mobilidade e Acessibilidade - Transporte, calçadas, acesso a serviços, mobilidade</t>
         </is>
       </c>
       <c r="I7" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="J7" t="n">
-        <v>28.76619148168748</v>
+        <v>63.30874465234245</v>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Forte relação inversa</t>
+          <t>Aderência positiva moderada</t>
         </is>
       </c>
       <c r="L7" t="n">
-        <v>-0.5567502013876867</v>
+        <v>0.4167583705219454</v>
       </c>
       <c r="M7" t="n">
-        <v>22.16248993061566</v>
+        <v>70.83791852609727</v>
       </c>
       <c r="N7" t="n">
-        <v>0.7798174513384127</v>
+        <v>0.9814860902605079</v>
       </c>
       <c r="O7" t="n">
-        <v>41.03020864796372</v>
+        <v>49.32599317251208</v>
       </c>
       <c r="P7" t="n">
-        <v>50.32344697494485</v>
+        <v>240.4783054321831</v>
       </c>
       <c r="Q7" t="n">
-        <v>39.24310216256525</v>
+        <v>236.0261117911057</v>
       </c>
       <c r="R7" t="inlineStr">
         <is>
@@ -1178,10 +1178,10 @@
         </is>
       </c>
       <c r="S7" t="n">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="T7" t="n">
-        <v>4722</v>
+        <v>17597</v>
       </c>
       <c r="U7" t="n">
         <v>0</v>
@@ -1201,12 +1201,12 @@
       </c>
       <c r="Y7" t="inlineStr">
         <is>
-          <t>C:\Users\guilh\Trabalho\Relatórios Alisson\Documentos gerais\Git\2\dataquadri\mapas2\mapa_aderencia_rogerio_itu_sp_2022_saude_ubs_consultas_exames_basicos_acesso_sus_cidade_inteira.html</t>
+          <t>C:\Users\guilh\Trabalho\Relatórios Alisson\Documentos gerais\Git\2\dataquadri\mapas2\mapa_aderencia_rogerio_salto_sp_2022_mobilidade_e_acessibilidade_transporte_calcadas_acesso_a_servicos_mobilidade_cidade_inteira.html</t>
         </is>
       </c>
       <c r="Z7" t="inlineStr">
         <is>
-          <t>https://quadrifygit.github.io/dataquadri/mapas2/mapa_aderencia_rogerio_itu_sp_2022_saude_ubs_consultas_exames_basicos_acesso_sus_cidade_inteira.html</t>
+          <t>https://quadrifygit.github.io/dataquadri/mapas2/mapa_aderencia_rogerio_salto_sp_2022_mobilidade_e_acessibilidade_transporte_calcadas_acesso_a_servicos_mobilidade_cidade_inteira.html</t>
         </is>
       </c>
     </row>
@@ -1218,7 +1218,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>itu</t>
+          <t>salto</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1252,33 +1252,33 @@
         </is>
       </c>
       <c r="I8" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="J8" t="n">
-        <v>28.69923724840312</v>
+        <v>60.40720914054178</v>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>Forte relação inversa</t>
+          <t>Aderência positiva moderada</t>
         </is>
       </c>
       <c r="L8" t="n">
-        <v>-0.5588103316425902</v>
+        <v>0.321048793129752</v>
       </c>
       <c r="M8" t="n">
-        <v>22.05948341787049</v>
+        <v>66.05243965648761</v>
       </c>
       <c r="N8" t="n">
-        <v>0.7798174513384127</v>
+        <v>0.9978731832195397</v>
       </c>
       <c r="O8" t="n">
-        <v>41.03020864796372</v>
+        <v>49.9232096109281</v>
       </c>
       <c r="P8" t="n">
-        <v>50.32344697494485</v>
+        <v>240.4783054321831</v>
       </c>
       <c r="Q8" t="n">
-        <v>39.24310216256525</v>
+        <v>239.9668521368533</v>
       </c>
       <c r="R8" t="inlineStr">
         <is>
@@ -1286,10 +1286,10 @@
         </is>
       </c>
       <c r="S8" t="n">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="T8" t="n">
-        <v>4722</v>
+        <v>17597</v>
       </c>
       <c r="U8" t="n">
         <v>0</v>
@@ -1309,12 +1309,12 @@
       </c>
       <c r="Y8" t="inlineStr">
         <is>
-          <t>C:\Users\guilh\Trabalho\Relatórios Alisson\Documentos gerais\Git\2\dataquadri\mapas2\mapa_aderencia_rogerio_itu_sp_2022_assistencia_social_protecao_social_seguridade_assistencia_rede_publica_cidade_inteira.html</t>
+          <t>C:\Users\guilh\Trabalho\Relatórios Alisson\Documentos gerais\Git\2\dataquadri\mapas2\mapa_aderencia_rogerio_salto_sp_2022_assistencia_social_protecao_social_seguridade_assistencia_rede_publica_cidade_inteira.html</t>
         </is>
       </c>
       <c r="Z8" t="inlineStr">
         <is>
-          <t>https://quadrifygit.github.io/dataquadri/mapas2/mapa_aderencia_rogerio_itu_sp_2022_assistencia_social_protecao_social_seguridade_assistencia_rede_publica_cidade_inteira.html</t>
+          <t>https://quadrifygit.github.io/dataquadri/mapas2/mapa_aderencia_rogerio_salto_sp_2022_assistencia_social_protecao_social_seguridade_assistencia_rede_publica_cidade_inteira.html</t>
         </is>
       </c>
     </row>
@@ -1356,14 +1356,14 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Mobilidade e Acessibilidade - Transporte, calçadas, acesso a serviços, mobilidade</t>
+          <t>Saúde - UBS, consultas, exames básicos, acesso SUS</t>
         </is>
       </c>
       <c r="I9" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J9" t="n">
-        <v>63.30874465234245</v>
+        <v>60.29994840725742</v>
       </c>
       <c r="K9" t="inlineStr">
         <is>
@@ -1371,22 +1371,22 @@
         </is>
       </c>
       <c r="L9" t="n">
-        <v>0.4167583705219454</v>
+        <v>0.3177484628748488</v>
       </c>
       <c r="M9" t="n">
-        <v>70.83791852609727</v>
+        <v>65.88742314374244</v>
       </c>
       <c r="N9" t="n">
-        <v>0.9814860902605079</v>
+        <v>0.9978731832195397</v>
       </c>
       <c r="O9" t="n">
-        <v>49.32599317251208</v>
+        <v>49.9232096109281</v>
       </c>
       <c r="P9" t="n">
         <v>240.4783054321831</v>
       </c>
       <c r="Q9" t="n">
-        <v>236.0261117911057</v>
+        <v>239.9668521368533</v>
       </c>
       <c r="R9" t="inlineStr">
         <is>
@@ -1417,12 +1417,12 @@
       </c>
       <c r="Y9" t="inlineStr">
         <is>
-          <t>C:\Users\guilh\Trabalho\Relatórios Alisson\Documentos gerais\Git\2\dataquadri\mapas2\mapa_aderencia_rogerio_salto_sp_2022_mobilidade_e_acessibilidade_transporte_calcadas_acesso_a_servicos_mobilidade_cidade_inteira.html</t>
+          <t>C:\Users\guilh\Trabalho\Relatórios Alisson\Documentos gerais\Git\2\dataquadri\mapas2\mapa_aderencia_rogerio_salto_sp_2022_saude_ubs_consultas_exames_basicos_acesso_sus_cidade_inteira.html</t>
         </is>
       </c>
       <c r="Z9" t="inlineStr">
         <is>
-          <t>https://quadrifygit.github.io/dataquadri/mapas2/mapa_aderencia_rogerio_salto_sp_2022_mobilidade_e_acessibilidade_transporte_calcadas_acesso_a_servicos_mobilidade_cidade_inteira.html</t>
+          <t>https://quadrifygit.github.io/dataquadri/mapas2/mapa_aderencia_rogerio_salto_sp_2022_saude_ubs_consultas_exames_basicos_acesso_sus_cidade_inteira.html</t>
         </is>
       </c>
     </row>
@@ -1464,37 +1464,37 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Bem-Estar e Serviços - Busca por qualidade de vida, serviços, lazer</t>
+          <t>Proteção Animal - Proteção animal, bem-estar, resgate, políticas pets</t>
         </is>
       </c>
       <c r="I10" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J10" t="n">
-        <v>62.58152253016321</v>
+        <v>53.43884739138753</v>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>Aderência positiva moderada</t>
+          <t>Relação fraca ou neutra</t>
         </is>
       </c>
       <c r="L10" t="n">
-        <v>0.3712871536766121</v>
+        <v>0.09479281898805356</v>
       </c>
       <c r="M10" t="n">
-        <v>68.56435768383061</v>
+        <v>54.73964094940268</v>
       </c>
       <c r="N10" t="n">
-        <v>1.041614703086268</v>
+        <v>1.028772167187943</v>
       </c>
       <c r="O10" t="n">
-        <v>51.47054295906663</v>
+        <v>51.02308792650224</v>
       </c>
       <c r="P10" t="n">
         <v>240.4783054321831</v>
       </c>
       <c r="Q10" t="n">
-        <v>250.4857387114324</v>
+        <v>247.3973874411511</v>
       </c>
       <c r="R10" t="inlineStr">
         <is>
@@ -1525,12 +1525,12 @@
       </c>
       <c r="Y10" t="inlineStr">
         <is>
-          <t>C:\Users\guilh\Trabalho\Relatórios Alisson\Documentos gerais\Git\2\dataquadri\mapas2\mapa_aderencia_rogerio_salto_sp_2022_bem_estar_e_servicos_busca_por_qualidade_de_vida_servicos_lazer_cidade_inteira.html</t>
+          <t>C:\Users\guilh\Trabalho\Relatórios Alisson\Documentos gerais\Git\2\dataquadri\mapas2\mapa_aderencia_rogerio_salto_sp_2022_protecao_animal_protecao_animal_bem_estar_resgate_politicas_pets_cidade_inteira.html</t>
         </is>
       </c>
       <c r="Z10" t="inlineStr">
         <is>
-          <t>https://quadrifygit.github.io/dataquadri/mapas2/mapa_aderencia_rogerio_salto_sp_2022_bem_estar_e_servicos_busca_por_qualidade_de_vida_servicos_lazer_cidade_inteira.html</t>
+          <t>https://quadrifygit.github.io/dataquadri/mapas2/mapa_aderencia_rogerio_salto_sp_2022_protecao_animal_protecao_animal_bem_estar_resgate_politicas_pets_cidade_inteira.html</t>
         </is>
       </c>
     </row>
@@ -1572,37 +1572,37 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Assistência Social - Proteção social, seguridade, assistência, rede pública</t>
+          <t>Bem-Estar e Serviços - Qualidade do bairro, serviços, segurança, lazer</t>
         </is>
       </c>
       <c r="I11" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J11" t="n">
-        <v>60.40720914054178</v>
+        <v>51.6473882332125</v>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>Aderência positiva moderada</t>
+          <t>Relação fraca ou neutra</t>
         </is>
       </c>
       <c r="L11" t="n">
-        <v>0.321048793129752</v>
+        <v>0.05592226265252676</v>
       </c>
       <c r="M11" t="n">
-        <v>66.05243965648761</v>
+        <v>52.79611313262635</v>
       </c>
       <c r="N11" t="n">
-        <v>0.9978731832195397</v>
+        <v>0.9866167459431195</v>
       </c>
       <c r="O11" t="n">
-        <v>49.9232096109281</v>
+        <v>49.51404199144392</v>
       </c>
       <c r="P11" t="n">
         <v>240.4783054321831</v>
       </c>
       <c r="Q11" t="n">
-        <v>239.9668521368533</v>
+        <v>237.2599231754161</v>
       </c>
       <c r="R11" t="inlineStr">
         <is>
@@ -1633,442 +1633,10 @@
       </c>
       <c r="Y11" t="inlineStr">
         <is>
-          <t>C:\Users\guilh\Trabalho\Relatórios Alisson\Documentos gerais\Git\2\dataquadri\mapas2\mapa_aderencia_rogerio_salto_sp_2022_assistencia_social_protecao_social_seguridade_assistencia_rede_publica_cidade_inteira.html</t>
+          <t>C:\Users\guilh\Trabalho\Relatórios Alisson\Documentos gerais\Git\2\dataquadri\mapas2\mapa_aderencia_rogerio_salto_sp_2022_bem_estar_e_servicos_qualidade_do_bairro_servicos_seguranca_lazer_cidade_inteira.html</t>
         </is>
       </c>
       <c r="Z11" t="inlineStr">
-        <is>
-          <t>https://quadrifygit.github.io/dataquadri/mapas2/mapa_aderencia_rogerio_salto_sp_2022_assistencia_social_protecao_social_seguridade_assistencia_rede_publica_cidade_inteira.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>SP</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>salto</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>2022</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>ROGERIO NOGUEIRA LOPES CRUZ</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>DEPUTADO ESTADUAL</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>cidade_inteira</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>Saúde - UBS, consultas, exames básicos, acesso SUS</t>
-        </is>
-      </c>
-      <c r="I12" t="n">
-        <v>4</v>
-      </c>
-      <c r="J12" t="n">
-        <v>60.29994840725742</v>
-      </c>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>Aderência positiva moderada</t>
-        </is>
-      </c>
-      <c r="L12" t="n">
-        <v>0.3177484628748488</v>
-      </c>
-      <c r="M12" t="n">
-        <v>65.88742314374244</v>
-      </c>
-      <c r="N12" t="n">
-        <v>0.9978731832195397</v>
-      </c>
-      <c r="O12" t="n">
-        <v>49.9232096109281</v>
-      </c>
-      <c r="P12" t="n">
-        <v>240.4783054321831</v>
-      </c>
-      <c r="Q12" t="n">
-        <v>239.9668521368533</v>
-      </c>
-      <c r="R12" t="inlineStr">
-        <is>
-          <t>votos por mil</t>
-        </is>
-      </c>
-      <c r="S12" t="n">
-        <v>32</v>
-      </c>
-      <c r="T12" t="n">
-        <v>17597</v>
-      </c>
-      <c r="U12" t="n">
-        <v>0</v>
-      </c>
-      <c r="V12" t="inlineStr">
-        <is>
-          <t>Alta</t>
-        </is>
-      </c>
-      <c r="W12" t="inlineStr">
-        <is>
-          <t>Total de votos do cargo/turno no local</t>
-        </is>
-      </c>
-      <c r="X12" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y12" t="inlineStr">
-        <is>
-          <t>C:\Users\guilh\Trabalho\Relatórios Alisson\Documentos gerais\Git\2\dataquadri\mapas2\mapa_aderencia_rogerio_salto_sp_2022_saude_ubs_consultas_exames_basicos_acesso_sus_cidade_inteira.html</t>
-        </is>
-      </c>
-      <c r="Z12" t="inlineStr">
-        <is>
-          <t>https://quadrifygit.github.io/dataquadri/mapas2/mapa_aderencia_rogerio_salto_sp_2022_saude_ubs_consultas_exames_basicos_acesso_sus_cidade_inteira.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>SP</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>salto</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>2022</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>ROGERIO NOGUEIRA LOPES CRUZ</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>DEPUTADO ESTADUAL</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>cidade_inteira</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>Comportamento Político - Qualidade de gestão, eficiência, entrega de serviços</t>
-        </is>
-      </c>
-      <c r="I13" t="n">
-        <v>5</v>
-      </c>
-      <c r="J13" t="n">
-        <v>55.6793858563519</v>
-      </c>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>Relação fraca ou neutra</t>
-        </is>
-      </c>
-      <c r="L13" t="n">
-        <v>0.1762009652756663</v>
-      </c>
-      <c r="M13" t="n">
-        <v>58.81004826378331</v>
-      </c>
-      <c r="N13" t="n">
-        <v>0.9962722475706126</v>
-      </c>
-      <c r="O13" t="n">
-        <v>49.86529852826499</v>
-      </c>
-      <c r="P13" t="n">
-        <v>240.4783054321831</v>
-      </c>
-      <c r="Q13" t="n">
-        <v>239.5818618448934</v>
-      </c>
-      <c r="R13" t="inlineStr">
-        <is>
-          <t>votos por mil</t>
-        </is>
-      </c>
-      <c r="S13" t="n">
-        <v>32</v>
-      </c>
-      <c r="T13" t="n">
-        <v>17597</v>
-      </c>
-      <c r="U13" t="n">
-        <v>0</v>
-      </c>
-      <c r="V13" t="inlineStr">
-        <is>
-          <t>Alta</t>
-        </is>
-      </c>
-      <c r="W13" t="inlineStr">
-        <is>
-          <t>Total de votos do cargo/turno no local</t>
-        </is>
-      </c>
-      <c r="X13" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y13" t="inlineStr">
-        <is>
-          <t>C:\Users\guilh\Trabalho\Relatórios Alisson\Documentos gerais\Git\2\dataquadri\mapas2\mapa_aderencia_rogerio_salto_sp_2022_comportamento_politico_qualidade_de_gestao_eficiencia_entrega_de_servicos_cidade_inteira.html</t>
-        </is>
-      </c>
-      <c r="Z13" t="inlineStr">
-        <is>
-          <t>https://quadrifygit.github.io/dataquadri/mapas2/mapa_aderencia_rogerio_salto_sp_2022_comportamento_politico_qualidade_de_gestao_eficiencia_entrega_de_servicos_cidade_inteira.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>SP</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>salto</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>2022</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>ROGERIO NOGUEIRA LOPES CRUZ</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>DEPUTADO ESTADUAL</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>cidade_inteira</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>Proteção Animal - Proteção animal, bem-estar, resgate, políticas pets</t>
-        </is>
-      </c>
-      <c r="I14" t="n">
-        <v>6</v>
-      </c>
-      <c r="J14" t="n">
-        <v>53.43884739138753</v>
-      </c>
-      <c r="K14" t="inlineStr">
-        <is>
-          <t>Relação fraca ou neutra</t>
-        </is>
-      </c>
-      <c r="L14" t="n">
-        <v>0.09479281898805356</v>
-      </c>
-      <c r="M14" t="n">
-        <v>54.73964094940268</v>
-      </c>
-      <c r="N14" t="n">
-        <v>1.028772167187943</v>
-      </c>
-      <c r="O14" t="n">
-        <v>51.02308792650224</v>
-      </c>
-      <c r="P14" t="n">
-        <v>240.4783054321831</v>
-      </c>
-      <c r="Q14" t="n">
-        <v>247.3973874411511</v>
-      </c>
-      <c r="R14" t="inlineStr">
-        <is>
-          <t>votos por mil</t>
-        </is>
-      </c>
-      <c r="S14" t="n">
-        <v>32</v>
-      </c>
-      <c r="T14" t="n">
-        <v>17597</v>
-      </c>
-      <c r="U14" t="n">
-        <v>0</v>
-      </c>
-      <c r="V14" t="inlineStr">
-        <is>
-          <t>Alta</t>
-        </is>
-      </c>
-      <c r="W14" t="inlineStr">
-        <is>
-          <t>Total de votos do cargo/turno no local</t>
-        </is>
-      </c>
-      <c r="X14" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y14" t="inlineStr">
-        <is>
-          <t>C:\Users\guilh\Trabalho\Relatórios Alisson\Documentos gerais\Git\2\dataquadri\mapas2\mapa_aderencia_rogerio_salto_sp_2022_protecao_animal_protecao_animal_bem_estar_resgate_politicas_pets_cidade_inteira.html</t>
-        </is>
-      </c>
-      <c r="Z14" t="inlineStr">
-        <is>
-          <t>https://quadrifygit.github.io/dataquadri/mapas2/mapa_aderencia_rogerio_salto_sp_2022_protecao_animal_protecao_animal_bem_estar_resgate_politicas_pets_cidade_inteira.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>SP</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>salto</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>2022</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>ROGERIO NOGUEIRA LOPES CRUZ</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>DEPUTADO ESTADUAL</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>cidade_inteira</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>Bem-Estar e Serviços - Qualidade do bairro, serviços, segurança, lazer</t>
-        </is>
-      </c>
-      <c r="I15" t="n">
-        <v>7</v>
-      </c>
-      <c r="J15" t="n">
-        <v>51.6473882332125</v>
-      </c>
-      <c r="K15" t="inlineStr">
-        <is>
-          <t>Relação fraca ou neutra</t>
-        </is>
-      </c>
-      <c r="L15" t="n">
-        <v>0.05592226265252676</v>
-      </c>
-      <c r="M15" t="n">
-        <v>52.79611313262635</v>
-      </c>
-      <c r="N15" t="n">
-        <v>0.9866167459431195</v>
-      </c>
-      <c r="O15" t="n">
-        <v>49.51404199144392</v>
-      </c>
-      <c r="P15" t="n">
-        <v>240.4783054321831</v>
-      </c>
-      <c r="Q15" t="n">
-        <v>237.2599231754161</v>
-      </c>
-      <c r="R15" t="inlineStr">
-        <is>
-          <t>votos por mil</t>
-        </is>
-      </c>
-      <c r="S15" t="n">
-        <v>32</v>
-      </c>
-      <c r="T15" t="n">
-        <v>17597</v>
-      </c>
-      <c r="U15" t="n">
-        <v>0</v>
-      </c>
-      <c r="V15" t="inlineStr">
-        <is>
-          <t>Alta</t>
-        </is>
-      </c>
-      <c r="W15" t="inlineStr">
-        <is>
-          <t>Total de votos do cargo/turno no local</t>
-        </is>
-      </c>
-      <c r="X15" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y15" t="inlineStr">
-        <is>
-          <t>C:\Users\guilh\Trabalho\Relatórios Alisson\Documentos gerais\Git\2\dataquadri\mapas2\mapa_aderencia_rogerio_salto_sp_2022_bem_estar_e_servicos_qualidade_do_bairro_servicos_seguranca_lazer_cidade_inteira.html</t>
-        </is>
-      </c>
-      <c r="Z15" t="inlineStr">
         <is>
           <t>https://quadrifygit.github.io/dataquadri/mapas2/mapa_aderencia_rogerio_salto_sp_2022_bem_estar_e_servicos_qualidade_do_bairro_servicos_seguranca_lazer_cidade_inteira.html</t>
         </is>
@@ -2085,7 +1653,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M57"/>
+  <dimension ref="A1:M41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2403,26 +1971,26 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Bem-Estar e Serviços - Busca por qualidade de vida, serviços, lazer</t>
+          <t>Bem-Estar e Serviços - Qualidade do bairro, serviços, segurança, lazer</t>
         </is>
       </c>
       <c r="G6" t="n">
         <v>1</v>
       </c>
       <c r="H6" t="n">
+        <v>1</v>
+      </c>
+      <c r="I6" t="n">
         <v>13</v>
       </c>
-      <c r="I6" t="n">
-        <v>2175</v>
-      </c>
       <c r="J6" t="n">
-        <v>40684</v>
+        <v>251</v>
       </c>
       <c r="K6" t="n">
-        <v>53.46081997836988</v>
+        <v>51.79282868525897</v>
       </c>
       <c r="L6" t="n">
-        <v>46.06099110546379</v>
+        <v>0.2753070732740364</v>
       </c>
       <c r="M6" t="inlineStr">
         <is>
@@ -2458,26 +2026,26 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Bem-Estar e Serviços - Busca por qualidade de vida, serviços, lazer</t>
+          <t>Bem-Estar e Serviços - Qualidade do bairro, serviços, segurança, lazer</t>
         </is>
       </c>
       <c r="G7" t="n">
         <v>2</v>
       </c>
       <c r="H7" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="I7" t="n">
-        <v>814</v>
+        <v>869</v>
       </c>
       <c r="J7" t="n">
-        <v>13655</v>
+        <v>22532</v>
       </c>
       <c r="K7" t="n">
-        <v>59.61186378615891</v>
+        <v>38.56737085034617</v>
       </c>
       <c r="L7" t="n">
-        <v>17.23845828038966</v>
+        <v>18.40321897501059</v>
       </c>
       <c r="M7" t="inlineStr">
         <is>
@@ -2513,26 +2081,26 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Bem-Estar e Serviços - Busca por qualidade de vida, serviços, lazer</t>
+          <t>Bem-Estar e Serviços - Qualidade do bairro, serviços, segurança, lazer</t>
         </is>
       </c>
       <c r="G8" t="n">
         <v>3</v>
       </c>
       <c r="H8" t="n">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="I8" t="n">
-        <v>576</v>
+        <v>2809</v>
       </c>
       <c r="J8" t="n">
-        <v>11524</v>
+        <v>52204</v>
       </c>
       <c r="K8" t="n">
-        <v>49.98264491496008</v>
+        <v>53.80813730748601</v>
       </c>
       <c r="L8" t="n">
-        <v>12.19822109275731</v>
+        <v>59.48750529436679</v>
       </c>
       <c r="M8" t="inlineStr">
         <is>
@@ -2568,26 +2136,26 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Bem-Estar e Serviços - Busca por qualidade de vida, serviços, lazer</t>
+          <t>Bem-Estar e Serviços - Qualidade do bairro, serviços, segurança, lazer</t>
         </is>
       </c>
       <c r="G9" t="n">
         <v>4</v>
       </c>
       <c r="H9" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="I9" t="n">
-        <v>1157</v>
+        <v>1031</v>
       </c>
       <c r="J9" t="n">
-        <v>27970</v>
+        <v>18846</v>
       </c>
       <c r="K9" t="n">
-        <v>41.36574901680372</v>
+        <v>54.7065690332166</v>
       </c>
       <c r="L9" t="n">
-        <v>24.50232952138924</v>
+        <v>21.83396865734858</v>
       </c>
       <c r="M9" t="inlineStr">
         <is>
@@ -2623,26 +2191,26 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Bem-Estar e Serviços - Qualidade do bairro, serviços, segurança, lazer</t>
+          <t>Mobilidade e Acessibilidade - Transporte, calçadas, acesso a serviços, mobilidade</t>
         </is>
       </c>
       <c r="G10" t="n">
         <v>1</v>
       </c>
       <c r="H10" t="n">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="I10" t="n">
-        <v>13</v>
+        <v>2149</v>
       </c>
       <c r="J10" t="n">
-        <v>251</v>
+        <v>40283</v>
       </c>
       <c r="K10" t="n">
-        <v>51.79282868525897</v>
+        <v>53.3475659707569</v>
       </c>
       <c r="L10" t="n">
-        <v>0.2753070732740364</v>
+        <v>45.51037695891571</v>
       </c>
       <c r="M10" t="inlineStr">
         <is>
@@ -2678,26 +2246,26 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Bem-Estar e Serviços - Qualidade do bairro, serviços, segurança, lazer</t>
+          <t>Mobilidade e Acessibilidade - Transporte, calçadas, acesso a serviços, mobilidade</t>
         </is>
       </c>
       <c r="G11" t="n">
         <v>2</v>
       </c>
       <c r="H11" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="I11" t="n">
-        <v>869</v>
+        <v>1154</v>
       </c>
       <c r="J11" t="n">
-        <v>22532</v>
+        <v>20731</v>
       </c>
       <c r="K11" t="n">
-        <v>38.56737085034617</v>
+        <v>55.66542858521056</v>
       </c>
       <c r="L11" t="n">
-        <v>18.40321897501059</v>
+        <v>24.43879711986446</v>
       </c>
       <c r="M11" t="inlineStr">
         <is>
@@ -2733,26 +2301,26 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Bem-Estar e Serviços - Qualidade do bairro, serviços, segurança, lazer</t>
+          <t>Mobilidade e Acessibilidade - Transporte, calçadas, acesso a serviços, mobilidade</t>
         </is>
       </c>
       <c r="G12" t="n">
         <v>3</v>
       </c>
       <c r="H12" t="n">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="I12" t="n">
-        <v>2809</v>
+        <v>1314</v>
       </c>
       <c r="J12" t="n">
-        <v>52204</v>
+        <v>29471</v>
       </c>
       <c r="K12" t="n">
-        <v>53.80813730748601</v>
+        <v>44.58620338637983</v>
       </c>
       <c r="L12" t="n">
-        <v>59.48750529436679</v>
+        <v>27.82719186785261</v>
       </c>
       <c r="M12" t="inlineStr">
         <is>
@@ -2788,26 +2356,26 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Bem-Estar e Serviços - Qualidade do bairro, serviços, segurança, lazer</t>
+          <t>Mobilidade e Acessibilidade - Transporte, calçadas, acesso a serviços, mobilidade</t>
         </is>
       </c>
       <c r="G13" t="n">
         <v>4</v>
       </c>
       <c r="H13" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="I13" t="n">
-        <v>1031</v>
+        <v>105</v>
       </c>
       <c r="J13" t="n">
-        <v>18846</v>
+        <v>3348</v>
       </c>
       <c r="K13" t="n">
-        <v>54.7065690332166</v>
+        <v>31.36200716845878</v>
       </c>
       <c r="L13" t="n">
-        <v>21.83396865734858</v>
+        <v>2.223634053367217</v>
       </c>
       <c r="M13" t="inlineStr">
         <is>
@@ -2843,26 +2411,26 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Comportamento Político - Qualidade de gestão, eficiência, entrega de serviços</t>
+          <t>Proteção Animal - Proteção animal, bem-estar, resgate, políticas pets</t>
         </is>
       </c>
       <c r="G14" t="n">
         <v>1</v>
       </c>
       <c r="H14" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="I14" t="n">
-        <v>179</v>
+        <v>1130</v>
       </c>
       <c r="J14" t="n">
-        <v>2311</v>
+        <v>20098</v>
       </c>
       <c r="K14" t="n">
-        <v>77.45564690610125</v>
+        <v>56.2244999502438</v>
       </c>
       <c r="L14" t="n">
-        <v>3.790766624311733</v>
+        <v>23.93053790766625</v>
       </c>
       <c r="M14" t="inlineStr">
         <is>
@@ -2898,26 +2466,26 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Comportamento Político - Qualidade de gestão, eficiência, entrega de serviços</t>
+          <t>Proteção Animal - Proteção animal, bem-estar, resgate, políticas pets</t>
         </is>
       </c>
       <c r="G15" t="n">
         <v>2</v>
       </c>
       <c r="H15" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="I15" t="n">
-        <v>2246</v>
+        <v>904</v>
       </c>
       <c r="J15" t="n">
-        <v>46189</v>
+        <v>18629</v>
       </c>
       <c r="K15" t="n">
-        <v>48.62629630431488</v>
+        <v>48.52649095496269</v>
       </c>
       <c r="L15" t="n">
-        <v>47.56459127488352</v>
+        <v>19.14443032613299</v>
       </c>
       <c r="M15" t="inlineStr">
         <is>
@@ -2953,26 +2521,26 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Comportamento Político - Qualidade de gestão, eficiência, entrega de serviços</t>
+          <t>Proteção Animal - Proteção animal, bem-estar, resgate, políticas pets</t>
         </is>
       </c>
       <c r="G16" t="n">
         <v>3</v>
       </c>
       <c r="H16" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="I16" t="n">
-        <v>1547</v>
+        <v>1531</v>
       </c>
       <c r="J16" t="n">
-        <v>30873</v>
+        <v>34091</v>
       </c>
       <c r="K16" t="n">
-        <v>50.10850905321802</v>
+        <v>44.90921357543046</v>
       </c>
       <c r="L16" t="n">
-        <v>32.76154171961034</v>
+        <v>32.42270224481152</v>
       </c>
       <c r="M16" t="inlineStr">
         <is>
@@ -3008,26 +2576,26 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Comportamento Político - Qualidade de gestão, eficiência, entrega de serviços</t>
+          <t>Proteção Animal - Proteção animal, bem-estar, resgate, políticas pets</t>
         </is>
       </c>
       <c r="G17" t="n">
         <v>4</v>
       </c>
       <c r="H17" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="I17" t="n">
-        <v>750</v>
+        <v>1157</v>
       </c>
       <c r="J17" t="n">
-        <v>14460</v>
+        <v>21015</v>
       </c>
       <c r="K17" t="n">
-        <v>51.86721991701245</v>
+        <v>55.05591244349274</v>
       </c>
       <c r="L17" t="n">
-        <v>15.88310038119441</v>
+        <v>24.50232952138924</v>
       </c>
       <c r="M17" t="inlineStr">
         <is>
@@ -3063,26 +2631,26 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Mobilidade e Acessibilidade - Transporte, calçadas, acesso a serviços, mobilidade</t>
+          <t>Saúde - UBS, consultas, exames básicos, acesso SUS</t>
         </is>
       </c>
       <c r="G18" t="n">
         <v>1</v>
       </c>
       <c r="H18" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="I18" t="n">
-        <v>2149</v>
+        <v>2445</v>
       </c>
       <c r="J18" t="n">
-        <v>40283</v>
+        <v>43069</v>
       </c>
       <c r="K18" t="n">
-        <v>53.3475659707569</v>
+        <v>56.76937008056839</v>
       </c>
       <c r="L18" t="n">
-        <v>45.51037695891571</v>
+        <v>51.77890724269377</v>
       </c>
       <c r="M18" t="inlineStr">
         <is>
@@ -3118,7 +2686,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Mobilidade e Acessibilidade - Transporte, calçadas, acesso a serviços, mobilidade</t>
+          <t>Saúde - UBS, consultas, exames básicos, acesso SUS</t>
         </is>
       </c>
       <c r="G19" t="n">
@@ -3128,16 +2696,16 @@
         <v>8</v>
       </c>
       <c r="I19" t="n">
-        <v>1154</v>
+        <v>966</v>
       </c>
       <c r="J19" t="n">
-        <v>20731</v>
+        <v>18608</v>
       </c>
       <c r="K19" t="n">
-        <v>55.66542858521056</v>
+        <v>51.91315563198624</v>
       </c>
       <c r="L19" t="n">
-        <v>24.43879711986446</v>
+        <v>20.4574332909784</v>
       </c>
       <c r="M19" t="inlineStr">
         <is>
@@ -3173,26 +2741,26 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Mobilidade e Acessibilidade - Transporte, calçadas, acesso a serviços, mobilidade</t>
+          <t>Saúde - UBS, consultas, exames básicos, acesso SUS</t>
         </is>
       </c>
       <c r="G20" t="n">
         <v>3</v>
       </c>
       <c r="H20" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="I20" t="n">
-        <v>1314</v>
+        <v>469</v>
       </c>
       <c r="J20" t="n">
-        <v>29471</v>
+        <v>10700</v>
       </c>
       <c r="K20" t="n">
-        <v>44.58620338637983</v>
+        <v>43.83177570093458</v>
       </c>
       <c r="L20" t="n">
-        <v>27.82719186785261</v>
+        <v>9.932232105040237</v>
       </c>
       <c r="M20" t="inlineStr">
         <is>
@@ -3228,26 +2796,26 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Mobilidade e Acessibilidade - Transporte, calçadas, acesso a serviços, mobilidade</t>
+          <t>Saúde - UBS, consultas, exames básicos, acesso SUS</t>
         </is>
       </c>
       <c r="G21" t="n">
         <v>4</v>
       </c>
       <c r="H21" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="I21" t="n">
-        <v>105</v>
+        <v>842</v>
       </c>
       <c r="J21" t="n">
-        <v>3348</v>
+        <v>21456</v>
       </c>
       <c r="K21" t="n">
-        <v>31.36200716845878</v>
+        <v>39.24310216256525</v>
       </c>
       <c r="L21" t="n">
-        <v>2.223634053367217</v>
+        <v>17.83142736128759</v>
       </c>
       <c r="M21" t="inlineStr">
         <is>
@@ -3263,7 +2831,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>itu</t>
+          <t>salto</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -3283,26 +2851,26 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Proteção Animal - Proteção animal, bem-estar, resgate, políticas pets</t>
+          <t>Assistência Social - Proteção social, seguridade, assistência, rede pública</t>
         </is>
       </c>
       <c r="G22" t="n">
         <v>1</v>
       </c>
       <c r="H22" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="I22" t="n">
-        <v>1130</v>
+        <v>5411</v>
       </c>
       <c r="J22" t="n">
-        <v>20098</v>
+        <v>24471</v>
       </c>
       <c r="K22" t="n">
-        <v>56.2244999502438</v>
+        <v>221.1188754035389</v>
       </c>
       <c r="L22" t="n">
-        <v>23.93053790766625</v>
+        <v>30.74955958402</v>
       </c>
       <c r="M22" t="inlineStr">
         <is>
@@ -3318,7 +2886,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>itu</t>
+          <t>salto</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -3338,7 +2906,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Proteção Animal - Proteção animal, bem-estar, resgate, políticas pets</t>
+          <t>Assistência Social - Proteção social, seguridade, assistência, rede pública</t>
         </is>
       </c>
       <c r="G23" t="n">
@@ -3348,16 +2916,16 @@
         <v>8</v>
       </c>
       <c r="I23" t="n">
-        <v>904</v>
+        <v>4640</v>
       </c>
       <c r="J23" t="n">
-        <v>18629</v>
+        <v>17952</v>
       </c>
       <c r="K23" t="n">
-        <v>48.52649095496269</v>
+        <v>258.4670231729056</v>
       </c>
       <c r="L23" t="n">
-        <v>19.14443032613299</v>
+        <v>26.36813093140876</v>
       </c>
       <c r="M23" t="inlineStr">
         <is>
@@ -3373,7 +2941,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>itu</t>
+          <t>salto</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -3393,26 +2961,26 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Proteção Animal - Proteção animal, bem-estar, resgate, políticas pets</t>
+          <t>Assistência Social - Proteção social, seguridade, assistência, rede pública</t>
         </is>
       </c>
       <c r="G24" t="n">
         <v>3</v>
       </c>
       <c r="H24" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="I24" t="n">
-        <v>1531</v>
+        <v>3492</v>
       </c>
       <c r="J24" t="n">
-        <v>34091</v>
+        <v>13858</v>
       </c>
       <c r="K24" t="n">
-        <v>44.90921357543046</v>
+        <v>251.9844133352576</v>
       </c>
       <c r="L24" t="n">
-        <v>32.42270224481152</v>
+        <v>19.84429164062056</v>
       </c>
       <c r="M24" t="inlineStr">
         <is>
@@ -3428,7 +2996,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>itu</t>
+          <t>salto</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -3448,26 +3016,26 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Proteção Animal - Proteção animal, bem-estar, resgate, políticas pets</t>
+          <t>Assistência Social - Proteção social, seguridade, assistência, rede pública</t>
         </is>
       </c>
       <c r="G25" t="n">
         <v>4</v>
       </c>
       <c r="H25" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="I25" t="n">
-        <v>1157</v>
+        <v>4054</v>
       </c>
       <c r="J25" t="n">
-        <v>21015</v>
+        <v>16894</v>
       </c>
       <c r="K25" t="n">
-        <v>55.05591244349274</v>
+        <v>239.9668521368533</v>
       </c>
       <c r="L25" t="n">
-        <v>24.50232952138924</v>
+        <v>23.03801784395067</v>
       </c>
       <c r="M25" t="inlineStr">
         <is>
@@ -3483,7 +3051,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>itu</t>
+          <t>salto</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -3503,26 +3071,26 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Saúde - UBS, consultas, exames básicos, acesso SUS</t>
+          <t>Bem-Estar e Serviços - Qualidade do bairro, serviços, segurança, lazer</t>
         </is>
       </c>
       <c r="G26" t="n">
         <v>1</v>
       </c>
       <c r="H26" t="n">
-        <v>14</v>
+        <v>5</v>
       </c>
       <c r="I26" t="n">
-        <v>2445</v>
+        <v>4213</v>
       </c>
       <c r="J26" t="n">
-        <v>43069</v>
+        <v>17547</v>
       </c>
       <c r="K26" t="n">
-        <v>56.76937008056839</v>
+        <v>240.0980224539807</v>
       </c>
       <c r="L26" t="n">
-        <v>51.77890724269377</v>
+        <v>23.94158095129852</v>
       </c>
       <c r="M26" t="inlineStr">
         <is>
@@ -3538,7 +3106,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>itu</t>
+          <t>salto</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -3558,26 +3126,26 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Saúde - UBS, consultas, exames básicos, acesso SUS</t>
+          <t>Bem-Estar e Serviços - Qualidade do bairro, serviços, segurança, lazer</t>
         </is>
       </c>
       <c r="G27" t="n">
         <v>2</v>
       </c>
       <c r="H27" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="I27" t="n">
-        <v>966</v>
+        <v>2502</v>
       </c>
       <c r="J27" t="n">
-        <v>18608</v>
+        <v>10764</v>
       </c>
       <c r="K27" t="n">
-        <v>51.91315563198624</v>
+        <v>232.4414715719064</v>
       </c>
       <c r="L27" t="n">
-        <v>20.4574332909784</v>
+        <v>14.21833267034154</v>
       </c>
       <c r="M27" t="inlineStr">
         <is>
@@ -3593,7 +3161,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>itu</t>
+          <t>salto</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -3613,26 +3181,26 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Saúde - UBS, consultas, exames básicos, acesso SUS</t>
+          <t>Bem-Estar e Serviços - Qualidade do bairro, serviços, segurança, lazer</t>
         </is>
       </c>
       <c r="G28" t="n">
         <v>3</v>
       </c>
       <c r="H28" t="n">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="I28" t="n">
-        <v>469</v>
+        <v>7176</v>
       </c>
       <c r="J28" t="n">
-        <v>10700</v>
+        <v>29244</v>
       </c>
       <c r="K28" t="n">
-        <v>43.83177570093458</v>
+        <v>245.3836684448092</v>
       </c>
       <c r="L28" t="n">
-        <v>9.932232105040237</v>
+        <v>40.77967835426493</v>
       </c>
       <c r="M28" t="inlineStr">
         <is>
@@ -3648,7 +3216,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>itu</t>
+          <t>salto</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -3668,26 +3236,26 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Saúde - UBS, consultas, exames básicos, acesso SUS</t>
+          <t>Bem-Estar e Serviços - Qualidade do bairro, serviços, segurança, lazer</t>
         </is>
       </c>
       <c r="G29" t="n">
         <v>4</v>
       </c>
       <c r="H29" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="I29" t="n">
-        <v>842</v>
+        <v>3706</v>
       </c>
       <c r="J29" t="n">
-        <v>21456</v>
+        <v>15620</v>
       </c>
       <c r="K29" t="n">
-        <v>39.24310216256525</v>
+        <v>237.2599231754161</v>
       </c>
       <c r="L29" t="n">
-        <v>17.83142736128759</v>
+        <v>21.06040802409502</v>
       </c>
       <c r="M29" t="inlineStr">
         <is>
@@ -3723,26 +3291,26 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Assistência Social - Proteção social, seguridade, assistência, rede pública</t>
+          <t>Mobilidade e Acessibilidade - Transporte, calçadas, acesso a serviços, mobilidade</t>
         </is>
       </c>
       <c r="G30" t="n">
         <v>1</v>
       </c>
       <c r="H30" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="I30" t="n">
-        <v>5411</v>
+        <v>4983</v>
       </c>
       <c r="J30" t="n">
-        <v>24471</v>
+        <v>22743</v>
       </c>
       <c r="K30" t="n">
-        <v>221.1188754035389</v>
+        <v>219.1003825352856</v>
       </c>
       <c r="L30" t="n">
-        <v>30.74955958402</v>
+        <v>28.31732681707109</v>
       </c>
       <c r="M30" t="inlineStr">
         <is>
@@ -3778,26 +3346,26 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Assistência Social - Proteção social, seguridade, assistência, rede pública</t>
+          <t>Mobilidade e Acessibilidade - Transporte, calçadas, acesso a serviços, mobilidade</t>
         </is>
       </c>
       <c r="G31" t="n">
         <v>2</v>
       </c>
       <c r="H31" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="I31" t="n">
-        <v>4640</v>
+        <v>4834</v>
       </c>
       <c r="J31" t="n">
-        <v>17952</v>
+        <v>19745</v>
       </c>
       <c r="K31" t="n">
-        <v>258.4670231729056</v>
+        <v>244.8214737908331</v>
       </c>
       <c r="L31" t="n">
-        <v>26.36813093140876</v>
+        <v>27.4705915781099</v>
       </c>
       <c r="M31" t="inlineStr">
         <is>
@@ -3833,26 +3401,26 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Assistência Social - Proteção social, seguridade, assistência, rede pública</t>
+          <t>Mobilidade e Acessibilidade - Transporte, calçadas, acesso a serviços, mobilidade</t>
         </is>
       </c>
       <c r="G32" t="n">
         <v>3</v>
       </c>
       <c r="H32" t="n">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="I32" t="n">
-        <v>3492</v>
+        <v>6623</v>
       </c>
       <c r="J32" t="n">
-        <v>13858</v>
+        <v>25785</v>
       </c>
       <c r="K32" t="n">
-        <v>251.9844133352576</v>
+        <v>256.854760519682</v>
       </c>
       <c r="L32" t="n">
-        <v>19.84429164062056</v>
+        <v>37.63709723248281</v>
       </c>
       <c r="M32" t="inlineStr">
         <is>
@@ -3888,26 +3456,26 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Assistência Social - Proteção social, seguridade, assistência, rede pública</t>
+          <t>Mobilidade e Acessibilidade - Transporte, calçadas, acesso a serviços, mobilidade</t>
         </is>
       </c>
       <c r="G33" t="n">
         <v>4</v>
       </c>
       <c r="H33" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="I33" t="n">
-        <v>4054</v>
+        <v>1157</v>
       </c>
       <c r="J33" t="n">
-        <v>16894</v>
+        <v>4902</v>
       </c>
       <c r="K33" t="n">
-        <v>239.9668521368533</v>
+        <v>236.0261117911057</v>
       </c>
       <c r="L33" t="n">
-        <v>23.03801784395067</v>
+        <v>6.574984372336194</v>
       </c>
       <c r="M33" t="inlineStr">
         <is>
@@ -3943,7 +3511,7 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Bem-Estar e Serviços - Busca por qualidade de vida, serviços, lazer</t>
+          <t>Proteção Animal - Proteção animal, bem-estar, resgate, políticas pets</t>
         </is>
       </c>
       <c r="G34" t="n">
@@ -3953,16 +3521,16 @@
         <v>8</v>
       </c>
       <c r="I34" t="n">
-        <v>4075</v>
+        <v>5330</v>
       </c>
       <c r="J34" t="n">
-        <v>18517</v>
+        <v>21963</v>
       </c>
       <c r="K34" t="n">
-        <v>220.0680455797375</v>
+        <v>242.6808723762692</v>
       </c>
       <c r="L34" t="n">
-        <v>23.15735636756265</v>
+        <v>30.28925385008808</v>
       </c>
       <c r="M34" t="inlineStr">
         <is>
@@ -3998,26 +3566,26 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Bem-Estar e Serviços - Busca por qualidade de vida, serviços, lazer</t>
+          <t>Proteção Animal - Proteção animal, bem-estar, resgate, políticas pets</t>
         </is>
       </c>
       <c r="G35" t="n">
         <v>2</v>
       </c>
       <c r="H35" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="I35" t="n">
-        <v>4938</v>
+        <v>5165</v>
       </c>
       <c r="J35" t="n">
-        <v>20661</v>
+        <v>22551</v>
       </c>
       <c r="K35" t="n">
-        <v>239.0010164077247</v>
+        <v>229.0364063677886</v>
       </c>
       <c r="L35" t="n">
-        <v>28.06160140933114</v>
+        <v>29.35159402170824</v>
       </c>
       <c r="M35" t="inlineStr">
         <is>
@@ -4053,26 +3621,26 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Bem-Estar e Serviços - Busca por qualidade de vida, serviços, lazer</t>
+          <t>Proteção Animal - Proteção animal, bem-estar, resgate, políticas pets</t>
         </is>
       </c>
       <c r="G36" t="n">
         <v>3</v>
       </c>
       <c r="H36" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="I36" t="n">
-        <v>5361</v>
+        <v>3371</v>
       </c>
       <c r="J36" t="n">
-        <v>21130</v>
+        <v>13580</v>
       </c>
       <c r="K36" t="n">
-        <v>253.7150970184572</v>
+        <v>248.2326951399116</v>
       </c>
       <c r="L36" t="n">
-        <v>30.46542024208672</v>
+        <v>19.15667443314201</v>
       </c>
       <c r="M36" t="inlineStr">
         <is>
@@ -4108,26 +3676,26 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Bem-Estar e Serviços - Busca por qualidade de vida, serviços, lazer</t>
+          <t>Proteção Animal - Proteção animal, bem-estar, resgate, políticas pets</t>
         </is>
       </c>
       <c r="G37" t="n">
         <v>4</v>
       </c>
       <c r="H37" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="I37" t="n">
-        <v>3223</v>
+        <v>3731</v>
       </c>
       <c r="J37" t="n">
-        <v>12867</v>
+        <v>15081</v>
       </c>
       <c r="K37" t="n">
-        <v>250.4857387114324</v>
+        <v>247.3973874411511</v>
       </c>
       <c r="L37" t="n">
-        <v>18.31562198101949</v>
+        <v>21.20247769506166</v>
       </c>
       <c r="M37" t="inlineStr">
         <is>
@@ -4163,26 +3731,26 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Bem-Estar e Serviços - Qualidade do bairro, serviços, segurança, lazer</t>
+          <t>Saúde - UBS, consultas, exames básicos, acesso SUS</t>
         </is>
       </c>
       <c r="G38" t="n">
         <v>1</v>
       </c>
       <c r="H38" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="I38" t="n">
-        <v>4213</v>
+        <v>5411</v>
       </c>
       <c r="J38" t="n">
-        <v>17547</v>
+        <v>24471</v>
       </c>
       <c r="K38" t="n">
-        <v>240.0980224539807</v>
+        <v>221.1188754035389</v>
       </c>
       <c r="L38" t="n">
-        <v>23.94158095129852</v>
+        <v>30.74955958402</v>
       </c>
       <c r="M38" t="inlineStr">
         <is>
@@ -4218,26 +3786,26 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Bem-Estar e Serviços - Qualidade do bairro, serviços, segurança, lazer</t>
+          <t>Saúde - UBS, consultas, exames básicos, acesso SUS</t>
         </is>
       </c>
       <c r="G39" t="n">
         <v>2</v>
       </c>
       <c r="H39" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="I39" t="n">
-        <v>2502</v>
+        <v>4640</v>
       </c>
       <c r="J39" t="n">
-        <v>10764</v>
+        <v>17952</v>
       </c>
       <c r="K39" t="n">
-        <v>232.4414715719064</v>
+        <v>258.4670231729056</v>
       </c>
       <c r="L39" t="n">
-        <v>14.21833267034154</v>
+        <v>26.36813093140876</v>
       </c>
       <c r="M39" t="inlineStr">
         <is>
@@ -4273,26 +3841,26 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Bem-Estar e Serviços - Qualidade do bairro, serviços, segurança, lazer</t>
+          <t>Saúde - UBS, consultas, exames básicos, acesso SUS</t>
         </is>
       </c>
       <c r="G40" t="n">
         <v>3</v>
       </c>
       <c r="H40" t="n">
-        <v>14</v>
+        <v>5</v>
       </c>
       <c r="I40" t="n">
-        <v>7176</v>
+        <v>3492</v>
       </c>
       <c r="J40" t="n">
-        <v>29244</v>
+        <v>13858</v>
       </c>
       <c r="K40" t="n">
-        <v>245.3836684448092</v>
+        <v>251.9844133352576</v>
       </c>
       <c r="L40" t="n">
-        <v>40.77967835426493</v>
+        <v>19.84429164062056</v>
       </c>
       <c r="M40" t="inlineStr">
         <is>
@@ -4328,908 +3896,28 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Bem-Estar e Serviços - Qualidade do bairro, serviços, segurança, lazer</t>
+          <t>Saúde - UBS, consultas, exames básicos, acesso SUS</t>
         </is>
       </c>
       <c r="G41" t="n">
         <v>4</v>
       </c>
       <c r="H41" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="I41" t="n">
-        <v>3706</v>
+        <v>4054</v>
       </c>
       <c r="J41" t="n">
-        <v>15620</v>
+        <v>16894</v>
       </c>
       <c r="K41" t="n">
-        <v>237.2599231754161</v>
+        <v>239.9668521368533</v>
       </c>
       <c r="L41" t="n">
-        <v>21.06040802409502</v>
+        <v>23.03801784395067</v>
       </c>
       <c r="M41" t="inlineStr">
-        <is>
-          <t>votos por mil</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>SP</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>salto</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>2022</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>ROGERIO NOGUEIRA LOPES CRUZ</t>
-        </is>
-      </c>
-      <c r="E42" t="inlineStr">
-        <is>
-          <t>cidade_inteira</t>
-        </is>
-      </c>
-      <c r="F42" t="inlineStr">
-        <is>
-          <t>Comportamento Político - Qualidade de gestão, eficiência, entrega de serviços</t>
-        </is>
-      </c>
-      <c r="G42" t="n">
-        <v>1</v>
-      </c>
-      <c r="H42" t="n">
-        <v>5</v>
-      </c>
-      <c r="I42" t="n">
-        <v>3212</v>
-      </c>
-      <c r="J42" t="n">
-        <v>14760</v>
-      </c>
-      <c r="K42" t="n">
-        <v>217.6151761517615</v>
-      </c>
-      <c r="L42" t="n">
-        <v>18.25311132579417</v>
-      </c>
-      <c r="M42" t="inlineStr">
-        <is>
-          <t>votos por mil</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>SP</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>salto</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>2022</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>ROGERIO NOGUEIRA LOPES CRUZ</t>
-        </is>
-      </c>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>cidade_inteira</t>
-        </is>
-      </c>
-      <c r="F43" t="inlineStr">
-        <is>
-          <t>Comportamento Político - Qualidade de gestão, eficiência, entrega de serviços</t>
-        </is>
-      </c>
-      <c r="G43" t="n">
-        <v>2</v>
-      </c>
-      <c r="H43" t="n">
-        <v>12</v>
-      </c>
-      <c r="I43" t="n">
-        <v>7153</v>
-      </c>
-      <c r="J43" t="n">
-        <v>29390</v>
-      </c>
-      <c r="K43" t="n">
-        <v>243.3821027560395</v>
-      </c>
-      <c r="L43" t="n">
-        <v>40.64897425697562</v>
-      </c>
-      <c r="M43" t="inlineStr">
-        <is>
-          <t>votos por mil</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>SP</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>salto</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>2022</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>ROGERIO NOGUEIRA LOPES CRUZ</t>
-        </is>
-      </c>
-      <c r="E44" t="inlineStr">
-        <is>
-          <t>cidade_inteira</t>
-        </is>
-      </c>
-      <c r="F44" t="inlineStr">
-        <is>
-          <t>Comportamento Político - Qualidade de gestão, eficiência, entrega de serviços</t>
-        </is>
-      </c>
-      <c r="G44" t="n">
-        <v>3</v>
-      </c>
-      <c r="H44" t="n">
-        <v>10</v>
-      </c>
-      <c r="I44" t="n">
-        <v>5536</v>
-      </c>
-      <c r="J44" t="n">
-        <v>21946</v>
-      </c>
-      <c r="K44" t="n">
-        <v>252.255536316413</v>
-      </c>
-      <c r="L44" t="n">
-        <v>31.45990793885322</v>
-      </c>
-      <c r="M44" t="inlineStr">
-        <is>
-          <t>votos por mil</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>SP</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>salto</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>2022</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>ROGERIO NOGUEIRA LOPES CRUZ</t>
-        </is>
-      </c>
-      <c r="E45" t="inlineStr">
-        <is>
-          <t>cidade_inteira</t>
-        </is>
-      </c>
-      <c r="F45" t="inlineStr">
-        <is>
-          <t>Comportamento Político - Qualidade de gestão, eficiência, entrega de serviços</t>
-        </is>
-      </c>
-      <c r="G45" t="n">
-        <v>4</v>
-      </c>
-      <c r="H45" t="n">
-        <v>5</v>
-      </c>
-      <c r="I45" t="n">
-        <v>1696</v>
-      </c>
-      <c r="J45" t="n">
-        <v>7079</v>
-      </c>
-      <c r="K45" t="n">
-        <v>239.5818618448934</v>
-      </c>
-      <c r="L45" t="n">
-        <v>9.638006478376997</v>
-      </c>
-      <c r="M45" t="inlineStr">
-        <is>
-          <t>votos por mil</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>SP</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>salto</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>2022</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>ROGERIO NOGUEIRA LOPES CRUZ</t>
-        </is>
-      </c>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>cidade_inteira</t>
-        </is>
-      </c>
-      <c r="F46" t="inlineStr">
-        <is>
-          <t>Mobilidade e Acessibilidade - Transporte, calçadas, acesso a serviços, mobilidade</t>
-        </is>
-      </c>
-      <c r="G46" t="n">
-        <v>1</v>
-      </c>
-      <c r="H46" t="n">
-        <v>11</v>
-      </c>
-      <c r="I46" t="n">
-        <v>4983</v>
-      </c>
-      <c r="J46" t="n">
-        <v>22743</v>
-      </c>
-      <c r="K46" t="n">
-        <v>219.1003825352856</v>
-      </c>
-      <c r="L46" t="n">
-        <v>28.31732681707109</v>
-      </c>
-      <c r="M46" t="inlineStr">
-        <is>
-          <t>votos por mil</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>SP</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>salto</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>2022</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>ROGERIO NOGUEIRA LOPES CRUZ</t>
-        </is>
-      </c>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>cidade_inteira</t>
-        </is>
-      </c>
-      <c r="F47" t="inlineStr">
-        <is>
-          <t>Mobilidade e Acessibilidade - Transporte, calçadas, acesso a serviços, mobilidade</t>
-        </is>
-      </c>
-      <c r="G47" t="n">
-        <v>2</v>
-      </c>
-      <c r="H47" t="n">
-        <v>7</v>
-      </c>
-      <c r="I47" t="n">
-        <v>4834</v>
-      </c>
-      <c r="J47" t="n">
-        <v>19745</v>
-      </c>
-      <c r="K47" t="n">
-        <v>244.8214737908331</v>
-      </c>
-      <c r="L47" t="n">
-        <v>27.4705915781099</v>
-      </c>
-      <c r="M47" t="inlineStr">
-        <is>
-          <t>votos por mil</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>SP</t>
-        </is>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>salto</t>
-        </is>
-      </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>2022</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>ROGERIO NOGUEIRA LOPES CRUZ</t>
-        </is>
-      </c>
-      <c r="E48" t="inlineStr">
-        <is>
-          <t>cidade_inteira</t>
-        </is>
-      </c>
-      <c r="F48" t="inlineStr">
-        <is>
-          <t>Mobilidade e Acessibilidade - Transporte, calçadas, acesso a serviços, mobilidade</t>
-        </is>
-      </c>
-      <c r="G48" t="n">
-        <v>3</v>
-      </c>
-      <c r="H48" t="n">
-        <v>11</v>
-      </c>
-      <c r="I48" t="n">
-        <v>6623</v>
-      </c>
-      <c r="J48" t="n">
-        <v>25785</v>
-      </c>
-      <c r="K48" t="n">
-        <v>256.854760519682</v>
-      </c>
-      <c r="L48" t="n">
-        <v>37.63709723248281</v>
-      </c>
-      <c r="M48" t="inlineStr">
-        <is>
-          <t>votos por mil</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>SP</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>salto</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>2022</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>ROGERIO NOGUEIRA LOPES CRUZ</t>
-        </is>
-      </c>
-      <c r="E49" t="inlineStr">
-        <is>
-          <t>cidade_inteira</t>
-        </is>
-      </c>
-      <c r="F49" t="inlineStr">
-        <is>
-          <t>Mobilidade e Acessibilidade - Transporte, calçadas, acesso a serviços, mobilidade</t>
-        </is>
-      </c>
-      <c r="G49" t="n">
-        <v>4</v>
-      </c>
-      <c r="H49" t="n">
-        <v>3</v>
-      </c>
-      <c r="I49" t="n">
-        <v>1157</v>
-      </c>
-      <c r="J49" t="n">
-        <v>4902</v>
-      </c>
-      <c r="K49" t="n">
-        <v>236.0261117911057</v>
-      </c>
-      <c r="L49" t="n">
-        <v>6.574984372336194</v>
-      </c>
-      <c r="M49" t="inlineStr">
-        <is>
-          <t>votos por mil</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>SP</t>
-        </is>
-      </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>salto</t>
-        </is>
-      </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>2022</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>ROGERIO NOGUEIRA LOPES CRUZ</t>
-        </is>
-      </c>
-      <c r="E50" t="inlineStr">
-        <is>
-          <t>cidade_inteira</t>
-        </is>
-      </c>
-      <c r="F50" t="inlineStr">
-        <is>
-          <t>Proteção Animal - Proteção animal, bem-estar, resgate, políticas pets</t>
-        </is>
-      </c>
-      <c r="G50" t="n">
-        <v>1</v>
-      </c>
-      <c r="H50" t="n">
-        <v>8</v>
-      </c>
-      <c r="I50" t="n">
-        <v>5330</v>
-      </c>
-      <c r="J50" t="n">
-        <v>21963</v>
-      </c>
-      <c r="K50" t="n">
-        <v>242.6808723762692</v>
-      </c>
-      <c r="L50" t="n">
-        <v>30.28925385008808</v>
-      </c>
-      <c r="M50" t="inlineStr">
-        <is>
-          <t>votos por mil</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>SP</t>
-        </is>
-      </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>salto</t>
-        </is>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>2022</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>ROGERIO NOGUEIRA LOPES CRUZ</t>
-        </is>
-      </c>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t>cidade_inteira</t>
-        </is>
-      </c>
-      <c r="F51" t="inlineStr">
-        <is>
-          <t>Proteção Animal - Proteção animal, bem-estar, resgate, políticas pets</t>
-        </is>
-      </c>
-      <c r="G51" t="n">
-        <v>2</v>
-      </c>
-      <c r="H51" t="n">
-        <v>10</v>
-      </c>
-      <c r="I51" t="n">
-        <v>5165</v>
-      </c>
-      <c r="J51" t="n">
-        <v>22551</v>
-      </c>
-      <c r="K51" t="n">
-        <v>229.0364063677886</v>
-      </c>
-      <c r="L51" t="n">
-        <v>29.35159402170824</v>
-      </c>
-      <c r="M51" t="inlineStr">
-        <is>
-          <t>votos por mil</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>SP</t>
-        </is>
-      </c>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t>salto</t>
-        </is>
-      </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>2022</t>
-        </is>
-      </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t>ROGERIO NOGUEIRA LOPES CRUZ</t>
-        </is>
-      </c>
-      <c r="E52" t="inlineStr">
-        <is>
-          <t>cidade_inteira</t>
-        </is>
-      </c>
-      <c r="F52" t="inlineStr">
-        <is>
-          <t>Proteção Animal - Proteção animal, bem-estar, resgate, políticas pets</t>
-        </is>
-      </c>
-      <c r="G52" t="n">
-        <v>3</v>
-      </c>
-      <c r="H52" t="n">
-        <v>8</v>
-      </c>
-      <c r="I52" t="n">
-        <v>3371</v>
-      </c>
-      <c r="J52" t="n">
-        <v>13580</v>
-      </c>
-      <c r="K52" t="n">
-        <v>248.2326951399116</v>
-      </c>
-      <c r="L52" t="n">
-        <v>19.15667443314201</v>
-      </c>
-      <c r="M52" t="inlineStr">
-        <is>
-          <t>votos por mil</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>SP</t>
-        </is>
-      </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>salto</t>
-        </is>
-      </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>2022</t>
-        </is>
-      </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>ROGERIO NOGUEIRA LOPES CRUZ</t>
-        </is>
-      </c>
-      <c r="E53" t="inlineStr">
-        <is>
-          <t>cidade_inteira</t>
-        </is>
-      </c>
-      <c r="F53" t="inlineStr">
-        <is>
-          <t>Proteção Animal - Proteção animal, bem-estar, resgate, políticas pets</t>
-        </is>
-      </c>
-      <c r="G53" t="n">
-        <v>4</v>
-      </c>
-      <c r="H53" t="n">
-        <v>6</v>
-      </c>
-      <c r="I53" t="n">
-        <v>3731</v>
-      </c>
-      <c r="J53" t="n">
-        <v>15081</v>
-      </c>
-      <c r="K53" t="n">
-        <v>247.3973874411511</v>
-      </c>
-      <c r="L53" t="n">
-        <v>21.20247769506166</v>
-      </c>
-      <c r="M53" t="inlineStr">
-        <is>
-          <t>votos por mil</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t>SP</t>
-        </is>
-      </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>salto</t>
-        </is>
-      </c>
-      <c r="C54" t="inlineStr">
-        <is>
-          <t>2022</t>
-        </is>
-      </c>
-      <c r="D54" t="inlineStr">
-        <is>
-          <t>ROGERIO NOGUEIRA LOPES CRUZ</t>
-        </is>
-      </c>
-      <c r="E54" t="inlineStr">
-        <is>
-          <t>cidade_inteira</t>
-        </is>
-      </c>
-      <c r="F54" t="inlineStr">
-        <is>
-          <t>Saúde - UBS, consultas, exames básicos, acesso SUS</t>
-        </is>
-      </c>
-      <c r="G54" t="n">
-        <v>1</v>
-      </c>
-      <c r="H54" t="n">
-        <v>10</v>
-      </c>
-      <c r="I54" t="n">
-        <v>5411</v>
-      </c>
-      <c r="J54" t="n">
-        <v>24471</v>
-      </c>
-      <c r="K54" t="n">
-        <v>221.1188754035389</v>
-      </c>
-      <c r="L54" t="n">
-        <v>30.74955958402</v>
-      </c>
-      <c r="M54" t="inlineStr">
-        <is>
-          <t>votos por mil</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="inlineStr">
-        <is>
-          <t>SP</t>
-        </is>
-      </c>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t>salto</t>
-        </is>
-      </c>
-      <c r="C55" t="inlineStr">
-        <is>
-          <t>2022</t>
-        </is>
-      </c>
-      <c r="D55" t="inlineStr">
-        <is>
-          <t>ROGERIO NOGUEIRA LOPES CRUZ</t>
-        </is>
-      </c>
-      <c r="E55" t="inlineStr">
-        <is>
-          <t>cidade_inteira</t>
-        </is>
-      </c>
-      <c r="F55" t="inlineStr">
-        <is>
-          <t>Saúde - UBS, consultas, exames básicos, acesso SUS</t>
-        </is>
-      </c>
-      <c r="G55" t="n">
-        <v>2</v>
-      </c>
-      <c r="H55" t="n">
-        <v>8</v>
-      </c>
-      <c r="I55" t="n">
-        <v>4640</v>
-      </c>
-      <c r="J55" t="n">
-        <v>17952</v>
-      </c>
-      <c r="K55" t="n">
-        <v>258.4670231729056</v>
-      </c>
-      <c r="L55" t="n">
-        <v>26.36813093140876</v>
-      </c>
-      <c r="M55" t="inlineStr">
-        <is>
-          <t>votos por mil</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t>SP</t>
-        </is>
-      </c>
-      <c r="B56" t="inlineStr">
-        <is>
-          <t>salto</t>
-        </is>
-      </c>
-      <c r="C56" t="inlineStr">
-        <is>
-          <t>2022</t>
-        </is>
-      </c>
-      <c r="D56" t="inlineStr">
-        <is>
-          <t>ROGERIO NOGUEIRA LOPES CRUZ</t>
-        </is>
-      </c>
-      <c r="E56" t="inlineStr">
-        <is>
-          <t>cidade_inteira</t>
-        </is>
-      </c>
-      <c r="F56" t="inlineStr">
-        <is>
-          <t>Saúde - UBS, consultas, exames básicos, acesso SUS</t>
-        </is>
-      </c>
-      <c r="G56" t="n">
-        <v>3</v>
-      </c>
-      <c r="H56" t="n">
-        <v>5</v>
-      </c>
-      <c r="I56" t="n">
-        <v>3492</v>
-      </c>
-      <c r="J56" t="n">
-        <v>13858</v>
-      </c>
-      <c r="K56" t="n">
-        <v>251.9844133352576</v>
-      </c>
-      <c r="L56" t="n">
-        <v>19.84429164062056</v>
-      </c>
-      <c r="M56" t="inlineStr">
-        <is>
-          <t>votos por mil</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="inlineStr">
-        <is>
-          <t>SP</t>
-        </is>
-      </c>
-      <c r="B57" t="inlineStr">
-        <is>
-          <t>salto</t>
-        </is>
-      </c>
-      <c r="C57" t="inlineStr">
-        <is>
-          <t>2022</t>
-        </is>
-      </c>
-      <c r="D57" t="inlineStr">
-        <is>
-          <t>ROGERIO NOGUEIRA LOPES CRUZ</t>
-        </is>
-      </c>
-      <c r="E57" t="inlineStr">
-        <is>
-          <t>cidade_inteira</t>
-        </is>
-      </c>
-      <c r="F57" t="inlineStr">
-        <is>
-          <t>Saúde - UBS, consultas, exames básicos, acesso SUS</t>
-        </is>
-      </c>
-      <c r="G57" t="n">
-        <v>4</v>
-      </c>
-      <c r="H57" t="n">
-        <v>9</v>
-      </c>
-      <c r="I57" t="n">
-        <v>4054</v>
-      </c>
-      <c r="J57" t="n">
-        <v>16894</v>
-      </c>
-      <c r="K57" t="n">
-        <v>239.9668521368533</v>
-      </c>
-      <c r="L57" t="n">
-        <v>23.03801784395067</v>
-      </c>
-      <c r="M57" t="inlineStr">
         <is>
           <t>votos por mil</t>
         </is>

</xml_diff>